<commit_message>
Preserve PDF calculation tokens in water outputs
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_consolidada_v1.xlsx
+++ b/config/taxonomy_config_consolidada_v1.xlsx
@@ -3964,7 +3964,7 @@
     <col width="49" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="45" customWidth="1" min="11" max="11"/>
     <col width="65" customWidth="1" min="12" max="12"/>
@@ -6044,7 +6044,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -6059,7 +6059,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Variacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -6102,7 +6102,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -6117,7 +6117,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Quantidade adicionada gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Recuperacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -8290,7 +8290,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -8305,7 +8305,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>Variacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -8363,7 +8363,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Quantidade adicionada gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -8406,7 +8406,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -8421,7 +8421,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>Recuperacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -10536,7 +10536,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>Variacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
         </is>
       </c>
       <c r="M118" t="inlineStr">
@@ -10594,7 +10594,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -10609,7 +10609,7 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>Quantidade adicionada gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M119" t="inlineStr">
@@ -10652,7 +10652,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -10667,7 +10667,7 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>Recuperacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M120" t="inlineStr">
@@ -12782,7 +12782,7 @@
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
@@ -12797,7 +12797,7 @@
       </c>
       <c r="L159" t="inlineStr">
         <is>
-          <t>Variacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
         </is>
       </c>
       <c r="M159" t="inlineStr">
@@ -12840,7 +12840,7 @@
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
@@ -12855,7 +12855,7 @@
       </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t>Quantidade adicionada gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M160" t="inlineStr">
@@ -12898,7 +12898,7 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
@@ -12913,7 +12913,7 @@
       </c>
       <c r="L161" t="inlineStr">
         <is>
-          <t>Recuperacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M161" t="inlineStr">
@@ -15028,7 +15028,7 @@
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
@@ -15043,7 +15043,7 @@
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t>Variacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
         </is>
       </c>
       <c r="M200" t="inlineStr">
@@ -15086,7 +15086,7 @@
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
@@ -15101,7 +15101,7 @@
       </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t>Quantidade adicionada gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M201" t="inlineStr">
@@ -15144,7 +15144,7 @@
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
@@ -15159,7 +15159,7 @@
       </c>
       <c r="L202" t="inlineStr">
         <is>
-          <t>Recuperacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M202" t="inlineStr">
@@ -17274,7 +17274,7 @@
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
@@ -17289,7 +17289,7 @@
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t>Variacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
         </is>
       </c>
       <c r="M241" t="inlineStr">
@@ -17332,7 +17332,7 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
@@ -17347,7 +17347,7 @@
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>Quantidade adicionada gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M242" t="inlineStr">
@@ -17390,7 +17390,7 @@
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
@@ -17405,7 +17405,7 @@
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t>Recuperacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M243" t="inlineStr">
@@ -19520,7 +19520,7 @@
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J282" t="inlineStr">
@@ -19535,7 +19535,7 @@
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>Variacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
         </is>
       </c>
       <c r="M282" t="inlineStr">
@@ -19578,7 +19578,7 @@
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J283" t="inlineStr">
@@ -19593,7 +19593,7 @@
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>Quantidade adicionada gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
@@ -19636,7 +19636,7 @@
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J284" t="inlineStr">
@@ -19651,7 +19651,7 @@
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t>Recuperacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M284" t="inlineStr">
@@ -21766,7 +21766,7 @@
       </c>
       <c r="I323" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J323" t="inlineStr">
@@ -21781,7 +21781,7 @@
       </c>
       <c r="L323" t="inlineStr">
         <is>
-          <t>Variacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
         </is>
       </c>
       <c r="M323" t="inlineStr">
@@ -21824,7 +21824,7 @@
       </c>
       <c r="I324" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J324" t="inlineStr">
@@ -21839,7 +21839,7 @@
       </c>
       <c r="L324" t="inlineStr">
         <is>
-          <t>Quantidade adicionada gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M324" t="inlineStr">
@@ -21882,7 +21882,7 @@
       </c>
       <c r="I325" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J325" t="inlineStr">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="L325" t="inlineStr">
         <is>
-          <t>Recuperacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M325" t="inlineStr">
@@ -24012,7 +24012,7 @@
       </c>
       <c r="I364" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J364" t="inlineStr">
@@ -24027,7 +24027,7 @@
       </c>
       <c r="L364" t="inlineStr">
         <is>
-          <t>Variacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
         </is>
       </c>
       <c r="M364" t="inlineStr">
@@ -24070,7 +24070,7 @@
       </c>
       <c r="I365" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J365" t="inlineStr">
@@ -24085,7 +24085,7 @@
       </c>
       <c r="L365" t="inlineStr">
         <is>
-          <t>Quantidade adicionada gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M365" t="inlineStr">
@@ -24128,7 +24128,7 @@
       </c>
       <c r="I366" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J366" t="inlineStr">
@@ -24143,7 +24143,7 @@
       </c>
       <c r="L366" t="inlineStr">
         <is>
-          <t>Recuperacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M366" t="inlineStr">
@@ -26258,7 +26258,7 @@
       </c>
       <c r="I405" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J405" t="inlineStr">
@@ -26273,7 +26273,7 @@
       </c>
       <c r="L405" t="inlineStr">
         <is>
-          <t>Variacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
         </is>
       </c>
       <c r="M405" t="inlineStr">
@@ -26316,7 +26316,7 @@
       </c>
       <c r="I406" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J406" t="inlineStr">
@@ -26331,7 +26331,7 @@
       </c>
       <c r="L406" t="inlineStr">
         <is>
-          <t>Quantidade adicionada gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M406" t="inlineStr">
@@ -26374,7 +26374,7 @@
       </c>
       <c r="I407" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J407" t="inlineStr">
@@ -26389,7 +26389,7 @@
       </c>
       <c r="L407" t="inlineStr">
         <is>
-          <t>Recuperacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M407" t="inlineStr">
@@ -28504,7 +28504,7 @@
       </c>
       <c r="I446" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J446" t="inlineStr">
@@ -28519,7 +28519,7 @@
       </c>
       <c r="L446" t="inlineStr">
         <is>
-          <t>Variacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
         </is>
       </c>
       <c r="M446" t="inlineStr">
@@ -28562,7 +28562,7 @@
       </c>
       <c r="I447" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J447" t="inlineStr">
@@ -28577,7 +28577,7 @@
       </c>
       <c r="L447" t="inlineStr">
         <is>
-          <t>Quantidade adicionada gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M447" t="inlineStr">
@@ -28620,7 +28620,7 @@
       </c>
       <c r="I448" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J448" t="inlineStr">
@@ -28635,7 +28635,7 @@
       </c>
       <c r="L448" t="inlineStr">
         <is>
-          <t>Recuperacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M448" t="inlineStr">
@@ -30750,7 +30750,7 @@
       </c>
       <c r="I487" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J487" t="inlineStr">
@@ -30765,7 +30765,7 @@
       </c>
       <c r="L487" t="inlineStr">
         <is>
-          <t>Variacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
         </is>
       </c>
       <c r="M487" t="inlineStr">
@@ -30808,7 +30808,7 @@
       </c>
       <c r="I488" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J488" t="inlineStr">
@@ -30823,7 +30823,7 @@
       </c>
       <c r="L488" t="inlineStr">
         <is>
-          <t>Quantidade adicionada gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M488" t="inlineStr">
@@ -30866,7 +30866,7 @@
       </c>
       <c r="I489" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J489" t="inlineStr">
@@ -30881,7 +30881,7 @@
       </c>
       <c r="L489" t="inlineStr">
         <is>
-          <t>Recuperacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M489" t="inlineStr">
@@ -32996,7 +32996,7 @@
       </c>
       <c r="I528" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J528" t="inlineStr">
@@ -33011,7 +33011,7 @@
       </c>
       <c r="L528" t="inlineStr">
         <is>
-          <t>Variacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
         </is>
       </c>
       <c r="M528" t="inlineStr">
@@ -33054,7 +33054,7 @@
       </c>
       <c r="I529" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J529" t="inlineStr">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="L529" t="inlineStr">
         <is>
-          <t>Quantidade adicionada gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M529" t="inlineStr">
@@ -33112,7 +33112,7 @@
       </c>
       <c r="I530" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J530" t="inlineStr">
@@ -33127,7 +33127,7 @@
       </c>
       <c r="L530" t="inlineStr">
         <is>
-          <t>Recuperacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M530" t="inlineStr">
@@ -35242,7 +35242,7 @@
       </c>
       <c r="I569" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J569" t="inlineStr">
@@ -35257,7 +35257,7 @@
       </c>
       <c r="L569" t="inlineStr">
         <is>
-          <t>Variacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
         </is>
       </c>
       <c r="M569" t="inlineStr">
@@ -35300,7 +35300,7 @@
       </c>
       <c r="I570" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J570" t="inlineStr">
@@ -35315,7 +35315,7 @@
       </c>
       <c r="L570" t="inlineStr">
         <is>
-          <t>Quantidade adicionada gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M570" t="inlineStr">
@@ -35358,7 +35358,7 @@
       </c>
       <c r="I571" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>decimal_ou_texto_pdf</t>
         </is>
       </c>
       <c r="J571" t="inlineStr">
@@ -35373,7 +35373,7 @@
       </c>
       <c r="L571" t="inlineStr">
         <is>
-          <t>Recuperacao percentual gravada como numero no Excel, com casas decimais preservadas conforme o PDF.</t>
+          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
         </is>
       </c>
       <c r="M571" t="inlineStr">

</xml_diff>

<commit_message>
Validate PDF text in numeric output fields
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_consolidada_v1.xlsx
+++ b/config/taxonomy_config_consolidada_v1.xlsx
@@ -3964,7 +3964,7 @@
     <col width="49" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="26" customWidth="1" min="8" max="8"/>
-    <col width="22" customWidth="1" min="9" max="9"/>
+    <col width="18" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
     <col width="45" customWidth="1" min="11" max="11"/>
     <col width="65" customWidth="1" min="12" max="12"/>
@@ -6044,7 +6044,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J36" t="inlineStr">
@@ -6059,7 +6059,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M36" t="inlineStr">
@@ -6102,7 +6102,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J37" t="inlineStr">
@@ -6117,7 +6117,7 @@
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M37" t="inlineStr">
@@ -6160,7 +6160,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J38" t="inlineStr">
@@ -6175,7 +6175,7 @@
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M38" t="inlineStr">
@@ -8290,7 +8290,7 @@
       </c>
       <c r="I77" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J77" t="inlineStr">
@@ -8305,7 +8305,7 @@
       </c>
       <c r="L77" t="inlineStr">
         <is>
-          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M77" t="inlineStr">
@@ -8348,7 +8348,7 @@
       </c>
       <c r="I78" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J78" t="inlineStr">
@@ -8363,7 +8363,7 @@
       </c>
       <c r="L78" t="inlineStr">
         <is>
-          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M78" t="inlineStr">
@@ -8406,7 +8406,7 @@
       </c>
       <c r="I79" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J79" t="inlineStr">
@@ -8421,7 +8421,7 @@
       </c>
       <c r="L79" t="inlineStr">
         <is>
-          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M79" t="inlineStr">
@@ -10536,7 +10536,7 @@
       </c>
       <c r="I118" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J118" t="inlineStr">
@@ -10551,7 +10551,7 @@
       </c>
       <c r="L118" t="inlineStr">
         <is>
-          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M118" t="inlineStr">
@@ -10594,7 +10594,7 @@
       </c>
       <c r="I119" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J119" t="inlineStr">
@@ -10609,7 +10609,7 @@
       </c>
       <c r="L119" t="inlineStr">
         <is>
-          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M119" t="inlineStr">
@@ -10652,7 +10652,7 @@
       </c>
       <c r="I120" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J120" t="inlineStr">
@@ -10667,7 +10667,7 @@
       </c>
       <c r="L120" t="inlineStr">
         <is>
-          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M120" t="inlineStr">
@@ -12782,7 +12782,7 @@
       </c>
       <c r="I159" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J159" t="inlineStr">
@@ -12797,7 +12797,7 @@
       </c>
       <c r="L159" t="inlineStr">
         <is>
-          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M159" t="inlineStr">
@@ -12840,7 +12840,7 @@
       </c>
       <c r="I160" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J160" t="inlineStr">
@@ -12855,7 +12855,7 @@
       </c>
       <c r="L160" t="inlineStr">
         <is>
-          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M160" t="inlineStr">
@@ -12898,7 +12898,7 @@
       </c>
       <c r="I161" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J161" t="inlineStr">
@@ -12913,7 +12913,7 @@
       </c>
       <c r="L161" t="inlineStr">
         <is>
-          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M161" t="inlineStr">
@@ -15028,7 +15028,7 @@
       </c>
       <c r="I200" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J200" t="inlineStr">
@@ -15043,7 +15043,7 @@
       </c>
       <c r="L200" t="inlineStr">
         <is>
-          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M200" t="inlineStr">
@@ -15086,7 +15086,7 @@
       </c>
       <c r="I201" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J201" t="inlineStr">
@@ -15101,7 +15101,7 @@
       </c>
       <c r="L201" t="inlineStr">
         <is>
-          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M201" t="inlineStr">
@@ -15144,7 +15144,7 @@
       </c>
       <c r="I202" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J202" t="inlineStr">
@@ -15159,7 +15159,7 @@
       </c>
       <c r="L202" t="inlineStr">
         <is>
-          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M202" t="inlineStr">
@@ -17274,7 +17274,7 @@
       </c>
       <c r="I241" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J241" t="inlineStr">
@@ -17289,7 +17289,7 @@
       </c>
       <c r="L241" t="inlineStr">
         <is>
-          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M241" t="inlineStr">
@@ -17332,7 +17332,7 @@
       </c>
       <c r="I242" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J242" t="inlineStr">
@@ -17347,7 +17347,7 @@
       </c>
       <c r="L242" t="inlineStr">
         <is>
-          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M242" t="inlineStr">
@@ -17390,7 +17390,7 @@
       </c>
       <c r="I243" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J243" t="inlineStr">
@@ -17405,7 +17405,7 @@
       </c>
       <c r="L243" t="inlineStr">
         <is>
-          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M243" t="inlineStr">
@@ -19520,7 +19520,7 @@
       </c>
       <c r="I282" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J282" t="inlineStr">
@@ -19535,7 +19535,7 @@
       </c>
       <c r="L282" t="inlineStr">
         <is>
-          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M282" t="inlineStr">
@@ -19578,7 +19578,7 @@
       </c>
       <c r="I283" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J283" t="inlineStr">
@@ -19593,7 +19593,7 @@
       </c>
       <c r="L283" t="inlineStr">
         <is>
-          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M283" t="inlineStr">
@@ -19636,7 +19636,7 @@
       </c>
       <c r="I284" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J284" t="inlineStr">
@@ -19651,7 +19651,7 @@
       </c>
       <c r="L284" t="inlineStr">
         <is>
-          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M284" t="inlineStr">
@@ -21766,7 +21766,7 @@
       </c>
       <c r="I323" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J323" t="inlineStr">
@@ -21781,7 +21781,7 @@
       </c>
       <c r="L323" t="inlineStr">
         <is>
-          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M323" t="inlineStr">
@@ -21824,7 +21824,7 @@
       </c>
       <c r="I324" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J324" t="inlineStr">
@@ -21839,7 +21839,7 @@
       </c>
       <c r="L324" t="inlineStr">
         <is>
-          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M324" t="inlineStr">
@@ -21882,7 +21882,7 @@
       </c>
       <c r="I325" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J325" t="inlineStr">
@@ -21897,7 +21897,7 @@
       </c>
       <c r="L325" t="inlineStr">
         <is>
-          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M325" t="inlineStr">
@@ -24012,7 +24012,7 @@
       </c>
       <c r="I364" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J364" t="inlineStr">
@@ -24027,7 +24027,7 @@
       </c>
       <c r="L364" t="inlineStr">
         <is>
-          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M364" t="inlineStr">
@@ -24070,7 +24070,7 @@
       </c>
       <c r="I365" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J365" t="inlineStr">
@@ -24085,7 +24085,7 @@
       </c>
       <c r="L365" t="inlineStr">
         <is>
-          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M365" t="inlineStr">
@@ -24128,7 +24128,7 @@
       </c>
       <c r="I366" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J366" t="inlineStr">
@@ -24143,7 +24143,7 @@
       </c>
       <c r="L366" t="inlineStr">
         <is>
-          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M366" t="inlineStr">
@@ -26258,7 +26258,7 @@
       </c>
       <c r="I405" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J405" t="inlineStr">
@@ -26273,7 +26273,7 @@
       </c>
       <c r="L405" t="inlineStr">
         <is>
-          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M405" t="inlineStr">
@@ -26316,7 +26316,7 @@
       </c>
       <c r="I406" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J406" t="inlineStr">
@@ -26331,7 +26331,7 @@
       </c>
       <c r="L406" t="inlineStr">
         <is>
-          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M406" t="inlineStr">
@@ -26374,7 +26374,7 @@
       </c>
       <c r="I407" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J407" t="inlineStr">
@@ -26389,7 +26389,7 @@
       </c>
       <c r="L407" t="inlineStr">
         <is>
-          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M407" t="inlineStr">
@@ -28504,7 +28504,7 @@
       </c>
       <c r="I446" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J446" t="inlineStr">
@@ -28519,7 +28519,7 @@
       </c>
       <c r="L446" t="inlineStr">
         <is>
-          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M446" t="inlineStr">
@@ -28562,7 +28562,7 @@
       </c>
       <c r="I447" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J447" t="inlineStr">
@@ -28577,7 +28577,7 @@
       </c>
       <c r="L447" t="inlineStr">
         <is>
-          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M447" t="inlineStr">
@@ -28620,7 +28620,7 @@
       </c>
       <c r="I448" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J448" t="inlineStr">
@@ -28635,7 +28635,7 @@
       </c>
       <c r="L448" t="inlineStr">
         <is>
-          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M448" t="inlineStr">
@@ -30750,7 +30750,7 @@
       </c>
       <c r="I487" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J487" t="inlineStr">
@@ -30765,7 +30765,7 @@
       </c>
       <c r="L487" t="inlineStr">
         <is>
-          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M487" t="inlineStr">
@@ -30808,7 +30808,7 @@
       </c>
       <c r="I488" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J488" t="inlineStr">
@@ -30823,7 +30823,7 @@
       </c>
       <c r="L488" t="inlineStr">
         <is>
-          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M488" t="inlineStr">
@@ -30866,7 +30866,7 @@
       </c>
       <c r="I489" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J489" t="inlineStr">
@@ -30881,7 +30881,7 @@
       </c>
       <c r="L489" t="inlineStr">
         <is>
-          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M489" t="inlineStr">
@@ -32996,7 +32996,7 @@
       </c>
       <c r="I528" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J528" t="inlineStr">
@@ -33011,7 +33011,7 @@
       </c>
       <c r="L528" t="inlineStr">
         <is>
-          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M528" t="inlineStr">
@@ -33054,7 +33054,7 @@
       </c>
       <c r="I529" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J529" t="inlineStr">
@@ -33069,7 +33069,7 @@
       </c>
       <c r="L529" t="inlineStr">
         <is>
-          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M529" t="inlineStr">
@@ -33112,7 +33112,7 @@
       </c>
       <c r="I530" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J530" t="inlineStr">
@@ -33127,7 +33127,7 @@
       </c>
       <c r="L530" t="inlineStr">
         <is>
-          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M530" t="inlineStr">
@@ -35242,7 +35242,7 @@
       </c>
       <c r="I569" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J569" t="inlineStr">
@@ -35257,7 +35257,7 @@
       </c>
       <c r="L569" t="inlineStr">
         <is>
-          <t>Variacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador como Value ou Div0.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M569" t="inlineStr">
@@ -35300,7 +35300,7 @@
       </c>
       <c r="I570" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J570" t="inlineStr">
@@ -35315,7 +35315,7 @@
       </c>
       <c r="L570" t="inlineStr">
         <is>
-          <t>Quantidade adicionada preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M570" t="inlineStr">
@@ -35358,7 +35358,7 @@
       </c>
       <c r="I571" t="inlineStr">
         <is>
-          <t>decimal_ou_texto_pdf</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J571" t="inlineStr">
@@ -35373,7 +35373,7 @@
       </c>
       <c r="L571" t="inlineStr">
         <is>
-          <t>Recuperacao percentual preservada como aparece no PDF; numerica quando houver numero e textual quando o PDF trouxer marcador de calculo.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
       <c r="M571" t="inlineStr">

</xml_diff>

<commit_message>
Format consolidated taxonomy workbook
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_consolidada_v1.xlsx
+++ b/config/taxonomy_config_consolidada_v1.xlsx
@@ -16,7 +16,16 @@
     <sheet name="section_rules" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="continuation_rules" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
-  <definedNames/>
+  <definedNames>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README_FORMATO'!$A$1:$C$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'templates'!$A$1:$H$15</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'template_rules'!$A$1:$G$78</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'output_model'!$A$1:$L$1037</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'text_extraction_rules'!$A$1:$G$85</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'table_extraction_rules'!$A$1:$H$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'section_rules'!$A$1:$L$54</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'continuation_rules'!$A$1:$E$4</definedName>
+  </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
 </file>
@@ -24,7 +33,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -32,16 +41,25 @@
       <sz val="11"/>
       <scheme val="minor"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+    </font>
   </fonts>
-  <fills count="2">
+  <fills count="3">
     <fill>
       <patternFill/>
     </fill>
     <fill>
       <patternFill patternType="gray125"/>
     </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="001F4E78"/>
+      </patternFill>
+    </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -49,12 +67,29 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="009EADCC"/>
+      </left>
+      <right style="thin">
+        <color rgb="009EADCC"/>
+      </right>
+      <top style="thin">
+        <color rgb="009EADCC"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="009EADCC"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -422,19 +457,24 @@
   </sheetPr>
   <dimension ref="A1:C8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="12" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="55" customWidth="1" min="3" max="3"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ordem</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>aba</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -546,6 +586,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:C8"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -558,44 +599,54 @@
   </sheetPr>
   <dimension ref="A1:H15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="54" customWidth="1" min="3" max="3"/>
+    <col width="17" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>theme_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>nome</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>schema_ref</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>prioridade</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>score_minimo</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
@@ -1106,6 +1157,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H15"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -1118,39 +1170,48 @@
   </sheetPr>
   <dimension ref="A1:G78"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="12" customWidth="1" min="2" max="2"/>
+    <col width="12" customWidth="1" min="3" max="3"/>
+    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="55" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>tipo_regra</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>fonte</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>padrao_regex</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>peso</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -3698,6 +3759,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G78"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -3710,64 +3772,78 @@
   </sheetPr>
   <dimension ref="A1:L1037"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="39" customWidth="1" min="1" max="1"/>
+    <col width="27" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="13" customWidth="1" min="7" max="7"/>
+    <col width="28" customWidth="1" min="8" max="8"/>
+    <col width="19" customWidth="1" min="9" max="9"/>
+    <col width="13" customWidth="1" min="10" max="10"/>
+    <col width="55" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>theme_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>sheet_name</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ordem_aba</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>ativo_aba</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>descricao_aba</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ordem_campo</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>campo</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>tipo_dado</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>obrigatorio</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>origem</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>descricao_campo</t>
         </is>
@@ -7634,14 +7710,9 @@
           <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
-      <c r="G73" t="inlineStr"/>
-      <c r="H73" t="inlineStr"/>
-      <c r="I73" t="inlineStr"/>
       <c r="J73" t="b">
         <v>0</v>
       </c>
-      <c r="K73" t="inlineStr"/>
-      <c r="L73" t="inlineStr"/>
     </row>
     <row r="74">
       <c r="A74" t="inlineStr">
@@ -7670,14 +7741,9 @@
           <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
-      <c r="G74" t="inlineStr"/>
-      <c r="H74" t="inlineStr"/>
-      <c r="I74" t="inlineStr"/>
       <c r="J74" t="b">
         <v>0</v>
       </c>
-      <c r="K74" t="inlineStr"/>
-      <c r="L74" t="inlineStr"/>
     </row>
     <row r="75">
       <c r="A75" t="inlineStr">
@@ -7706,14 +7772,9 @@
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="G75" t="inlineStr"/>
-      <c r="H75" t="inlineStr"/>
-      <c r="I75" t="inlineStr"/>
       <c r="J75" t="b">
         <v>0</v>
       </c>
-      <c r="K75" t="inlineStr"/>
-      <c r="L75" t="inlineStr"/>
     </row>
     <row r="76">
       <c r="A76" t="inlineStr">
@@ -11576,14 +11637,9 @@
           <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
-      <c r="G147" t="inlineStr"/>
-      <c r="H147" t="inlineStr"/>
-      <c r="I147" t="inlineStr"/>
       <c r="J147" t="b">
         <v>0</v>
       </c>
-      <c r="K147" t="inlineStr"/>
-      <c r="L147" t="inlineStr"/>
     </row>
     <row r="148">
       <c r="A148" t="inlineStr">
@@ -11612,14 +11668,9 @@
           <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
-      <c r="G148" t="inlineStr"/>
-      <c r="H148" t="inlineStr"/>
-      <c r="I148" t="inlineStr"/>
       <c r="J148" t="b">
         <v>0</v>
       </c>
-      <c r="K148" t="inlineStr"/>
-      <c r="L148" t="inlineStr"/>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
@@ -11648,14 +11699,9 @@
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="G149" t="inlineStr"/>
-      <c r="H149" t="inlineStr"/>
-      <c r="I149" t="inlineStr"/>
       <c r="J149" t="b">
         <v>0</v>
       </c>
-      <c r="K149" t="inlineStr"/>
-      <c r="L149" t="inlineStr"/>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
@@ -15518,14 +15564,9 @@
           <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
-      <c r="G221" t="inlineStr"/>
-      <c r="H221" t="inlineStr"/>
-      <c r="I221" t="inlineStr"/>
       <c r="J221" t="b">
         <v>0</v>
       </c>
-      <c r="K221" t="inlineStr"/>
-      <c r="L221" t="inlineStr"/>
     </row>
     <row r="222">
       <c r="A222" t="inlineStr">
@@ -15554,14 +15595,9 @@
           <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
-      <c r="G222" t="inlineStr"/>
-      <c r="H222" t="inlineStr"/>
-      <c r="I222" t="inlineStr"/>
       <c r="J222" t="b">
         <v>0</v>
       </c>
-      <c r="K222" t="inlineStr"/>
-      <c r="L222" t="inlineStr"/>
     </row>
     <row r="223">
       <c r="A223" t="inlineStr">
@@ -15590,14 +15626,9 @@
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="G223" t="inlineStr"/>
-      <c r="H223" t="inlineStr"/>
-      <c r="I223" t="inlineStr"/>
       <c r="J223" t="b">
         <v>0</v>
       </c>
-      <c r="K223" t="inlineStr"/>
-      <c r="L223" t="inlineStr"/>
     </row>
     <row r="224">
       <c r="A224" t="inlineStr">
@@ -19460,14 +19491,9 @@
           <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
-      <c r="G295" t="inlineStr"/>
-      <c r="H295" t="inlineStr"/>
-      <c r="I295" t="inlineStr"/>
       <c r="J295" t="b">
         <v>0</v>
       </c>
-      <c r="K295" t="inlineStr"/>
-      <c r="L295" t="inlineStr"/>
     </row>
     <row r="296">
       <c r="A296" t="inlineStr">
@@ -19496,14 +19522,9 @@
           <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
-      <c r="G296" t="inlineStr"/>
-      <c r="H296" t="inlineStr"/>
-      <c r="I296" t="inlineStr"/>
       <c r="J296" t="b">
         <v>0</v>
       </c>
-      <c r="K296" t="inlineStr"/>
-      <c r="L296" t="inlineStr"/>
     </row>
     <row r="297">
       <c r="A297" t="inlineStr">
@@ -19532,14 +19553,9 @@
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="G297" t="inlineStr"/>
-      <c r="H297" t="inlineStr"/>
-      <c r="I297" t="inlineStr"/>
       <c r="J297" t="b">
         <v>0</v>
       </c>
-      <c r="K297" t="inlineStr"/>
-      <c r="L297" t="inlineStr"/>
     </row>
     <row r="298">
       <c r="A298" t="inlineStr">
@@ -23402,14 +23418,9 @@
           <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
-      <c r="G369" t="inlineStr"/>
-      <c r="H369" t="inlineStr"/>
-      <c r="I369" t="inlineStr"/>
       <c r="J369" t="b">
         <v>0</v>
       </c>
-      <c r="K369" t="inlineStr"/>
-      <c r="L369" t="inlineStr"/>
     </row>
     <row r="370">
       <c r="A370" t="inlineStr">
@@ -23438,14 +23449,9 @@
           <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
-      <c r="G370" t="inlineStr"/>
-      <c r="H370" t="inlineStr"/>
-      <c r="I370" t="inlineStr"/>
       <c r="J370" t="b">
         <v>0</v>
       </c>
-      <c r="K370" t="inlineStr"/>
-      <c r="L370" t="inlineStr"/>
     </row>
     <row r="371">
       <c r="A371" t="inlineStr">
@@ -23474,14 +23480,9 @@
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="G371" t="inlineStr"/>
-      <c r="H371" t="inlineStr"/>
-      <c r="I371" t="inlineStr"/>
       <c r="J371" t="b">
         <v>0</v>
       </c>
-      <c r="K371" t="inlineStr"/>
-      <c r="L371" t="inlineStr"/>
     </row>
     <row r="372">
       <c r="A372" t="inlineStr">
@@ -27344,14 +27345,9 @@
           <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
-      <c r="G443" t="inlineStr"/>
-      <c r="H443" t="inlineStr"/>
-      <c r="I443" t="inlineStr"/>
       <c r="J443" t="b">
         <v>0</v>
       </c>
-      <c r="K443" t="inlineStr"/>
-      <c r="L443" t="inlineStr"/>
     </row>
     <row r="444">
       <c r="A444" t="inlineStr">
@@ -27380,14 +27376,9 @@
           <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
-      <c r="G444" t="inlineStr"/>
-      <c r="H444" t="inlineStr"/>
-      <c r="I444" t="inlineStr"/>
       <c r="J444" t="b">
         <v>0</v>
       </c>
-      <c r="K444" t="inlineStr"/>
-      <c r="L444" t="inlineStr"/>
     </row>
     <row r="445">
       <c r="A445" t="inlineStr">
@@ -27416,14 +27407,9 @@
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="G445" t="inlineStr"/>
-      <c r="H445" t="inlineStr"/>
-      <c r="I445" t="inlineStr"/>
       <c r="J445" t="b">
         <v>0</v>
       </c>
-      <c r="K445" t="inlineStr"/>
-      <c r="L445" t="inlineStr"/>
     </row>
     <row r="446">
       <c r="A446" t="inlineStr">
@@ -31286,14 +31272,9 @@
           <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
-      <c r="G517" t="inlineStr"/>
-      <c r="H517" t="inlineStr"/>
-      <c r="I517" t="inlineStr"/>
       <c r="J517" t="b">
         <v>0</v>
       </c>
-      <c r="K517" t="inlineStr"/>
-      <c r="L517" t="inlineStr"/>
     </row>
     <row r="518">
       <c r="A518" t="inlineStr">
@@ -31322,14 +31303,9 @@
           <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
-      <c r="G518" t="inlineStr"/>
-      <c r="H518" t="inlineStr"/>
-      <c r="I518" t="inlineStr"/>
       <c r="J518" t="b">
         <v>0</v>
       </c>
-      <c r="K518" t="inlineStr"/>
-      <c r="L518" t="inlineStr"/>
     </row>
     <row r="519">
       <c r="A519" t="inlineStr">
@@ -31358,14 +31334,9 @@
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="G519" t="inlineStr"/>
-      <c r="H519" t="inlineStr"/>
-      <c r="I519" t="inlineStr"/>
       <c r="J519" t="b">
         <v>0</v>
       </c>
-      <c r="K519" t="inlineStr"/>
-      <c r="L519" t="inlineStr"/>
     </row>
     <row r="520">
       <c r="A520" t="inlineStr">
@@ -35228,14 +35199,9 @@
           <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
-      <c r="G591" t="inlineStr"/>
-      <c r="H591" t="inlineStr"/>
-      <c r="I591" t="inlineStr"/>
       <c r="J591" t="b">
         <v>0</v>
       </c>
-      <c r="K591" t="inlineStr"/>
-      <c r="L591" t="inlineStr"/>
     </row>
     <row r="592">
       <c r="A592" t="inlineStr">
@@ -35264,14 +35230,9 @@
           <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
-      <c r="G592" t="inlineStr"/>
-      <c r="H592" t="inlineStr"/>
-      <c r="I592" t="inlineStr"/>
       <c r="J592" t="b">
         <v>0</v>
       </c>
-      <c r="K592" t="inlineStr"/>
-      <c r="L592" t="inlineStr"/>
     </row>
     <row r="593">
       <c r="A593" t="inlineStr">
@@ -35300,14 +35261,9 @@
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="G593" t="inlineStr"/>
-      <c r="H593" t="inlineStr"/>
-      <c r="I593" t="inlineStr"/>
       <c r="J593" t="b">
         <v>0</v>
       </c>
-      <c r="K593" t="inlineStr"/>
-      <c r="L593" t="inlineStr"/>
     </row>
     <row r="594">
       <c r="A594" t="inlineStr">
@@ -39170,14 +39126,9 @@
           <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
-      <c r="G665" t="inlineStr"/>
-      <c r="H665" t="inlineStr"/>
-      <c r="I665" t="inlineStr"/>
       <c r="J665" t="b">
         <v>0</v>
       </c>
-      <c r="K665" t="inlineStr"/>
-      <c r="L665" t="inlineStr"/>
     </row>
     <row r="666">
       <c r="A666" t="inlineStr">
@@ -39206,14 +39157,9 @@
           <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
-      <c r="G666" t="inlineStr"/>
-      <c r="H666" t="inlineStr"/>
-      <c r="I666" t="inlineStr"/>
       <c r="J666" t="b">
         <v>0</v>
       </c>
-      <c r="K666" t="inlineStr"/>
-      <c r="L666" t="inlineStr"/>
     </row>
     <row r="667">
       <c r="A667" t="inlineStr">
@@ -39242,14 +39188,9 @@
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="G667" t="inlineStr"/>
-      <c r="H667" t="inlineStr"/>
-      <c r="I667" t="inlineStr"/>
       <c r="J667" t="b">
         <v>0</v>
       </c>
-      <c r="K667" t="inlineStr"/>
-      <c r="L667" t="inlineStr"/>
     </row>
     <row r="668">
       <c r="A668" t="inlineStr">
@@ -43112,14 +43053,9 @@
           <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
-      <c r="G739" t="inlineStr"/>
-      <c r="H739" t="inlineStr"/>
-      <c r="I739" t="inlineStr"/>
       <c r="J739" t="b">
         <v>0</v>
       </c>
-      <c r="K739" t="inlineStr"/>
-      <c r="L739" t="inlineStr"/>
     </row>
     <row r="740">
       <c r="A740" t="inlineStr">
@@ -43148,14 +43084,9 @@
           <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
-      <c r="G740" t="inlineStr"/>
-      <c r="H740" t="inlineStr"/>
-      <c r="I740" t="inlineStr"/>
       <c r="J740" t="b">
         <v>0</v>
       </c>
-      <c r="K740" t="inlineStr"/>
-      <c r="L740" t="inlineStr"/>
     </row>
     <row r="741">
       <c r="A741" t="inlineStr">
@@ -43184,14 +43115,9 @@
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="G741" t="inlineStr"/>
-      <c r="H741" t="inlineStr"/>
-      <c r="I741" t="inlineStr"/>
       <c r="J741" t="b">
         <v>0</v>
       </c>
-      <c r="K741" t="inlineStr"/>
-      <c r="L741" t="inlineStr"/>
     </row>
     <row r="742">
       <c r="A742" t="inlineStr">
@@ -47054,14 +46980,9 @@
           <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
-      <c r="G813" t="inlineStr"/>
-      <c r="H813" t="inlineStr"/>
-      <c r="I813" t="inlineStr"/>
       <c r="J813" t="b">
         <v>0</v>
       </c>
-      <c r="K813" t="inlineStr"/>
-      <c r="L813" t="inlineStr"/>
     </row>
     <row r="814">
       <c r="A814" t="inlineStr">
@@ -47090,14 +47011,9 @@
           <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
-      <c r="G814" t="inlineStr"/>
-      <c r="H814" t="inlineStr"/>
-      <c r="I814" t="inlineStr"/>
       <c r="J814" t="b">
         <v>0</v>
       </c>
-      <c r="K814" t="inlineStr"/>
-      <c r="L814" t="inlineStr"/>
     </row>
     <row r="815">
       <c r="A815" t="inlineStr">
@@ -47126,14 +47042,9 @@
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="G815" t="inlineStr"/>
-      <c r="H815" t="inlineStr"/>
-      <c r="I815" t="inlineStr"/>
       <c r="J815" t="b">
         <v>0</v>
       </c>
-      <c r="K815" t="inlineStr"/>
-      <c r="L815" t="inlineStr"/>
     </row>
     <row r="816">
       <c r="A816" t="inlineStr">
@@ -50996,14 +50907,9 @@
           <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
-      <c r="G887" t="inlineStr"/>
-      <c r="H887" t="inlineStr"/>
-      <c r="I887" t="inlineStr"/>
       <c r="J887" t="b">
         <v>0</v>
       </c>
-      <c r="K887" t="inlineStr"/>
-      <c r="L887" t="inlineStr"/>
     </row>
     <row r="888">
       <c r="A888" t="inlineStr">
@@ -51032,14 +50938,9 @@
           <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
-      <c r="G888" t="inlineStr"/>
-      <c r="H888" t="inlineStr"/>
-      <c r="I888" t="inlineStr"/>
       <c r="J888" t="b">
         <v>0</v>
       </c>
-      <c r="K888" t="inlineStr"/>
-      <c r="L888" t="inlineStr"/>
     </row>
     <row r="889">
       <c r="A889" t="inlineStr">
@@ -51068,14 +50969,9 @@
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="G889" t="inlineStr"/>
-      <c r="H889" t="inlineStr"/>
-      <c r="I889" t="inlineStr"/>
       <c r="J889" t="b">
         <v>0</v>
       </c>
-      <c r="K889" t="inlineStr"/>
-      <c r="L889" t="inlineStr"/>
     </row>
     <row r="890">
       <c r="A890" t="inlineStr">
@@ -54938,14 +54834,9 @@
           <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
-      <c r="G961" t="inlineStr"/>
-      <c r="H961" t="inlineStr"/>
-      <c r="I961" t="inlineStr"/>
       <c r="J961" t="b">
         <v>0</v>
       </c>
-      <c r="K961" t="inlineStr"/>
-      <c r="L961" t="inlineStr"/>
     </row>
     <row r="962">
       <c r="A962" t="inlineStr">
@@ -54974,14 +54865,9 @@
           <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
-      <c r="G962" t="inlineStr"/>
-      <c r="H962" t="inlineStr"/>
-      <c r="I962" t="inlineStr"/>
       <c r="J962" t="b">
         <v>0</v>
       </c>
-      <c r="K962" t="inlineStr"/>
-      <c r="L962" t="inlineStr"/>
     </row>
     <row r="963">
       <c r="A963" t="inlineStr">
@@ -55010,14 +54896,9 @@
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="G963" t="inlineStr"/>
-      <c r="H963" t="inlineStr"/>
-      <c r="I963" t="inlineStr"/>
       <c r="J963" t="b">
         <v>0</v>
       </c>
-      <c r="K963" t="inlineStr"/>
-      <c r="L963" t="inlineStr"/>
     </row>
     <row r="964">
       <c r="A964" t="inlineStr">
@@ -58880,14 +58761,9 @@
           <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
-      <c r="G1035" t="inlineStr"/>
-      <c r="H1035" t="inlineStr"/>
-      <c r="I1035" t="inlineStr"/>
       <c r="J1035" t="b">
         <v>0</v>
       </c>
-      <c r="K1035" t="inlineStr"/>
-      <c r="L1035" t="inlineStr"/>
     </row>
     <row r="1036">
       <c r="A1036" t="inlineStr">
@@ -58916,14 +58792,9 @@
           <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
-      <c r="G1036" t="inlineStr"/>
-      <c r="H1036" t="inlineStr"/>
-      <c r="I1036" t="inlineStr"/>
       <c r="J1036" t="b">
         <v>0</v>
       </c>
-      <c r="K1036" t="inlineStr"/>
-      <c r="L1036" t="inlineStr"/>
     </row>
     <row r="1037">
       <c r="A1037" t="inlineStr">
@@ -58952,16 +58823,12 @@
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="G1037" t="inlineStr"/>
-      <c r="H1037" t="inlineStr"/>
-      <c r="I1037" t="inlineStr"/>
       <c r="J1037" t="b">
         <v>0</v>
       </c>
-      <c r="K1037" t="inlineStr"/>
-      <c r="L1037" t="inlineStr"/>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L1037"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -58974,39 +58841,48 @@
   </sheetPr>
   <dimension ref="A1:G85"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="29" customWidth="1" min="2" max="2"/>
+    <col width="16" customWidth="1" min="3" max="3"/>
+    <col width="28" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="12" customWidth="1" min="6" max="6"/>
+    <col width="54" customWidth="1" min="7" max="7"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>regra_origem</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>tabela_destino</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>campo</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>padrao_regex</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -59041,7 +58917,6 @@
       <c r="F2" t="b">
         <v>1</v>
       </c>
-      <c r="G2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -59072,7 +58947,6 @@
       <c r="F3" t="b">
         <v>1</v>
       </c>
-      <c r="G3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -59103,7 +58977,6 @@
       <c r="F4" t="b">
         <v>1</v>
       </c>
-      <c r="G4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -59134,7 +59007,6 @@
       <c r="F5" t="b">
         <v>1</v>
       </c>
-      <c r="G5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -59165,7 +59037,6 @@
       <c r="F6" t="b">
         <v>1</v>
       </c>
-      <c r="G6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -59196,7 +59067,6 @@
       <c r="F7" t="b">
         <v>1</v>
       </c>
-      <c r="G7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -59227,7 +59097,6 @@
       <c r="F8" t="b">
         <v>1</v>
       </c>
-      <c r="G8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -59258,7 +59127,6 @@
       <c r="F9" t="b">
         <v>1</v>
       </c>
-      <c r="G9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -59289,7 +59157,6 @@
       <c r="F10" t="b">
         <v>1</v>
       </c>
-      <c r="G10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -59320,7 +59187,6 @@
       <c r="F11" t="b">
         <v>1</v>
       </c>
-      <c r="G11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -59351,7 +59217,6 @@
       <c r="F12" t="b">
         <v>1</v>
       </c>
-      <c r="G12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -59382,7 +59247,6 @@
       <c r="F13" t="b">
         <v>1</v>
       </c>
-      <c r="G13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -59413,7 +59277,6 @@
       <c r="F14" t="b">
         <v>1</v>
       </c>
-      <c r="G14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -59444,7 +59307,6 @@
       <c r="F15" t="b">
         <v>1</v>
       </c>
-      <c r="G15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -59475,7 +59337,6 @@
       <c r="F16" t="b">
         <v>1</v>
       </c>
-      <c r="G16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -59506,7 +59367,6 @@
       <c r="F17" t="b">
         <v>1</v>
       </c>
-      <c r="G17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -59537,7 +59397,6 @@
       <c r="F18" t="b">
         <v>1</v>
       </c>
-      <c r="G18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -59568,7 +59427,6 @@
       <c r="F19" t="b">
         <v>1</v>
       </c>
-      <c r="G19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -59599,7 +59457,6 @@
       <c r="F20" t="b">
         <v>1</v>
       </c>
-      <c r="G20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -59630,7 +59487,6 @@
       <c r="F21" t="b">
         <v>1</v>
       </c>
-      <c r="G21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -59661,7 +59517,6 @@
       <c r="F22" t="b">
         <v>1</v>
       </c>
-      <c r="G22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -59692,7 +59547,6 @@
       <c r="F23" t="b">
         <v>1</v>
       </c>
-      <c r="G23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -59723,7 +59577,6 @@
       <c r="F24" t="b">
         <v>1</v>
       </c>
-      <c r="G24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -59754,7 +59607,6 @@
       <c r="F25" t="b">
         <v>1</v>
       </c>
-      <c r="G25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -59785,7 +59637,6 @@
       <c r="F26" t="b">
         <v>1</v>
       </c>
-      <c r="G26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -59816,7 +59667,6 @@
       <c r="F27" t="b">
         <v>1</v>
       </c>
-      <c r="G27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -59847,7 +59697,6 @@
       <c r="F28" t="b">
         <v>1</v>
       </c>
-      <c r="G28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -59878,7 +59727,6 @@
       <c r="F29" t="b">
         <v>1</v>
       </c>
-      <c r="G29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -59909,7 +59757,6 @@
       <c r="F30" t="b">
         <v>1</v>
       </c>
-      <c r="G30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -59940,7 +59787,6 @@
       <c r="F31" t="b">
         <v>1</v>
       </c>
-      <c r="G31" t="inlineStr"/>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
@@ -59971,7 +59817,6 @@
       <c r="F32" t="b">
         <v>1</v>
       </c>
-      <c r="G32" t="inlineStr"/>
     </row>
     <row r="33">
       <c r="A33" t="inlineStr">
@@ -60002,7 +59847,6 @@
       <c r="F33" t="b">
         <v>1</v>
       </c>
-      <c r="G33" t="inlineStr"/>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
@@ -60033,7 +59877,6 @@
       <c r="F34" t="b">
         <v>1</v>
       </c>
-      <c r="G34" t="inlineStr"/>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
@@ -60064,7 +59907,6 @@
       <c r="F35" t="b">
         <v>1</v>
       </c>
-      <c r="G35" t="inlineStr"/>
     </row>
     <row r="36">
       <c r="A36" t="inlineStr">
@@ -60095,7 +59937,6 @@
       <c r="F36" t="b">
         <v>1</v>
       </c>
-      <c r="G36" t="inlineStr"/>
     </row>
     <row r="37">
       <c r="A37" t="inlineStr">
@@ -60126,7 +59967,6 @@
       <c r="F37" t="b">
         <v>1</v>
       </c>
-      <c r="G37" t="inlineStr"/>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
@@ -60157,7 +59997,6 @@
       <c r="F38" t="b">
         <v>1</v>
       </c>
-      <c r="G38" t="inlineStr"/>
     </row>
     <row r="39">
       <c r="A39" t="inlineStr">
@@ -60188,7 +60027,6 @@
       <c r="F39" t="b">
         <v>1</v>
       </c>
-      <c r="G39" t="inlineStr"/>
     </row>
     <row r="40">
       <c r="A40" t="inlineStr">
@@ -60219,7 +60057,6 @@
       <c r="F40" t="b">
         <v>1</v>
       </c>
-      <c r="G40" t="inlineStr"/>
     </row>
     <row r="41">
       <c r="A41" t="inlineStr">
@@ -60250,7 +60087,6 @@
       <c r="F41" t="b">
         <v>1</v>
       </c>
-      <c r="G41" t="inlineStr"/>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
@@ -60281,7 +60117,6 @@
       <c r="F42" t="b">
         <v>1</v>
       </c>
-      <c r="G42" t="inlineStr"/>
     </row>
     <row r="43">
       <c r="A43" t="inlineStr">
@@ -60312,7 +60147,6 @@
       <c r="F43" t="b">
         <v>1</v>
       </c>
-      <c r="G43" t="inlineStr"/>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
@@ -60343,7 +60177,6 @@
       <c r="F44" t="b">
         <v>1</v>
       </c>
-      <c r="G44" t="inlineStr"/>
     </row>
     <row r="45">
       <c r="A45" t="inlineStr">
@@ -60374,7 +60207,6 @@
       <c r="F45" t="b">
         <v>1</v>
       </c>
-      <c r="G45" t="inlineStr"/>
     </row>
     <row r="46">
       <c r="A46" t="inlineStr">
@@ -60405,7 +60237,6 @@
       <c r="F46" t="b">
         <v>1</v>
       </c>
-      <c r="G46" t="inlineStr"/>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
@@ -60436,7 +60267,6 @@
       <c r="F47" t="b">
         <v>1</v>
       </c>
-      <c r="G47" t="inlineStr"/>
     </row>
     <row r="48">
       <c r="A48" t="inlineStr">
@@ -60467,7 +60297,6 @@
       <c r="F48" t="b">
         <v>1</v>
       </c>
-      <c r="G48" t="inlineStr"/>
     </row>
     <row r="49">
       <c r="A49" t="inlineStr">
@@ -60498,7 +60327,6 @@
       <c r="F49" t="b">
         <v>1</v>
       </c>
-      <c r="G49" t="inlineStr"/>
     </row>
     <row r="50">
       <c r="A50" t="inlineStr">
@@ -60529,7 +60357,6 @@
       <c r="F50" t="b">
         <v>1</v>
       </c>
-      <c r="G50" t="inlineStr"/>
     </row>
     <row r="51">
       <c r="A51" t="inlineStr">
@@ -60560,7 +60387,6 @@
       <c r="F51" t="b">
         <v>1</v>
       </c>
-      <c r="G51" t="inlineStr"/>
     </row>
     <row r="52">
       <c r="A52" t="inlineStr">
@@ -60591,7 +60417,6 @@
       <c r="F52" t="b">
         <v>1</v>
       </c>
-      <c r="G52" t="inlineStr"/>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
@@ -60622,7 +60447,6 @@
       <c r="F53" t="b">
         <v>1</v>
       </c>
-      <c r="G53" t="inlineStr"/>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
@@ -60653,7 +60477,6 @@
       <c r="F54" t="b">
         <v>1</v>
       </c>
-      <c r="G54" t="inlineStr"/>
     </row>
     <row r="55">
       <c r="A55" t="inlineStr">
@@ -60684,7 +60507,6 @@
       <c r="F55" t="b">
         <v>1</v>
       </c>
-      <c r="G55" t="inlineStr"/>
     </row>
     <row r="56">
       <c r="A56" t="inlineStr">
@@ -60715,7 +60537,6 @@
       <c r="F56" t="b">
         <v>1</v>
       </c>
-      <c r="G56" t="inlineStr"/>
     </row>
     <row r="57">
       <c r="A57" t="inlineStr">
@@ -60746,7 +60567,6 @@
       <c r="F57" t="b">
         <v>1</v>
       </c>
-      <c r="G57" t="inlineStr"/>
     </row>
     <row r="58">
       <c r="A58" t="inlineStr">
@@ -60777,7 +60597,6 @@
       <c r="F58" t="b">
         <v>1</v>
       </c>
-      <c r="G58" t="inlineStr"/>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
@@ -60808,7 +60627,6 @@
       <c r="F59" t="b">
         <v>1</v>
       </c>
-      <c r="G59" t="inlineStr"/>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
@@ -60839,7 +60657,6 @@
       <c r="F60" t="b">
         <v>1</v>
       </c>
-      <c r="G60" t="inlineStr"/>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
@@ -60870,7 +60687,6 @@
       <c r="F61" t="b">
         <v>1</v>
       </c>
-      <c r="G61" t="inlineStr"/>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
@@ -60901,7 +60717,6 @@
       <c r="F62" t="b">
         <v>1</v>
       </c>
-      <c r="G62" t="inlineStr"/>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
@@ -60932,7 +60747,6 @@
       <c r="F63" t="b">
         <v>1</v>
       </c>
-      <c r="G63" t="inlineStr"/>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
@@ -60963,7 +60777,6 @@
       <c r="F64" t="b">
         <v>1</v>
       </c>
-      <c r="G64" t="inlineStr"/>
     </row>
     <row r="65">
       <c r="A65" t="inlineStr">
@@ -61701,6 +61514,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:G85"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -61713,44 +61527,54 @@
   </sheetPr>
   <dimension ref="A1:H25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="24" customWidth="1" min="2" max="2"/>
+    <col width="17" customWidth="1" min="3" max="3"/>
+    <col width="15" customWidth="1" min="4" max="4"/>
+    <col width="24" customWidth="1" min="5" max="5"/>
+    <col width="15" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="55" customWidth="1" min="8" max="8"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>regra_origem</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>tabela_destino</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>campo</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>coluna_origem</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -62669,6 +62493,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:H25"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -62681,64 +62506,78 @@
   </sheetPr>
   <dimension ref="A1:L54"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="19" customWidth="1" min="1" max="1"/>
+    <col width="19" customWidth="1" min="2" max="2"/>
+    <col width="24" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="23" customWidth="1" min="6" max="6"/>
+    <col width="41" customWidth="1" min="7" max="7"/>
+    <col width="15" customWidth="1" min="8" max="8"/>
+    <col width="13" customWidth="1" min="9" max="9"/>
+    <col width="22" customWidth="1" min="10" max="10"/>
+    <col width="12" customWidth="1" min="11" max="11"/>
+    <col width="55" customWidth="1" min="12" max="12"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>regra_origem</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>tipo_regra</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>prioridade</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>padrao_regex</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>subcategoria</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>local</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>extrair_subcategoria</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -62760,7 +62599,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D2" t="inlineStr"/>
       <c r="E2" t="inlineStr">
         <is>
           <t>controle\ de\ qualidade</t>
@@ -62771,13 +62609,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G2" t="inlineStr"/>
       <c r="H2" t="inlineStr">
         <is>
           <t>AMOSTRA</t>
         </is>
       </c>
-      <c r="I2" t="inlineStr"/>
       <c r="J2" t="b">
         <v>0</v>
       </c>
@@ -62806,7 +62642,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D3" t="inlineStr"/>
       <c r="E3" t="inlineStr">
         <is>
           <t>branco\ \-\ físico\-químico\.parâmetros</t>
@@ -62817,13 +62652,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr"/>
       <c r="H3" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I3" t="inlineStr"/>
       <c r="J3" t="b">
         <v>0</v>
       </c>
@@ -62852,7 +62685,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D4" t="inlineStr"/>
       <c r="E4" t="inlineStr">
         <is>
           <t>branco\ \-\ físico\-químico\.número\ do\ cq</t>
@@ -62863,13 +62695,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr"/>
       <c r="H4" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr"/>
       <c r="J4" t="b">
         <v>0</v>
       </c>
@@ -62898,7 +62728,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D5" t="inlineStr"/>
       <c r="E5" t="inlineStr">
         <is>
           <t>branco\ \-\ físico\-químico\.resultado</t>
@@ -62909,13 +62738,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G5" t="inlineStr"/>
       <c r="H5" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I5" t="inlineStr"/>
       <c r="J5" t="b">
         <v>0</v>
       </c>
@@ -62944,7 +62771,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D6" t="inlineStr"/>
       <c r="E6" t="inlineStr">
         <is>
           <t>branco\ \-\ físico\-químico\.unidade</t>
@@ -62955,13 +62781,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G6" t="inlineStr"/>
       <c r="H6" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I6" t="inlineStr"/>
       <c r="J6" t="b">
         <v>0</v>
       </c>
@@ -62990,7 +62814,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D7" t="inlineStr"/>
       <c r="E7" t="inlineStr">
         <is>
           <t>branco\ \-\ físico\-químico\.limite\ de\ quantificação</t>
@@ -63001,13 +62824,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G7" t="inlineStr"/>
       <c r="H7" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I7" t="inlineStr"/>
       <c r="J7" t="b">
         <v>0</v>
       </c>
@@ -63036,7 +62857,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D8" t="inlineStr"/>
       <c r="E8" t="inlineStr">
         <is>
           <t>branco\ \-\ metais\.parâmetros</t>
@@ -63047,13 +62867,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G8" t="inlineStr"/>
       <c r="H8" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I8" t="inlineStr"/>
       <c r="J8" t="b">
         <v>0</v>
       </c>
@@ -63082,7 +62900,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr"/>
       <c r="E9" t="inlineStr">
         <is>
           <t>branco\ \-\ metais\.número\ do\ cq</t>
@@ -63093,13 +62910,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G9" t="inlineStr"/>
       <c r="H9" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I9" t="inlineStr"/>
       <c r="J9" t="b">
         <v>0</v>
       </c>
@@ -63128,7 +62943,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr"/>
       <c r="E10" t="inlineStr">
         <is>
           <t>branco\ \-\ metais\.resultado</t>
@@ -63139,13 +62953,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G10" t="inlineStr"/>
       <c r="H10" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I10" t="inlineStr"/>
       <c r="J10" t="b">
         <v>0</v>
       </c>
@@ -63174,7 +62986,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D11" t="inlineStr"/>
       <c r="E11" t="inlineStr">
         <is>
           <t>branco\ \-\ metais\.unidade</t>
@@ -63185,13 +62996,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G11" t="inlineStr"/>
       <c r="H11" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I11" t="inlineStr"/>
       <c r="J11" t="b">
         <v>0</v>
       </c>
@@ -63220,7 +63029,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D12" t="inlineStr"/>
       <c r="E12" t="inlineStr">
         <is>
           <t>branco\ \-\ metais\.limite\ de\ quantificação</t>
@@ -63231,13 +63039,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G12" t="inlineStr"/>
       <c r="H12" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I12" t="inlineStr"/>
       <c r="J12" t="b">
         <v>0</v>
       </c>
@@ -63266,7 +63072,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D13" t="inlineStr"/>
       <c r="E13" t="inlineStr">
         <is>
           <t>branco\ \-\ microbiológicos\.parâmetros</t>
@@ -63277,13 +63082,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G13" t="inlineStr"/>
       <c r="H13" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I13" t="inlineStr"/>
       <c r="J13" t="b">
         <v>0</v>
       </c>
@@ -63312,7 +63115,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D14" t="inlineStr"/>
       <c r="E14" t="inlineStr">
         <is>
           <t>branco\ \-\ microbiológicos\.número\ do\ cq</t>
@@ -63323,13 +63125,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G14" t="inlineStr"/>
       <c r="H14" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I14" t="inlineStr"/>
       <c r="J14" t="b">
         <v>0</v>
       </c>
@@ -63358,7 +63158,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D15" t="inlineStr"/>
       <c r="E15" t="inlineStr">
         <is>
           <t>branco\ \-\ microbiológicos\.resultado</t>
@@ -63369,13 +63168,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G15" t="inlineStr"/>
       <c r="H15" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I15" t="inlineStr"/>
       <c r="J15" t="b">
         <v>0</v>
       </c>
@@ -63404,7 +63201,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D16" t="inlineStr"/>
       <c r="E16" t="inlineStr">
         <is>
           <t>branco\ \-\ microbiológicos\.unidade</t>
@@ -63415,13 +63211,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G16" t="inlineStr"/>
       <c r="H16" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I16" t="inlineStr"/>
       <c r="J16" t="b">
         <v>0</v>
       </c>
@@ -63450,7 +63244,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D17" t="inlineStr"/>
       <c r="E17" t="inlineStr">
         <is>
           <t>branco\ \-\ microbiológicos\.limite\ de\ quantificação</t>
@@ -63461,13 +63254,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G17" t="inlineStr"/>
       <c r="H17" t="inlineStr">
         <is>
           <t>BRANCO</t>
         </is>
       </c>
-      <c r="I17" t="inlineStr"/>
       <c r="J17" t="b">
         <v>0</v>
       </c>
@@ -63496,7 +63287,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D18" t="inlineStr"/>
       <c r="E18" t="inlineStr">
         <is>
           <t>duplicata\ \-\ físico\-químico\.parâmetros</t>
@@ -63507,13 +63297,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G18" t="inlineStr"/>
       <c r="H18" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I18" t="inlineStr"/>
       <c r="J18" t="b">
         <v>0</v>
       </c>
@@ -63542,7 +63330,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D19" t="inlineStr"/>
       <c r="E19" t="inlineStr">
         <is>
           <t>duplicata\ \-\ físico\-químico\.número\ do\ cq</t>
@@ -63553,13 +63340,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G19" t="inlineStr"/>
       <c r="H19" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I19" t="inlineStr"/>
       <c r="J19" t="b">
         <v>0</v>
       </c>
@@ -63588,7 +63373,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D20" t="inlineStr"/>
       <c r="E20" t="inlineStr">
         <is>
           <t>duplicata\ \-\ físico\-químico\.resultado</t>
@@ -63599,13 +63383,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G20" t="inlineStr"/>
       <c r="H20" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I20" t="inlineStr"/>
       <c r="J20" t="b">
         <v>0</v>
       </c>
@@ -63634,7 +63416,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D21" t="inlineStr"/>
       <c r="E21" t="inlineStr">
         <is>
           <t>duplicata\ \-\ físico\-químico\.duplicata</t>
@@ -63645,13 +63426,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G21" t="inlineStr"/>
       <c r="H21" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I21" t="inlineStr"/>
       <c r="J21" t="b">
         <v>0</v>
       </c>
@@ -63680,7 +63459,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D22" t="inlineStr"/>
       <c r="E22" t="inlineStr">
         <is>
           <t>duplicata\ \-\ físico\-químico\.unidade</t>
@@ -63691,13 +63469,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G22" t="inlineStr"/>
       <c r="H22" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I22" t="inlineStr"/>
       <c r="J22" t="b">
         <v>0</v>
       </c>
@@ -63726,7 +63502,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D23" t="inlineStr"/>
       <c r="E23" t="inlineStr">
         <is>
           <t>duplicata\ \-\ físico\-químico\.faixa\ de\ aceitação</t>
@@ -63737,13 +63512,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G23" t="inlineStr"/>
       <c r="H23" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I23" t="inlineStr"/>
       <c r="J23" t="b">
         <v>0</v>
       </c>
@@ -63772,7 +63545,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D24" t="inlineStr"/>
       <c r="E24" t="inlineStr">
         <is>
           <t>duplicata\ \-\ físico\-químico\.variação\ \(%\)</t>
@@ -63783,13 +63555,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G24" t="inlineStr"/>
       <c r="H24" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I24" t="inlineStr"/>
       <c r="J24" t="b">
         <v>0</v>
       </c>
@@ -63818,7 +63588,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D25" t="inlineStr"/>
       <c r="E25" t="inlineStr">
         <is>
           <t>duplicata\ \-\ metais\.parâmetros</t>
@@ -63829,13 +63598,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G25" t="inlineStr"/>
       <c r="H25" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I25" t="inlineStr"/>
       <c r="J25" t="b">
         <v>0</v>
       </c>
@@ -63864,7 +63631,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D26" t="inlineStr"/>
       <c r="E26" t="inlineStr">
         <is>
           <t>duplicata\ \-\ metais\.número\ do\ cq</t>
@@ -63875,13 +63641,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G26" t="inlineStr"/>
       <c r="H26" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I26" t="inlineStr"/>
       <c r="J26" t="b">
         <v>0</v>
       </c>
@@ -63910,7 +63674,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D27" t="inlineStr"/>
       <c r="E27" t="inlineStr">
         <is>
           <t>duplicata\ \-\ metais\.resultado</t>
@@ -63921,13 +63684,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G27" t="inlineStr"/>
       <c r="H27" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I27" t="inlineStr"/>
       <c r="J27" t="b">
         <v>0</v>
       </c>
@@ -63956,7 +63717,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D28" t="inlineStr"/>
       <c r="E28" t="inlineStr">
         <is>
           <t>duplicata\ \-\ metais\.duplicata</t>
@@ -63967,13 +63727,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G28" t="inlineStr"/>
       <c r="H28" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I28" t="inlineStr"/>
       <c r="J28" t="b">
         <v>0</v>
       </c>
@@ -64002,7 +63760,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D29" t="inlineStr"/>
       <c r="E29" t="inlineStr">
         <is>
           <t>duplicata\ \-\ metais\.unidade</t>
@@ -64013,13 +63770,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G29" t="inlineStr"/>
       <c r="H29" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I29" t="inlineStr"/>
       <c r="J29" t="b">
         <v>0</v>
       </c>
@@ -64048,7 +63803,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D30" t="inlineStr"/>
       <c r="E30" t="inlineStr">
         <is>
           <t>duplicata\ \-\ metais\.faixa\ de\ aceitação</t>
@@ -64059,13 +63813,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G30" t="inlineStr"/>
       <c r="H30" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I30" t="inlineStr"/>
       <c r="J30" t="b">
         <v>0</v>
       </c>
@@ -64094,7 +63846,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D31" t="inlineStr"/>
       <c r="E31" t="inlineStr">
         <is>
           <t>duplicata\ \-\ metais\.variação\ \(%\)</t>
@@ -64105,13 +63856,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G31" t="inlineStr"/>
       <c r="H31" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I31" t="inlineStr"/>
       <c r="J31" t="b">
         <v>0</v>
       </c>
@@ -64140,7 +63889,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D32" t="inlineStr"/>
       <c r="E32" t="inlineStr">
         <is>
           <t>duplicata\ \-\ microbiológicos\.parâmetros</t>
@@ -64151,13 +63899,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G32" t="inlineStr"/>
       <c r="H32" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I32" t="inlineStr"/>
       <c r="J32" t="b">
         <v>0</v>
       </c>
@@ -64186,7 +63932,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D33" t="inlineStr"/>
       <c r="E33" t="inlineStr">
         <is>
           <t>duplicata\ \-\ microbiológicos\.número\ do\ cq</t>
@@ -64197,13 +63942,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G33" t="inlineStr"/>
       <c r="H33" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I33" t="inlineStr"/>
       <c r="J33" t="b">
         <v>0</v>
       </c>
@@ -64232,7 +63975,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D34" t="inlineStr"/>
       <c r="E34" t="inlineStr">
         <is>
           <t>duplicata\ \-\ microbiológicos\.resultado</t>
@@ -64243,13 +63985,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G34" t="inlineStr"/>
       <c r="H34" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I34" t="inlineStr"/>
       <c r="J34" t="b">
         <v>0</v>
       </c>
@@ -64278,7 +64018,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D35" t="inlineStr"/>
       <c r="E35" t="inlineStr">
         <is>
           <t>duplicata\ \-\ microbiológicos\.duplicata</t>
@@ -64289,13 +64028,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G35" t="inlineStr"/>
       <c r="H35" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I35" t="inlineStr"/>
       <c r="J35" t="b">
         <v>0</v>
       </c>
@@ -64324,7 +64061,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D36" t="inlineStr"/>
       <c r="E36" t="inlineStr">
         <is>
           <t>duplicata\ \-\ microbiológicos\.unidade</t>
@@ -64335,13 +64071,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G36" t="inlineStr"/>
       <c r="H36" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I36" t="inlineStr"/>
       <c r="J36" t="b">
         <v>0</v>
       </c>
@@ -64370,7 +64104,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D37" t="inlineStr"/>
       <c r="E37" t="inlineStr">
         <is>
           <t>duplicata\ \-\ microbiológicos\.faixa\ de\ aceitação</t>
@@ -64381,13 +64114,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G37" t="inlineStr"/>
       <c r="H37" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I37" t="inlineStr"/>
       <c r="J37" t="b">
         <v>0</v>
       </c>
@@ -64416,7 +64147,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D38" t="inlineStr"/>
       <c r="E38" t="inlineStr">
         <is>
           <t>duplicata\ \-\ microbiológicos\.variação\ \(%\)</t>
@@ -64427,13 +64157,11 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G38" t="inlineStr"/>
       <c r="H38" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
         </is>
       </c>
-      <c r="I38" t="inlineStr"/>
       <c r="J38" t="b">
         <v>0</v>
       </c>
@@ -64462,7 +64190,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D39" t="inlineStr"/>
       <c r="E39" t="inlineStr">
         <is>
           <t>^resultados\s+analiticos</t>
@@ -64473,8 +64200,6 @@
           <t>Resultados Analíticos</t>
         </is>
       </c>
-      <c r="G39" t="inlineStr"/>
-      <c r="H39" t="inlineStr"/>
       <c r="I39" t="inlineStr">
         <is>
           <t>laboratorio</t>
@@ -64508,7 +64233,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D40" t="inlineStr"/>
       <c r="E40" t="inlineStr">
         <is>
           <t>^controle\s+de\s+qualidade</t>
@@ -64519,8 +64243,6 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G40" t="inlineStr"/>
-      <c r="H40" t="inlineStr"/>
       <c r="I40" t="inlineStr">
         <is>
           <t>laboratorio</t>
@@ -64554,7 +64276,6 @@
           <t>template_laudo_agua_v1</t>
         </is>
       </c>
-      <c r="D41" t="inlineStr"/>
       <c r="E41" t="inlineStr">
         <is>
           <t>^(provedores?\s+externos?|ethica\s+ambiental)</t>
@@ -64565,8 +64286,6 @@
           <t>Provedores Externos</t>
         </is>
       </c>
-      <c r="G41" t="inlineStr"/>
-      <c r="H41" t="inlineStr"/>
       <c r="I41" t="inlineStr">
         <is>
           <t>laboratorio</t>
@@ -65173,7 +64892,6 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G52" t="inlineStr"/>
       <c r="H52" t="inlineStr">
         <is>
           <t>BRANCO</t>
@@ -65225,7 +64943,6 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G53" t="inlineStr"/>
       <c r="H53" t="inlineStr">
         <is>
           <t>DUPLICATA</t>
@@ -65277,7 +64994,6 @@
           <t>Controle de Qualidade</t>
         </is>
       </c>
-      <c r="G54" t="inlineStr"/>
       <c r="H54" t="inlineStr">
         <is>
           <t>RECUPERACAO</t>
@@ -65301,6 +65017,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:L54"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -65313,29 +65030,36 @@
   </sheetPr>
   <dimension ref="A1:E4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="24" customWidth="1" min="1" max="1"/>
+    <col width="15" customWidth="1" min="2" max="2"/>
+    <col width="14" customWidth="1" min="3" max="3"/>
+    <col width="12" customWidth="1" min="4" max="4"/>
+    <col width="55" customWidth="1" min="5" max="5"/>
+  </cols>
   <sheetData>
-    <row r="1">
-      <c r="A1" t="inlineStr">
+    <row r="1" ht="28" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>padrao_regex</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -65417,6 +65141,7 @@
       </c>
     </row>
   </sheetData>
+  <autoFilter ref="A1:E4"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Map normative headers from taxonomy
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_consolidada_v1.xlsx
+++ b/config/taxonomy_config_consolidada_v1.xlsx
@@ -22,7 +22,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'template_rules'!$A$1:$G$78</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'output_model'!$A$1:$L$75</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'text_extraction_rules'!$A$1:$G$85</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'table_extraction_rules'!$A$1:$H$25</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'table_extraction_rules'!$A$1:$I$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'section_rules'!$A$1:$L$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'continuation_rules'!$A$1:$E$4</definedName>
   </definedNames>
@@ -85,10 +85,13 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -460,21 +463,21 @@
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
     <col width="24" customWidth="1" min="2" max="2"/>
-    <col width="55" customWidth="1" min="3" max="3"/>
+    <col width="60" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>ordem</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>aba</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -551,7 +554,7 @@
       </c>
       <c r="C6" t="inlineStr">
         <is>
-          <t>Regras de extracao tabular por tipo de registro e campo de saida.</t>
+          <t>Regras de extracao tabular por tipo de registro, campo de saida e aliases de cabecalho.</t>
         </is>
       </c>
     </row>
@@ -604,49 +607,49 @@
     <col width="27" customWidth="1" min="2" max="2"/>
     <col width="54" customWidth="1" min="3" max="3"/>
     <col width="17" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
     <col width="14" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>theme_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>nome</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>schema_ref</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>prioridade</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>score_minimo</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
@@ -1174,44 +1177,44 @@
     <col width="39" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="12" customWidth="1" min="3" max="3"/>
-    <col width="55" customWidth="1" min="4" max="4"/>
+    <col width="60" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>tipo_regra</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>fonte</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>padrao_regex</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>peso</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -3778,72 +3781,72 @@
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
-    <col width="55" customWidth="1" min="6" max="6"/>
+    <col width="60" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
     <col width="28" customWidth="1" min="8" max="8"/>
     <col width="19" customWidth="1" min="9" max="9"/>
     <col width="13" customWidth="1" min="10" max="10"/>
-    <col width="55" customWidth="1" min="11" max="11"/>
-    <col width="55" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="11" max="11"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>theme_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>sheet_name</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>ordem_aba</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>ativo_aba</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>descricao_aba</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>ordem_campo</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>campo</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>tipo_dado</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>obrigatorio</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>origem</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -7810,43 +7813,43 @@
     <col width="29" customWidth="1" min="2" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="28" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
     <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="55" customWidth="1" min="7" max="7"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>regra_origem</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>tabela_destino</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>campo</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>padrao_regex</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -10804,7 +10807,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H25"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10813,47 +10816,53 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="12" customWidth="1" min="7" max="7"/>
-    <col width="55" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="12" customWidth="1" min="8" max="8"/>
+    <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>regra_origem</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>tabela_destino</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>campo</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>coluna_origem</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
+        <is>
+          <t>header_regex</t>
+        </is>
+      </c>
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -10888,10 +10897,15 @@
       <c r="F2" t="n">
         <v>4</v>
       </c>
-      <c r="G2" t="b">
-        <v>1</v>
-      </c>
-      <c r="H2" t="inlineStr">
+      <c r="G2" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H2" t="b">
+        <v>1</v>
+      </c>
+      <c r="I2" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -10926,10 +10940,15 @@
       <c r="F3" t="n">
         <v>1</v>
       </c>
-      <c r="G3" t="b">
-        <v>1</v>
-      </c>
-      <c r="H3" t="inlineStr">
+      <c r="G3" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H3" t="b">
+        <v>1</v>
+      </c>
+      <c r="I3" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -10964,10 +10983,15 @@
       <c r="F4" t="n">
         <v>2</v>
       </c>
-      <c r="G4" t="b">
-        <v>1</v>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="G4" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H4" t="b">
+        <v>1</v>
+      </c>
+      <c r="I4" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11002,10 +11026,15 @@
       <c r="F5" t="n">
         <v>3</v>
       </c>
-      <c r="G5" t="b">
-        <v>1</v>
-      </c>
-      <c r="H5" t="inlineStr">
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H5" t="b">
+        <v>1</v>
+      </c>
+      <c r="I5" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11040,10 +11069,15 @@
       <c r="F6" t="n">
         <v>5</v>
       </c>
-      <c r="G6" t="b">
-        <v>1</v>
-      </c>
-      <c r="H6" t="inlineStr">
+      <c r="G6" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H6" t="b">
+        <v>1</v>
+      </c>
+      <c r="I6" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11078,10 +11112,15 @@
       <c r="F7" t="n">
         <v>6</v>
       </c>
-      <c r="G7" t="b">
-        <v>1</v>
-      </c>
-      <c r="H7" t="inlineStr">
+      <c r="G7" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H7" t="b">
+        <v>1</v>
+      </c>
+      <c r="I7" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11116,10 +11155,15 @@
       <c r="F8" t="n">
         <v>7</v>
       </c>
-      <c r="G8" t="b">
-        <v>1</v>
-      </c>
-      <c r="H8" t="inlineStr">
+      <c r="G8" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H8" t="b">
+        <v>1</v>
+      </c>
+      <c r="I8" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11154,10 +11198,15 @@
       <c r="F9" t="n">
         <v>8</v>
       </c>
-      <c r="G9" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="G9" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H9" t="b">
+        <v>1</v>
+      </c>
+      <c r="I9" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11192,10 +11241,15 @@
       <c r="F10" t="n">
         <v>2</v>
       </c>
-      <c r="G10" t="b">
-        <v>1</v>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="G10" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H10" t="b">
+        <v>1</v>
+      </c>
+      <c r="I10" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11230,10 +11284,15 @@
       <c r="F11" t="n">
         <v>3</v>
       </c>
-      <c r="G11" t="b">
-        <v>1</v>
-      </c>
-      <c r="H11" t="inlineStr">
+      <c r="G11" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H11" t="b">
+        <v>1</v>
+      </c>
+      <c r="I11" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11268,10 +11327,15 @@
       <c r="F12" t="n">
         <v>4</v>
       </c>
-      <c r="G12" t="b">
-        <v>1</v>
-      </c>
-      <c r="H12" t="inlineStr">
+      <c r="G12" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H12" t="b">
+        <v>1</v>
+      </c>
+      <c r="I12" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11306,10 +11370,15 @@
       <c r="F13" t="n">
         <v>1</v>
       </c>
-      <c r="G13" t="b">
-        <v>1</v>
-      </c>
-      <c r="H13" t="inlineStr">
+      <c r="G13" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H13" t="b">
+        <v>1</v>
+      </c>
+      <c r="I13" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11344,10 +11413,15 @@
       <c r="F14" t="n">
         <v>2</v>
       </c>
-      <c r="G14" t="b">
-        <v>1</v>
-      </c>
-      <c r="H14" t="inlineStr">
+      <c r="G14" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H14" t="b">
+        <v>1</v>
+      </c>
+      <c r="I14" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11382,10 +11456,15 @@
       <c r="F15" t="n">
         <v>4</v>
       </c>
-      <c r="G15" t="b">
-        <v>1</v>
-      </c>
-      <c r="H15" t="inlineStr">
+      <c r="G15" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H15" t="b">
+        <v>1</v>
+      </c>
+      <c r="I15" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11420,10 +11499,15 @@
       <c r="F16" t="n">
         <v>1</v>
       </c>
-      <c r="G16" t="b">
-        <v>1</v>
-      </c>
-      <c r="H16" t="inlineStr">
+      <c r="G16" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H16" t="b">
+        <v>1</v>
+      </c>
+      <c r="I16" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11458,10 +11542,15 @@
       <c r="F17" t="n">
         <v>3</v>
       </c>
-      <c r="G17" t="b">
-        <v>1</v>
-      </c>
-      <c r="H17" t="inlineStr">
+      <c r="G17" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H17" t="b">
+        <v>1</v>
+      </c>
+      <c r="I17" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11496,10 +11585,15 @@
       <c r="F18" t="n">
         <v>5</v>
       </c>
-      <c r="G18" t="b">
-        <v>1</v>
-      </c>
-      <c r="H18" t="inlineStr">
+      <c r="G18" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H18" t="b">
+        <v>1</v>
+      </c>
+      <c r="I18" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11534,10 +11628,15 @@
       <c r="F19" t="n">
         <v>6</v>
       </c>
-      <c r="G19" t="b">
-        <v>1</v>
-      </c>
-      <c r="H19" t="inlineStr">
+      <c r="G19" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H19" t="b">
+        <v>1</v>
+      </c>
+      <c r="I19" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11572,10 +11671,15 @@
       <c r="F20" t="n">
         <v>5</v>
       </c>
-      <c r="G20" t="b">
-        <v>1</v>
-      </c>
-      <c r="H20" t="inlineStr">
+      <c r="G20" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H20" t="b">
+        <v>1</v>
+      </c>
+      <c r="I20" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11610,10 +11714,15 @@
       <c r="F21" t="n">
         <v>3</v>
       </c>
-      <c r="G21" t="b">
-        <v>1</v>
-      </c>
-      <c r="H21" t="inlineStr">
+      <c r="G21" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H21" t="b">
+        <v>1</v>
+      </c>
+      <c r="I21" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11648,10 +11757,15 @@
       <c r="F22" t="n">
         <v>1</v>
       </c>
-      <c r="G22" t="b">
-        <v>1</v>
-      </c>
-      <c r="H22" t="inlineStr">
+      <c r="G22" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H22" t="b">
+        <v>1</v>
+      </c>
+      <c r="I22" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11686,10 +11800,15 @@
       <c r="F23" t="n">
         <v>4</v>
       </c>
-      <c r="G23" t="b">
-        <v>1</v>
-      </c>
-      <c r="H23" t="inlineStr">
+      <c r="G23" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H23" t="b">
+        <v>1</v>
+      </c>
+      <c r="I23" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11724,10 +11843,15 @@
       <c r="F24" t="n">
         <v>2</v>
       </c>
-      <c r="G24" t="b">
-        <v>1</v>
-      </c>
-      <c r="H24" t="inlineStr">
+      <c r="G24" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H24" t="b">
+        <v>1</v>
+      </c>
+      <c r="I24" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
@@ -11762,17 +11886,697 @@
       <c r="F25" t="n">
         <v>5</v>
       </c>
-      <c r="G25" t="b">
-        <v>1</v>
-      </c>
-      <c r="H25" t="inlineStr">
+      <c r="G25" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="H25" t="b">
+        <v>1</v>
+      </c>
+      <c r="I25" t="inlineStr">
         <is>
           <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
         </is>
       </c>
     </row>
+    <row r="26">
+      <c r="A26" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B26" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D26" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E26" t="inlineStr">
+        <is>
+          <t>parameter</t>
+        </is>
+      </c>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G26" t="inlineStr">
+        <is>
+          <t>^(analise|parametros?)$</t>
+        </is>
+      </c>
+      <c r="H26" t="b">
+        <v>1</v>
+      </c>
+      <c r="I26" t="inlineStr">
+        <is>
+          <t>Reconhece a coluna de parametro/analise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B27" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D27" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E27" t="inlineStr">
+        <is>
+          <t>unidade</t>
+        </is>
+      </c>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G27" t="inlineStr">
+        <is>
+          <t>^(unidade|unid)$</t>
+        </is>
+      </c>
+      <c r="H27" t="b">
+        <v>1</v>
+      </c>
+      <c r="I27" t="inlineStr">
+        <is>
+          <t>Reconhece a coluna de unidade de medida.</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B28" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C28" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D28" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E28" t="inlineStr">
+        <is>
+          <t>ld</t>
+        </is>
+      </c>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G28" t="inlineStr">
+        <is>
+          <t>(^ld$|limite\s+de\s+deteccao)</t>
+        </is>
+      </c>
+      <c r="H28" t="b">
+        <v>1</v>
+      </c>
+      <c r="I28" t="inlineStr">
+        <is>
+          <t>Reconhece a coluna de limite de deteccao.</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B29" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D29" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E29" t="inlineStr">
+        <is>
+          <t>lq</t>
+        </is>
+      </c>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G29" t="inlineStr">
+        <is>
+          <t>(^lq$|limite\s+de\s+quantificacao)</t>
+        </is>
+      </c>
+      <c r="H29" t="b">
+        <v>1</v>
+      </c>
+      <c r="I29" t="inlineStr">
+        <is>
+          <t>Reconhece a coluna de limite de quantificacao.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B30" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C30" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D30" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E30" t="inlineStr">
+        <is>
+          <t>resultado</t>
+        </is>
+      </c>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G30" t="inlineStr">
+        <is>
+          <t>^resultados?$</t>
+        </is>
+      </c>
+      <c r="H30" t="b">
+        <v>1</v>
+      </c>
+      <c r="I30" t="inlineStr">
+        <is>
+          <t>Reconhece a coluna de resultado.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B31" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C31" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D31" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>incerteza</t>
+        </is>
+      </c>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G31" t="inlineStr">
+        <is>
+          <t>incerteza</t>
+        </is>
+      </c>
+      <c r="H31" t="b">
+        <v>1</v>
+      </c>
+      <c r="I31" t="inlineStr">
+        <is>
+          <t>Reconhece a coluna de incerteza.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B32" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C32" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D32" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E32" t="inlineStr">
+        <is>
+          <t>referencia</t>
+        </is>
+      </c>
+      <c r="F32" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G32" t="inlineStr">
+        <is>
+          <t>referencia</t>
+        </is>
+      </c>
+      <c r="H32" t="b">
+        <v>1</v>
+      </c>
+      <c r="I32" t="inlineStr">
+        <is>
+          <t>Reconhece a coluna de referencia metodologica.</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B33" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C33" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D33" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E33" t="inlineStr">
+        <is>
+          <t>data_inicio</t>
+        </is>
+      </c>
+      <c r="F33" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G33" t="inlineStr">
+        <is>
+          <t>data\s+de\s+inicio|data\s+inicio</t>
+        </is>
+      </c>
+      <c r="H33" t="b">
+        <v>1</v>
+      </c>
+      <c r="I33" t="inlineStr">
+        <is>
+          <t>Reconhece a coluna de data de inicio da analise.</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B34" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C34" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D34" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E34" t="inlineStr">
+        <is>
+          <t>numero_cq</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G34" t="inlineStr">
+        <is>
+          <t>numero\s+do\s+cq|^cq$</t>
+        </is>
+      </c>
+      <c r="H34" t="b">
+        <v>1</v>
+      </c>
+      <c r="I34" t="inlineStr">
+        <is>
+          <t>Reconhece a coluna de numero do controle de qualidade.</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B35" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D35" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E35" t="inlineStr">
+        <is>
+          <t>duplicata</t>
+        </is>
+      </c>
+      <c r="F35" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G35" t="inlineStr">
+        <is>
+          <t>^duplicata$</t>
+        </is>
+      </c>
+      <c r="H35" t="b">
+        <v>1</v>
+      </c>
+      <c r="I35" t="inlineStr">
+        <is>
+          <t>Reconhece a coluna de duplicata.</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B36" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D36" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E36" t="inlineStr">
+        <is>
+          <t>faixa_aceitacao</t>
+        </is>
+      </c>
+      <c r="F36" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G36" t="inlineStr">
+        <is>
+          <t>faixa\s+de\s+aceitacao</t>
+        </is>
+      </c>
+      <c r="H36" t="b">
+        <v>1</v>
+      </c>
+      <c r="I36" t="inlineStr">
+        <is>
+          <t>Reconhece a coluna de faixa de aceitacao.</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B37" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C37" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D37" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E37" t="inlineStr">
+        <is>
+          <t>variacao_percentual</t>
+        </is>
+      </c>
+      <c r="F37" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G37" t="inlineStr">
+        <is>
+          <t>variacao</t>
+        </is>
+      </c>
+      <c r="H37" t="b">
+        <v>1</v>
+      </c>
+      <c r="I37" t="inlineStr">
+        <is>
+          <t>Reconhece a coluna de variacao percentual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B38" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D38" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E38" t="inlineStr">
+        <is>
+          <t>quantidade_adicionada</t>
+        </is>
+      </c>
+      <c r="F38" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G38" t="inlineStr">
+        <is>
+          <t>quantidade\s+adicionada|^qtd\s+adicionada$</t>
+        </is>
+      </c>
+      <c r="H38" t="b">
+        <v>1</v>
+      </c>
+      <c r="I38" t="inlineStr">
+        <is>
+          <t>Reconhece a coluna de quantidade adicionada.</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B39" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C39" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D39" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E39" t="inlineStr">
+        <is>
+          <t>recuperacao_percentual</t>
+        </is>
+      </c>
+      <c r="F39" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G39" t="inlineStr">
+        <is>
+          <t>recuperacao</t>
+        </is>
+      </c>
+      <c r="H39" t="b">
+        <v>1</v>
+      </c>
+      <c r="I39" t="inlineStr">
+        <is>
+          <t>Reconhece a coluna de recuperacao percentual.</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B40" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C40" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D40" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E40" t="inlineStr">
+        <is>
+          <t>criterio_conformidade</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>resolucao|conama|criterio|deliberacao\s+normativa|copam|cerh</t>
+        </is>
+      </c>
+      <c r="H40" t="b">
+        <v>1</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Reconhece colunas normativas como criterio de conformidade, incluindo CONAMA e COPAM/CERH.</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H25"/>
+  <autoFilter ref="A1:I40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -11790,73 +12594,73 @@
     <col width="19" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
     <col width="15" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="56" customWidth="1" min="5" max="5"/>
     <col width="23" customWidth="1" min="6" max="6"/>
     <col width="41" customWidth="1" min="7" max="7"/>
     <col width="15" customWidth="1" min="8" max="8"/>
     <col width="15" customWidth="1" min="9" max="9"/>
     <col width="22" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
-    <col width="55" customWidth="1" min="12" max="12"/>
+    <col width="60" customWidth="1" min="12" max="12"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>regra_origem</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>tipo_regra</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>prioridade</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>padrao_regex</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" s="2" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" s="2" t="inlineStr">
         <is>
           <t>subcategoria</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" s="2" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" s="2" t="inlineStr">
         <is>
           <t>local</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" s="2" t="inlineStr">
         <is>
           <t>extrair_subcategoria</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" s="2" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" s="2" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -14929,31 +15733,31 @@
     <col width="15" customWidth="1" min="2" max="2"/>
     <col width="14" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
-    <col width="55" customWidth="1" min="5" max="5"/>
+    <col width="60" customWidth="1" min="5" max="5"/>
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" s="2" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" s="2" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" s="2" t="inlineStr">
         <is>
           <t>padrao_regex</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" s="2" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" s="2" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>

</xml_diff>

<commit_message>
Preserve source field names in results output
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_consolidada_v1.xlsx
+++ b/config/taxonomy_config_consolidada_v1.xlsx
@@ -467,17 +467,17 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>ordem</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>aba</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -614,42 +614,42 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>theme_id</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>nome</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>schema_ref</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>prioridade</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>score_minimo</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
@@ -1184,37 +1184,37 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>tipo_regra</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>fonte</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>padrao_regex</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>peso</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -3791,62 +3791,62 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>theme_id</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>sheet_name</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ordem_aba</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>ativo_aba</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>descricao_aba</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>ordem_campo</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>campo</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>tipo_dado</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>obrigatorio</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>origem</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>ld_original</t>
+          <t>ld</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -4707,12 +4707,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.ld_col</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>LD original extraido diretamente do PDF.</t>
+          <t>LD extraido diretamente do PDF, preservado como texto original.</t>
         </is>
       </c>
     </row>
@@ -4766,7 +4766,7 @@
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Valor minimo do LD gravado como numero no Excel, com casas decimais preservadas conforme o LD original.</t>
+          <t>Valor minimo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
         </is>
       </c>
     </row>
@@ -4820,7 +4820,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Valor maximo do LD gravado como numero no Excel, com casas decimais preservadas conforme o LD original.</t>
+          <t>Valor maximo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
         </is>
       </c>
     </row>
@@ -4874,7 +4874,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Unidade de medida do LD, quando informada no PDF.</t>
+          <t>Unidade de medida do LD, quando informada no campo ld.</t>
         </is>
       </c>
     </row>
@@ -4910,7 +4910,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>lq_original</t>
+          <t>lq</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -4923,12 +4923,12 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.lq_col</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Coluna lq_original da aba results_extract.</t>
+          <t>LQ extraido diretamente do PDF, preservado como texto original.</t>
         </is>
       </c>
     </row>
@@ -4982,7 +4982,7 @@
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Valor minimo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o LQ original.</t>
+          <t>Valor minimo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
         </is>
       </c>
     </row>
@@ -5036,7 +5036,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Valor maximo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o LQ original.</t>
+          <t>Valor maximo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
         </is>
       </c>
     </row>
@@ -5090,7 +5090,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Coluna lq_unidade da aba results_extract.</t>
+          <t>Unidade de medida do LQ, quando informada no campo lq.</t>
         </is>
       </c>
     </row>
@@ -5180,7 +5180,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>incerteza_original</t>
+          <t>incerteza</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -5193,12 +5193,12 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.incerteza_col</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Coluna incerteza_original da aba results_extract.</t>
+          <t>Incerteza extraida diretamente do PDF, preservada como texto original.</t>
         </is>
       </c>
     </row>
@@ -5252,7 +5252,7 @@
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Valor da incerteza gravado como numero no Excel, com casas decimais preservadas conforme a incerteza original.</t>
+          <t>Valor da incerteza gravado como numero no Excel, com casas decimais preservadas conforme o campo incerteza.</t>
         </is>
       </c>
     </row>
@@ -5306,7 +5306,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Coluna incerteza_unidade da aba results_extract.</t>
+          <t>Unidade de medida da incerteza, quando informada no campo incerteza.</t>
         </is>
       </c>
     </row>
@@ -5450,7 +5450,7 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_original</t>
+          <t>faixa_aceitacao</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
@@ -5463,12 +5463,12 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.faixa_aceitacao_col</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Coluna faixa_aceitacao_original da aba results_extract.</t>
+          <t>Faixa de aceitacao extraida diretamente do PDF, preservada como texto original.</t>
         </is>
       </c>
     </row>
@@ -5522,7 +5522,7 @@
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Coluna faixa_aceitacao_operador da aba results_extract.</t>
+          <t>Operador extraido da faixa de aceitacao, quando informado no PDF.</t>
         </is>
       </c>
     </row>
@@ -5576,7 +5576,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Valor minimo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme a faixa original.</t>
+          <t>Valor minimo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -5630,7 +5630,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Valor maximo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme a faixa original.</t>
+          <t>Valor maximo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -5684,7 +5684,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Coluna faixa_aceitacao_unidade da aba results_extract.</t>
+          <t>Unidade de medida da faixa de aceitacao, quando informada no campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -7819,37 +7819,37 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>regra_origem</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>tabela_destino</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>campo</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>padrao_regex</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -10822,47 +10822,47 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>regra_origem</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>tabela_destino</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>campo</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>coluna_origem</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>header_regex</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -12605,62 +12605,62 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>regra_origem</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>tipo_regra</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>prioridade</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>padrao_regex</t>
         </is>
       </c>
-      <c r="F1" s="2" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="G1" s="2" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>subcategoria</t>
         </is>
       </c>
-      <c r="H1" s="2" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="I1" s="2" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>local</t>
         </is>
       </c>
-      <c r="J1" s="2" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>extrair_subcategoria</t>
         </is>
       </c>
-      <c r="K1" s="2" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="L1" s="2" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
@@ -15737,27 +15737,27 @@
   </cols>
   <sheetData>
     <row r="1" ht="28" customHeight="1">
-      <c r="A1" s="2" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>template_id</t>
         </is>
       </c>
-      <c r="B1" s="2" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>tipo_registro</t>
         </is>
       </c>
-      <c r="C1" s="2" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>padrao_regex</t>
         </is>
       </c>
-      <c r="D1" s="2" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>ativo</t>
         </is>
       </c>
-      <c r="E1" s="2" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>

</xml_diff>

<commit_message>
Split normative reference from conformity criterion
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_consolidada_v1.xlsx
+++ b/config/taxonomy_config_consolidada_v1.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README_FORMATO'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'templates'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'template_rules'!$A$1:$G$78</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'output_model'!$A$1:$L$75</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'output_model'!$A$1:$L$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'text_extraction_rules'!$A$1:$G$85</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'table_extraction_rules'!$A$1:$I$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'section_rules'!$A$1:$L$54</definedName>
@@ -3773,7 +3773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L75"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4640,7 +4640,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>criterio_conformidade</t>
+          <t>referencia_normativa</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -4653,12 +4653,12 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>table_extraction_rules.criterio_conformidade_col</t>
+          <t>cabecalho_detectado.criterio_conformidade_col</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Criterio de conformidade extraido diretamente do PDF.</t>
+          <t>Nome da referencia normativa detectada no cabecalho da coluna de criterio, como CONAMA, COPAM/CERH ou deliberacao normativa.</t>
         </is>
       </c>
     </row>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>ld</t>
+          <t>criterio_conformidade</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -4707,12 +4707,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>table_extraction_rules.ld_col</t>
+          <t>table_extraction_rules.criterio_conformidade_col</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>LD extraido diretamente do PDF, preservado como texto original.</t>
+          <t>Valor do criterio de conformidade extraido da celula da tabela.</t>
         </is>
       </c>
     </row>
@@ -4748,12 +4748,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>ld_minimo</t>
+          <t>ld</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J18" t="b">
@@ -4761,12 +4761,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.ld_col</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Valor minimo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
+          <t>LD extraido diretamente do PDF, preservado como texto original.</t>
         </is>
       </c>
     </row>
@@ -4802,7 +4802,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ld_maximo</t>
+          <t>ld_minimo</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Valor maximo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
+          <t>Valor minimo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
         </is>
       </c>
     </row>
@@ -4856,12 +4856,12 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>ld_unidade</t>
+          <t>ld_maximo</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J20" t="b">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Unidade de medida do LD, quando informada no campo ld.</t>
+          <t>Valor maximo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
         </is>
       </c>
     </row>
@@ -4910,7 +4910,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>lq</t>
+          <t>ld_unidade</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -4923,12 +4923,12 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>table_extraction_rules.lq_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>LQ extraido diretamente do PDF, preservado como texto original.</t>
+          <t>Unidade de medida do LD, quando informada no campo ld.</t>
         </is>
       </c>
     </row>
@@ -4964,12 +4964,12 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>lq_minimo</t>
+          <t>lq</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J22" t="b">
@@ -4977,12 +4977,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.lq_col</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Valor minimo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
+          <t>LQ extraido diretamente do PDF, preservado como texto original.</t>
         </is>
       </c>
     </row>
@@ -5018,7 +5018,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>lq_maximo</t>
+          <t>lq_minimo</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -5036,7 +5036,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Valor maximo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
+          <t>Valor minimo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
         </is>
       </c>
     </row>
@@ -5072,12 +5072,12 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>lq_unidade</t>
+          <t>lq_maximo</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J24" t="b">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Unidade de medida do LQ, quando informada no campo lq.</t>
+          <t>Valor maximo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>referencia</t>
+          <t>lq_unidade</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -5144,7 +5144,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Coluna referencia da aba results_extract.</t>
+          <t>Unidade de medida do LQ, quando informada no campo lq.</t>
         </is>
       </c>
     </row>
@@ -5180,7 +5180,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>incerteza</t>
+          <t>referencia</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -5193,12 +5193,12 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>table_extraction_rules.incerteza_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Incerteza extraida diretamente do PDF, preservada como texto original.</t>
+          <t>Coluna referencia da aba results_extract.</t>
         </is>
       </c>
     </row>
@@ -5234,12 +5234,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>incerteza_valor</t>
+          <t>incerteza</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J27" t="b">
@@ -5247,12 +5247,12 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.incerteza_col</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Valor da incerteza gravado como numero no Excel, com casas decimais preservadas conforme o campo incerteza.</t>
+          <t>Incerteza extraida diretamente do PDF, preservada como texto original.</t>
         </is>
       </c>
     </row>
@@ -5288,12 +5288,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>incerteza_unidade</t>
+          <t>incerteza_valor</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J28" t="b">
@@ -5306,7 +5306,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Unidade de medida da incerteza, quando informada no campo incerteza.</t>
+          <t>Valor da incerteza gravado como numero no Excel, com casas decimais preservadas conforme o campo incerteza.</t>
         </is>
       </c>
     </row>
@@ -5342,7 +5342,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>numero_cq</t>
+          <t>incerteza_unidade</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -5360,7 +5360,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Coluna numero_cq da aba results_extract.</t>
+          <t>Unidade de medida da incerteza, quando informada no campo incerteza.</t>
         </is>
       </c>
     </row>
@@ -5396,12 +5396,12 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>duplicata</t>
+          <t>numero_cq</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>texto_numerico</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J30" t="b">
@@ -5409,12 +5409,12 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>table_extraction_rules.duplicata_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Valor de duplicata extraido diretamente do PDF; validado como texto numerico.</t>
+          <t>Coluna numero_cq da aba results_extract.</t>
         </is>
       </c>
     </row>
@@ -5450,12 +5450,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>faixa_aceitacao</t>
+          <t>duplicata</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>texto_numerico</t>
         </is>
       </c>
       <c r="J31" t="b">
@@ -5463,12 +5463,12 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>table_extraction_rules.faixa_aceitacao_col</t>
+          <t>table_extraction_rules.duplicata_col</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Faixa de aceitacao extraida diretamente do PDF, preservada como texto original.</t>
+          <t>Valor de duplicata extraido diretamente do PDF; validado como texto numerico.</t>
         </is>
       </c>
     </row>
@@ -5504,7 +5504,7 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_operador</t>
+          <t>faixa_aceitacao</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
@@ -5517,12 +5517,12 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.faixa_aceitacao_col</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Operador extraido da faixa de aceitacao, quando informado no PDF.</t>
+          <t>Faixa de aceitacao extraida diretamente do PDF, preservada como texto original.</t>
         </is>
       </c>
     </row>
@@ -5558,12 +5558,12 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_minimo</t>
+          <t>faixa_aceitacao_operador</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J33" t="b">
@@ -5576,7 +5576,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Valor minimo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
+          <t>Operador extraido da faixa de aceitacao, quando informado no PDF.</t>
         </is>
       </c>
     </row>
@@ -5612,7 +5612,7 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_maximo</t>
+          <t>faixa_aceitacao_minimo</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
@@ -5630,7 +5630,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Valor maximo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
+          <t>Valor minimo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -5666,12 +5666,12 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_unidade</t>
+          <t>faixa_aceitacao_maximo</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J35" t="b">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Unidade de medida da faixa de aceitacao, quando informada no campo faixa_aceitacao.</t>
+          <t>Valor maximo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -5720,12 +5720,12 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>variacao_percentual</t>
+          <t>faixa_aceitacao_unidade</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J36" t="b">
@@ -5733,12 +5733,12 @@
       </c>
       <c r="K36" t="inlineStr">
         <is>
-          <t>table_extraction_rules.variacao_percentual_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
+          <t>Unidade de medida da faixa de aceitacao, quando informada no campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -5774,7 +5774,7 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>quantidade_adicionada</t>
+          <t>variacao_percentual</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
@@ -5787,12 +5787,12 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>table_extraction_rules.quantidade_adicionada_col</t>
+          <t>table_extraction_rules.variacao_percentual_col</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
     </row>
@@ -5828,7 +5828,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>recuperacao_percentual</t>
+          <t>quantidade_adicionada</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -5841,12 +5841,12 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>table_extraction_rules.recuperacao_percentual_col</t>
+          <t>table_extraction_rules.quantidade_adicionada_col</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
     </row>
@@ -5863,31 +5863,31 @@
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E39" t="b">
         <v>1</v>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
       <c r="G39" t="n">
-        <v>1</v>
+        <v>38</v>
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>nome_do_arquivo</t>
+          <t>recuperacao_percentual</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J39" t="b">
@@ -5895,12 +5895,12 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>arquivo_pdf</t>
+          <t>table_extraction_rules.recuperacao_percentual_col</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Nome do arquivo PDF de origem do registro.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
     </row>
@@ -5932,11 +5932,11 @@
         </is>
       </c>
       <c r="G40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>template_id</t>
+          <t>nome_do_arquivo</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -5949,12 +5949,12 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>document_scope</t>
+          <t>arquivo_pdf</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
+          <t>Nome do arquivo PDF de origem do registro.</t>
         </is>
       </c>
     </row>
@@ -5986,11 +5986,11 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>tipo_laudo</t>
+          <t>template_id</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -6003,12 +6003,12 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>templates.theme_id</t>
+          <t>document_scope</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
+          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
         </is>
       </c>
     </row>
@@ -6040,16 +6040,16 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>id_amostra</t>
+          <t>tipo_laudo</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>inteiro_ou_texto</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J42" t="b">
@@ -6057,12 +6057,12 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>text_extraction_rules.metadata.id_amostra</t>
+          <t>templates.theme_id</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Coluna id_amostra da aba sample.</t>
+          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
         </is>
       </c>
     </row>
@@ -6094,16 +6094,16 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>tipo_amostra</t>
+          <t>id_amostra</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>inteiro_ou_texto</t>
         </is>
       </c>
       <c r="J43" t="b">
@@ -6111,12 +6111,12 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>text_extraction_rules.metadata.id_amostra</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Coluna tipo_amostra da aba sample.</t>
+          <t>Coluna id_amostra da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6148,11 +6148,11 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>criterio_conformidade</t>
+          <t>tipo_amostra</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Coluna criterio_conformidade da aba sample.</t>
+          <t>Coluna tipo_amostra da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6202,16 +6202,16 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>data_coleta</t>
+          <t>criterio_conformidade</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J45" t="b">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Coluna data_coleta da aba sample.</t>
+          <t>Coluna criterio_conformidade da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6256,16 +6256,16 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>dh_coleta</t>
+          <t>data_coleta</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>data</t>
         </is>
       </c>
       <c r="J46" t="b">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Coluna dh_coleta da aba sample.</t>
+          <t>Coluna data_coleta da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6310,16 +6310,16 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>data_publicacao</t>
+          <t>dh_coleta</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="J47" t="b">
@@ -6332,7 +6332,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Coluna data_publicacao da aba sample.</t>
+          <t>Coluna dh_coleta da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6364,16 +6364,16 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>dh_publicacao</t>
+          <t>data_publicacao</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>data</t>
         </is>
       </c>
       <c r="J48" t="b">
@@ -6386,7 +6386,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Coluna dh_publicacao da aba sample.</t>
+          <t>Coluna data_publicacao da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6418,16 +6418,16 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>data_recebimento</t>
+          <t>dh_publicacao</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="J49" t="b">
@@ -6440,7 +6440,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Coluna data_recebimento da aba sample.</t>
+          <t>Coluna dh_publicacao da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6472,16 +6472,16 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>dh_recebimento</t>
+          <t>data_recebimento</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>data</t>
         </is>
       </c>
       <c r="J50" t="b">
@@ -6494,7 +6494,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Coluna dh_recebimento da aba sample.</t>
+          <t>Coluna data_recebimento da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6526,16 +6526,16 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>observacoes</t>
+          <t>dh_recebimento</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="J51" t="b">
@@ -6548,7 +6548,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Coluna observacoes da aba sample.</t>
+          <t>Coluna dh_recebimento da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6580,16 +6580,16 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>dh_inicio_atividade</t>
+          <t>observacoes</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>data_ou_data_hora</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J52" t="b">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Coluna dh_inicio_atividade da aba sample.</t>
+          <t>Coluna observacoes da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6634,16 +6634,16 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>localizacao</t>
+          <t>dh_inicio_atividade</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>data_ou_data_hora</t>
         </is>
       </c>
       <c r="J53" t="b">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Coluna localizacao da aba sample.</t>
+          <t>Coluna dh_inicio_atividade da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6688,16 +6688,16 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>latitude</t>
+          <t>localizacao</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J54" t="b">
@@ -6710,7 +6710,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Coluna latitude da aba sample.</t>
+          <t>Coluna localizacao da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6742,11 +6742,11 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>longitude</t>
+          <t>latitude</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Coluna longitude da aba sample.</t>
+          <t>Coluna latitude da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6796,16 +6796,16 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>coordenadas</t>
+          <t>longitude</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J56" t="b">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Coluna coordenadas da aba sample.</t>
+          <t>Coluna longitude da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6850,11 +6850,11 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>clima_ultimas_24h</t>
+          <t>coordenadas</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
@@ -6872,7 +6872,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Coluna clima_ultimas_24h da aba sample.</t>
+          <t>Coluna coordenadas da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6904,11 +6904,11 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>clima</t>
+          <t>clima_ultimas_24h</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -6926,7 +6926,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Coluna clima da aba sample.</t>
+          <t>Coluna clima_ultimas_24h da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6958,11 +6958,11 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>tipo_coleta</t>
+          <t>clima</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -6980,7 +6980,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Coluna tipo_coleta da aba sample.</t>
+          <t>Coluna clima da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7012,11 +7012,11 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>responsavel_amostra</t>
+          <t>tipo_coleta</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Coluna responsavel_amostra da aba sample.</t>
+          <t>Coluna tipo_coleta da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7066,11 +7066,11 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>planejamento_amostragem</t>
+          <t>responsavel_amostra</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -7088,7 +7088,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Coluna planejamento_amostragem da aba sample.</t>
+          <t>Coluna responsavel_amostra da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7120,11 +7120,11 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>descricao_nao_conformidade</t>
+          <t>planejamento_amostragem</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -7142,7 +7142,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Coluna descricao_nao_conformidade da aba sample.</t>
+          <t>Coluna planejamento_amostragem da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7159,26 +7159,26 @@
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E63" t="b">
         <v>1</v>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
       <c r="G63" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>nome_do_arquivo</t>
+          <t>descricao_nao_conformidade</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -7191,12 +7191,12 @@
       </c>
       <c r="K63" t="inlineStr">
         <is>
-          <t>arquivo_pdf</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Nome do arquivo PDF de origem do registro.</t>
+          <t>Coluna descricao_nao_conformidade da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7228,11 +7228,11 @@
         </is>
       </c>
       <c r="G64" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>template_id</t>
+          <t>nome_do_arquivo</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -7245,12 +7245,12 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>document_scope</t>
+          <t>arquivo_pdf</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
+          <t>Nome do arquivo PDF de origem do registro.</t>
         </is>
       </c>
     </row>
@@ -7282,11 +7282,11 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>tipo_laudo</t>
+          <t>template_id</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -7299,12 +7299,12 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>templates.theme_id</t>
+          <t>document_scope</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
+          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
         </is>
       </c>
     </row>
@@ -7336,16 +7336,16 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>id_amostra</t>
+          <t>tipo_laudo</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
         <is>
-          <t>inteiro_ou_texto</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J66" t="b">
@@ -7353,12 +7353,12 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>text_extraction_rules.metadata.id_amostra</t>
+          <t>templates.theme_id</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Coluna id_amostra da aba client.</t>
+          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
         </is>
       </c>
     </row>
@@ -7390,16 +7390,16 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>proposta_comercial</t>
+          <t>id_amostra</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>inteiro_ou_texto</t>
         </is>
       </c>
       <c r="J67" t="b">
@@ -7407,12 +7407,12 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>text_extraction_rules.metadata.id_amostra</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Coluna proposta_comercial da aba client.</t>
+          <t>Coluna id_amostra da aba client.</t>
         </is>
       </c>
     </row>
@@ -7444,11 +7444,11 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>cliente</t>
+          <t>proposta_comercial</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -7466,7 +7466,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Coluna cliente da aba client.</t>
+          <t>Coluna proposta_comercial da aba client.</t>
         </is>
       </c>
     </row>
@@ -7498,11 +7498,11 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>cnpj_cpf</t>
+          <t>cliente</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Coluna cnpj_cpf da aba client.</t>
+          <t>Coluna cliente da aba client.</t>
         </is>
       </c>
     </row>
@@ -7552,11 +7552,11 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>contato</t>
+          <t>cnpj_cpf</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -7574,7 +7574,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>Coluna contato da aba client.</t>
+          <t>Coluna cnpj_cpf da aba client.</t>
         </is>
       </c>
     </row>
@@ -7606,11 +7606,11 @@
         </is>
       </c>
       <c r="G71" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>telefone</t>
+          <t>contato</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -7628,7 +7628,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>Coluna telefone da aba client.</t>
+          <t>Coluna contato da aba client.</t>
         </is>
       </c>
     </row>
@@ -7660,11 +7660,11 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>endereco</t>
+          <t>telefone</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -7682,7 +7682,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Coluna endereco da aba client.</t>
+          <t>Coluna telefone da aba client.</t>
         </is>
       </c>
     </row>
@@ -7699,26 +7699,44 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>table_extraction_audit</t>
+          <t>client</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>97</v>
+        <v>3</v>
       </c>
       <c r="E73" t="b">
         <v>1</v>
       </c>
       <c r="F73" t="inlineStr">
         <is>
-          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+      <c r="G73" t="n">
+        <v>10</v>
+      </c>
+      <c r="H73" t="inlineStr">
+        <is>
+          <t>endereco</t>
+        </is>
+      </c>
+      <c r="I73" t="inlineStr">
+        <is>
+          <t>texto</t>
         </is>
       </c>
       <c r="J73" t="b">
         <v>0</v>
       </c>
+      <c r="K73" t="inlineStr">
+        <is>
+          <t>parser</t>
+        </is>
+      </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Aba de auditoria das tabelas processadas, incluindo colunas detectadas, campos esperados e status da leitura.</t>
+          <t>Coluna endereco da aba client.</t>
         </is>
       </c>
     </row>
@@ -7735,18 +7753,18 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>table_extraction_audit</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E74" t="b">
         <v>1</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
       <c r="J74" t="b">
@@ -7754,7 +7772,7 @@
       </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>Aba de auditoria da classificacao do template, incluindo regras encontradas, score e status por candidato.</t>
+          <t>Aba de auditoria das tabelas processadas, incluindo colunas detectadas, campos esperados e status da leitura.</t>
         </is>
       </c>
     </row>
@@ -7771,31 +7789,67 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>98</v>
+      </c>
+      <c r="E75" t="b">
+        <v>1</v>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+      <c r="J75" t="b">
+        <v>0</v>
+      </c>
+      <c r="L75" t="inlineStr">
+        <is>
+          <t>Aba de auditoria da classificacao do template, incluindo regras encontradas, score e status por candidato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>laudo_agua</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
           <t>validation_errors</t>
         </is>
       </c>
-      <c r="D75" t="n">
+      <c r="D76" t="n">
         <v>99</v>
       </c>
-      <c r="E75" t="b">
-        <v>1</v>
-      </c>
-      <c r="F75" t="inlineStr">
+      <c r="E76" t="b">
+        <v>1</v>
+      </c>
+      <c r="F76" t="inlineStr">
         <is>
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="J75" t="b">
-        <v>0</v>
-      </c>
-      <c r="L75" t="inlineStr">
+      <c r="J76" t="b">
+        <v>0</v>
+      </c>
+      <c r="L76" t="inlineStr">
         <is>
           <t>Aba de erros de validacao final, preenchida quando algum campo nao atende ao contrato esperado.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L75"/>
+  <autoFilter ref="A1:L76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Map normative columns to explicit output fields
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_consolidada_v1.xlsx
+++ b/config/taxonomy_config_consolidada_v1.xlsx
@@ -20,9 +20,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README_FORMATO'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'templates'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'template_rules'!$A$1:$G$78</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'output_model'!$A$1:$L$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'output_model'!$A$1:$L$77</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'text_extraction_rules'!$A$1:$G$85</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'table_extraction_rules'!$A$1:$I$40</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'table_extraction_rules'!$A$1:$I$42</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'section_rules'!$A$1:$L$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'continuation_rules'!$A$1:$E$4</definedName>
   </definedNames>
@@ -3773,7 +3773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4640,7 +4640,7 @@
       </c>
       <c r="H16" t="inlineStr">
         <is>
-          <t>referencia_normativa</t>
+          <t>conama</t>
         </is>
       </c>
       <c r="I16" t="inlineStr">
@@ -4653,12 +4653,12 @@
       </c>
       <c r="K16" t="inlineStr">
         <is>
-          <t>cabecalho_detectado.criterio_conformidade_col</t>
+          <t>table_extraction_rules.conama_col</t>
         </is>
       </c>
       <c r="L16" t="inlineStr">
         <is>
-          <t>Nome da referencia normativa detectada no cabecalho da coluna de criterio, como CONAMA, COPAM/CERH ou deliberacao normativa.</t>
+          <t>Valor extraido da coluna normativa CONAMA, quando esse cabecalho existir na tabela.</t>
         </is>
       </c>
     </row>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>criterio_conformidade</t>
+          <t>copam_cerh</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -4707,12 +4707,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>table_extraction_rules.criterio_conformidade_col</t>
+          <t>table_extraction_rules.copam_cerh_col</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Valor do criterio de conformidade extraido da celula da tabela.</t>
+          <t>Valor extraido da coluna normativa COPAM/CERH, quando esse cabecalho existir na tabela.</t>
         </is>
       </c>
     </row>
@@ -4748,7 +4748,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>ld</t>
+          <t>criterio_conformidade</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -4761,12 +4761,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>table_extraction_rules.ld_col</t>
+          <t>table_extraction_rules.criterio_conformidade_col</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>LD extraido diretamente do PDF, preservado como texto original.</t>
+          <t>Valor extraido de uma coluna generica de criterio de conformidade, quando o cabecalho nao for CONAMA nem COPAM/CERH.</t>
         </is>
       </c>
     </row>
@@ -4802,12 +4802,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ld_minimo</t>
+          <t>ld</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J19" t="b">
@@ -4815,12 +4815,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.ld_col</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Valor minimo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
+          <t>LD extraido diretamente do PDF, preservado como texto original.</t>
         </is>
       </c>
     </row>
@@ -4856,7 +4856,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>ld_maximo</t>
+          <t>ld_minimo</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Valor maximo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
+          <t>Valor minimo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
         </is>
       </c>
     </row>
@@ -4910,12 +4910,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>ld_unidade</t>
+          <t>ld_maximo</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J21" t="b">
@@ -4928,7 +4928,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Unidade de medida do LD, quando informada no campo ld.</t>
+          <t>Valor maximo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
         </is>
       </c>
     </row>
@@ -4964,7 +4964,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>lq</t>
+          <t>ld_unidade</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -4977,12 +4977,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>table_extraction_rules.lq_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>LQ extraido diretamente do PDF, preservado como texto original.</t>
+          <t>Unidade de medida do LD, quando informada no campo ld.</t>
         </is>
       </c>
     </row>
@@ -5018,12 +5018,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>lq_minimo</t>
+          <t>lq</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J23" t="b">
@@ -5031,12 +5031,12 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.lq_col</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Valor minimo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
+          <t>LQ extraido diretamente do PDF, preservado como texto original.</t>
         </is>
       </c>
     </row>
@@ -5072,7 +5072,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>lq_maximo</t>
+          <t>lq_minimo</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Valor maximo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
+          <t>Valor minimo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
         </is>
       </c>
     </row>
@@ -5126,12 +5126,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>lq_unidade</t>
+          <t>lq_maximo</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J25" t="b">
@@ -5144,7 +5144,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Unidade de medida do LQ, quando informada no campo lq.</t>
+          <t>Valor maximo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
         </is>
       </c>
     </row>
@@ -5180,7 +5180,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>referencia</t>
+          <t>lq_unidade</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -5198,7 +5198,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Coluna referencia da aba results_extract.</t>
+          <t>Unidade de medida do LQ, quando informada no campo lq.</t>
         </is>
       </c>
     </row>
@@ -5234,7 +5234,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>incerteza</t>
+          <t>referencia</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -5247,12 +5247,12 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>table_extraction_rules.incerteza_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Incerteza extraida diretamente do PDF, preservada como texto original.</t>
+          <t>Coluna referencia da aba results_extract.</t>
         </is>
       </c>
     </row>
@@ -5288,12 +5288,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>incerteza_valor</t>
+          <t>incerteza</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J28" t="b">
@@ -5301,12 +5301,12 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.incerteza_col</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Valor da incerteza gravado como numero no Excel, com casas decimais preservadas conforme o campo incerteza.</t>
+          <t>Incerteza extraida diretamente do PDF, preservada como texto original.</t>
         </is>
       </c>
     </row>
@@ -5342,12 +5342,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>incerteza_unidade</t>
+          <t>incerteza_valor</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J29" t="b">
@@ -5360,7 +5360,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Unidade de medida da incerteza, quando informada no campo incerteza.</t>
+          <t>Valor da incerteza gravado como numero no Excel, com casas decimais preservadas conforme o campo incerteza.</t>
         </is>
       </c>
     </row>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>numero_cq</t>
+          <t>incerteza_unidade</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Coluna numero_cq da aba results_extract.</t>
+          <t>Unidade de medida da incerteza, quando informada no campo incerteza.</t>
         </is>
       </c>
     </row>
@@ -5450,12 +5450,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>duplicata</t>
+          <t>numero_cq</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>texto_numerico</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J31" t="b">
@@ -5463,12 +5463,12 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>table_extraction_rules.duplicata_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Valor de duplicata extraido diretamente do PDF; validado como texto numerico.</t>
+          <t>Coluna numero_cq da aba results_extract.</t>
         </is>
       </c>
     </row>
@@ -5504,12 +5504,12 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>faixa_aceitacao</t>
+          <t>duplicata</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>texto_numerico</t>
         </is>
       </c>
       <c r="J32" t="b">
@@ -5517,12 +5517,12 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>table_extraction_rules.faixa_aceitacao_col</t>
+          <t>table_extraction_rules.duplicata_col</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Faixa de aceitacao extraida diretamente do PDF, preservada como texto original.</t>
+          <t>Valor de duplicata extraido diretamente do PDF; validado como texto numerico.</t>
         </is>
       </c>
     </row>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_operador</t>
+          <t>faixa_aceitacao</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -5571,12 +5571,12 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.faixa_aceitacao_col</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Operador extraido da faixa de aceitacao, quando informado no PDF.</t>
+          <t>Faixa de aceitacao extraida diretamente do PDF, preservada como texto original.</t>
         </is>
       </c>
     </row>
@@ -5612,12 +5612,12 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_minimo</t>
+          <t>faixa_aceitacao_operador</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J34" t="b">
@@ -5630,7 +5630,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Valor minimo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
+          <t>Operador extraido da faixa de aceitacao, quando informado no PDF.</t>
         </is>
       </c>
     </row>
@@ -5666,7 +5666,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_maximo</t>
+          <t>faixa_aceitacao_minimo</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Valor maximo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
+          <t>Valor minimo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -5720,12 +5720,12 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_unidade</t>
+          <t>faixa_aceitacao_maximo</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J36" t="b">
@@ -5738,7 +5738,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Unidade de medida da faixa de aceitacao, quando informada no campo faixa_aceitacao.</t>
+          <t>Valor maximo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -5774,12 +5774,12 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>variacao_percentual</t>
+          <t>faixa_aceitacao_unidade</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J37" t="b">
@@ -5787,12 +5787,12 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>table_extraction_rules.variacao_percentual_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
+          <t>Unidade de medida da faixa de aceitacao, quando informada no campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -5828,7 +5828,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>quantidade_adicionada</t>
+          <t>variacao_percentual</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -5841,12 +5841,12 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>table_extraction_rules.quantidade_adicionada_col</t>
+          <t>table_extraction_rules.variacao_percentual_col</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
     </row>
@@ -5882,7 +5882,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>recuperacao_percentual</t>
+          <t>quantidade_adicionada</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -5895,12 +5895,12 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>table_extraction_rules.recuperacao_percentual_col</t>
+          <t>table_extraction_rules.quantidade_adicionada_col</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
     </row>
@@ -5917,31 +5917,31 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E40" t="b">
         <v>1</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>nome_do_arquivo</t>
+          <t>recuperacao_percentual</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J40" t="b">
@@ -5949,12 +5949,12 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>arquivo_pdf</t>
+          <t>table_extraction_rules.recuperacao_percentual_col</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Nome do arquivo PDF de origem do registro.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
     </row>
@@ -5986,11 +5986,11 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>template_id</t>
+          <t>nome_do_arquivo</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -6003,12 +6003,12 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>document_scope</t>
+          <t>arquivo_pdf</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
+          <t>Nome do arquivo PDF de origem do registro.</t>
         </is>
       </c>
     </row>
@@ -6040,11 +6040,11 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>tipo_laudo</t>
+          <t>template_id</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -6057,12 +6057,12 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>templates.theme_id</t>
+          <t>document_scope</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
+          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
         </is>
       </c>
     </row>
@@ -6094,16 +6094,16 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>id_amostra</t>
+          <t>tipo_laudo</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>inteiro_ou_texto</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J43" t="b">
@@ -6111,12 +6111,12 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>text_extraction_rules.metadata.id_amostra</t>
+          <t>templates.theme_id</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Coluna id_amostra da aba sample.</t>
+          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
         </is>
       </c>
     </row>
@@ -6148,16 +6148,16 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>tipo_amostra</t>
+          <t>id_amostra</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>inteiro_ou_texto</t>
         </is>
       </c>
       <c r="J44" t="b">
@@ -6165,12 +6165,12 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>text_extraction_rules.metadata.id_amostra</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Coluna tipo_amostra da aba sample.</t>
+          <t>Coluna id_amostra da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6202,11 +6202,11 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>criterio_conformidade</t>
+          <t>tipo_amostra</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Coluna criterio_conformidade da aba sample.</t>
+          <t>Coluna tipo_amostra da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6256,16 +6256,16 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>data_coleta</t>
+          <t>criterio_conformidade</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J46" t="b">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Coluna data_coleta da aba sample.</t>
+          <t>Coluna criterio_conformidade da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6310,16 +6310,16 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>dh_coleta</t>
+          <t>data_coleta</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>data</t>
         </is>
       </c>
       <c r="J47" t="b">
@@ -6332,7 +6332,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Coluna dh_coleta da aba sample.</t>
+          <t>Coluna data_coleta da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6364,16 +6364,16 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>data_publicacao</t>
+          <t>dh_coleta</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="J48" t="b">
@@ -6386,7 +6386,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Coluna data_publicacao da aba sample.</t>
+          <t>Coluna dh_coleta da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6418,16 +6418,16 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>dh_publicacao</t>
+          <t>data_publicacao</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>data</t>
         </is>
       </c>
       <c r="J49" t="b">
@@ -6440,7 +6440,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Coluna dh_publicacao da aba sample.</t>
+          <t>Coluna data_publicacao da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6472,16 +6472,16 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>data_recebimento</t>
+          <t>dh_publicacao</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="J50" t="b">
@@ -6494,7 +6494,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Coluna data_recebimento da aba sample.</t>
+          <t>Coluna dh_publicacao da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6526,16 +6526,16 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>dh_recebimento</t>
+          <t>data_recebimento</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>data</t>
         </is>
       </c>
       <c r="J51" t="b">
@@ -6548,7 +6548,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Coluna dh_recebimento da aba sample.</t>
+          <t>Coluna data_recebimento da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6580,16 +6580,16 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>observacoes</t>
+          <t>dh_recebimento</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="J52" t="b">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Coluna observacoes da aba sample.</t>
+          <t>Coluna dh_recebimento da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6634,16 +6634,16 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>14</v>
+        <v>13</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>dh_inicio_atividade</t>
+          <t>observacoes</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>data_ou_data_hora</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J53" t="b">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Coluna dh_inicio_atividade da aba sample.</t>
+          <t>Coluna observacoes da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6688,16 +6688,16 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>15</v>
+        <v>14</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>localizacao</t>
+          <t>dh_inicio_atividade</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>data_ou_data_hora</t>
         </is>
       </c>
       <c r="J54" t="b">
@@ -6710,7 +6710,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Coluna localizacao da aba sample.</t>
+          <t>Coluna dh_inicio_atividade da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6742,16 +6742,16 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>16</v>
+        <v>15</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>latitude</t>
+          <t>localizacao</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J55" t="b">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Coluna latitude da aba sample.</t>
+          <t>Coluna localizacao da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6796,11 +6796,11 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>longitude</t>
+          <t>latitude</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Coluna longitude da aba sample.</t>
+          <t>Coluna latitude da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6850,16 +6850,16 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>18</v>
+        <v>17</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>coordenadas</t>
+          <t>longitude</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J57" t="b">
@@ -6872,7 +6872,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Coluna coordenadas da aba sample.</t>
+          <t>Coluna longitude da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6904,11 +6904,11 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>clima_ultimas_24h</t>
+          <t>coordenadas</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -6926,7 +6926,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Coluna clima_ultimas_24h da aba sample.</t>
+          <t>Coluna coordenadas da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6958,11 +6958,11 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>clima</t>
+          <t>clima_ultimas_24h</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -6980,7 +6980,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Coluna clima da aba sample.</t>
+          <t>Coluna clima_ultimas_24h da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7012,11 +7012,11 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>tipo_coleta</t>
+          <t>clima</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Coluna tipo_coleta da aba sample.</t>
+          <t>Coluna clima da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7066,11 +7066,11 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>responsavel_amostra</t>
+          <t>tipo_coleta</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -7088,7 +7088,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Coluna responsavel_amostra da aba sample.</t>
+          <t>Coluna tipo_coleta da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7120,11 +7120,11 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>planejamento_amostragem</t>
+          <t>responsavel_amostra</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -7142,7 +7142,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Coluna planejamento_amostragem da aba sample.</t>
+          <t>Coluna responsavel_amostra da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7174,11 +7174,11 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>descricao_nao_conformidade</t>
+          <t>planejamento_amostragem</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -7196,7 +7196,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Coluna descricao_nao_conformidade da aba sample.</t>
+          <t>Coluna planejamento_amostragem da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7213,26 +7213,26 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E64" t="b">
         <v>1</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
       <c r="G64" t="n">
-        <v>1</v>
+        <v>24</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>nome_do_arquivo</t>
+          <t>descricao_nao_conformidade</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -7245,12 +7245,12 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>arquivo_pdf</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Nome do arquivo PDF de origem do registro.</t>
+          <t>Coluna descricao_nao_conformidade da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7282,11 +7282,11 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>template_id</t>
+          <t>nome_do_arquivo</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -7299,12 +7299,12 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>document_scope</t>
+          <t>arquivo_pdf</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
+          <t>Nome do arquivo PDF de origem do registro.</t>
         </is>
       </c>
     </row>
@@ -7336,11 +7336,11 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>tipo_laudo</t>
+          <t>template_id</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -7353,12 +7353,12 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>templates.theme_id</t>
+          <t>document_scope</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
+          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
         </is>
       </c>
     </row>
@@ -7390,16 +7390,16 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>id_amostra</t>
+          <t>tipo_laudo</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>inteiro_ou_texto</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J67" t="b">
@@ -7407,12 +7407,12 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>text_extraction_rules.metadata.id_amostra</t>
+          <t>templates.theme_id</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Coluna id_amostra da aba client.</t>
+          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
         </is>
       </c>
     </row>
@@ -7444,16 +7444,16 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>proposta_comercial</t>
+          <t>id_amostra</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>inteiro_ou_texto</t>
         </is>
       </c>
       <c r="J68" t="b">
@@ -7461,12 +7461,12 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>text_extraction_rules.metadata.id_amostra</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Coluna proposta_comercial da aba client.</t>
+          <t>Coluna id_amostra da aba client.</t>
         </is>
       </c>
     </row>
@@ -7498,11 +7498,11 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>cliente</t>
+          <t>proposta_comercial</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Coluna cliente da aba client.</t>
+          <t>Coluna proposta_comercial da aba client.</t>
         </is>
       </c>
     </row>
@@ -7552,11 +7552,11 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>cnpj_cpf</t>
+          <t>cliente</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -7574,7 +7574,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>Coluna cnpj_cpf da aba client.</t>
+          <t>Coluna cliente da aba client.</t>
         </is>
       </c>
     </row>
@@ -7606,11 +7606,11 @@
         </is>
       </c>
       <c r="G71" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>contato</t>
+          <t>cnpj_cpf</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -7628,7 +7628,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>Coluna contato da aba client.</t>
+          <t>Coluna cnpj_cpf da aba client.</t>
         </is>
       </c>
     </row>
@@ -7660,11 +7660,11 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>telefone</t>
+          <t>contato</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -7682,7 +7682,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Coluna telefone da aba client.</t>
+          <t>Coluna contato da aba client.</t>
         </is>
       </c>
     </row>
@@ -7714,11 +7714,11 @@
         </is>
       </c>
       <c r="G73" t="n">
-        <v>10</v>
+        <v>9</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>endereco</t>
+          <t>telefone</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -7736,7 +7736,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Coluna endereco da aba client.</t>
+          <t>Coluna telefone da aba client.</t>
         </is>
       </c>
     </row>
@@ -7753,26 +7753,44 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>table_extraction_audit</t>
+          <t>client</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>97</v>
+        <v>3</v>
       </c>
       <c r="E74" t="b">
         <v>1</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>10</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>endereco</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>texto</t>
         </is>
       </c>
       <c r="J74" t="b">
         <v>0</v>
       </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>parser</t>
+        </is>
+      </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>Aba de auditoria das tabelas processadas, incluindo colunas detectadas, campos esperados e status da leitura.</t>
+          <t>Coluna endereco da aba client.</t>
         </is>
       </c>
     </row>
@@ -7789,18 +7807,18 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>table_extraction_audit</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="E75" t="b">
         <v>1</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
       <c r="J75" t="b">
@@ -7808,7 +7826,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Aba de auditoria da classificacao do template, incluindo regras encontradas, score e status por candidato.</t>
+          <t>Aba de auditoria das tabelas processadas, incluindo colunas detectadas, campos esperados e status da leitura.</t>
         </is>
       </c>
     </row>
@@ -7825,31 +7843,67 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>98</v>
+      </c>
+      <c r="E76" t="b">
+        <v>1</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+      <c r="J76" t="b">
+        <v>0</v>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Aba de auditoria da classificacao do template, incluindo regras encontradas, score e status por candidato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>laudo_agua</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
           <t>validation_errors</t>
         </is>
       </c>
-      <c r="D76" t="n">
+      <c r="D77" t="n">
         <v>99</v>
       </c>
-      <c r="E76" t="b">
-        <v>1</v>
-      </c>
-      <c r="F76" t="inlineStr">
+      <c r="E77" t="b">
+        <v>1</v>
+      </c>
+      <c r="F77" t="inlineStr">
         <is>
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="J76" t="b">
-        <v>0</v>
-      </c>
-      <c r="L76" t="inlineStr">
+      <c r="J77" t="b">
+        <v>0</v>
+      </c>
+      <c r="L77" t="inlineStr">
         <is>
           <t>Aba de erros de validacao final, preenchida quando algum campo nao atende ao contrato esperado.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L76"/>
+  <autoFilter ref="A1:L77"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10861,7 +10915,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I40"/>
+  <dimension ref="A1:I42"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -10870,7 +10924,7 @@
     <col width="15" customWidth="1" min="4" max="4"/>
     <col width="24" customWidth="1" min="5" max="5"/>
     <col width="15" customWidth="1" min="6" max="6"/>
-    <col width="60" customWidth="1" min="7" max="7"/>
+    <col width="44" customWidth="1" min="7" max="7"/>
     <col width="12" customWidth="1" min="8" max="8"/>
     <col width="60" customWidth="1" min="9" max="9"/>
   </cols>
@@ -12607,30 +12661,120 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
+          <t>conama</t>
+        </is>
+      </c>
+      <c r="F40" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G40" t="inlineStr">
+        <is>
+          <t>conama</t>
+        </is>
+      </c>
+      <c r="H40" t="b">
+        <v>1</v>
+      </c>
+      <c r="I40" t="inlineStr">
+        <is>
+          <t>Reconhece colunas normativas CONAMA; o valor da linha sai no campo conama.</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>copam_cerh</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>copam|cerh|deliberacao\s+normativa</t>
+        </is>
+      </c>
+      <c r="H41" t="b">
+        <v>1</v>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Reconhece colunas normativas COPAM/CERH; o valor da linha sai no campo copam_cerh.</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="inlineStr">
+        <is>
+          <t>header_alias</t>
+        </is>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>results_extract</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
           <t>criterio_conformidade</t>
         </is>
       </c>
-      <c r="F40" t="inlineStr">
-        <is>
-          <t>NAO_APLICAVEL</t>
-        </is>
-      </c>
-      <c r="G40" t="inlineStr">
-        <is>
-          <t>resolucao|conama|criterio|deliberacao\s+normativa|copam|cerh</t>
-        </is>
-      </c>
-      <c r="H40" t="b">
-        <v>1</v>
-      </c>
-      <c r="I40" t="inlineStr">
-        <is>
-          <t>Reconhece colunas normativas como criterio de conformidade, incluindo CONAMA e COPAM/CERH.</t>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>criterio</t>
+        </is>
+      </c>
+      <c r="H42" t="b">
+        <v>1</v>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Reconhece colunas genericas de criterio de conformidade quando nao forem CONAMA ou COPAM/CERH.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:I40"/>
+  <autoFilter ref="A1:I42"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Remove generic conformity field from results
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_consolidada_v1.xlsx
+++ b/config/taxonomy_config_consolidada_v1.xlsx
@@ -20,9 +20,9 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README_FORMATO'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'templates'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'template_rules'!$A$1:$G$78</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'output_model'!$A$1:$L$77</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'output_model'!$A$1:$L$76</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'text_extraction_rules'!$A$1:$G$85</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'table_extraction_rules'!$A$1:$I$42</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'table_extraction_rules'!$A$1:$I$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'section_rules'!$A$1:$L$54</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'continuation_rules'!$A$1:$E$4</definedName>
   </definedNames>
@@ -3773,7 +3773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L77"/>
+  <dimension ref="A1:L76"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4748,7 +4748,7 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>criterio_conformidade</t>
+          <t>ld</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
@@ -4761,12 +4761,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>table_extraction_rules.criterio_conformidade_col</t>
+          <t>table_extraction_rules.ld_col</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>Valor extraido de uma coluna generica de criterio de conformidade, quando o cabecalho nao for CONAMA nem COPAM/CERH.</t>
+          <t>LD extraido diretamente do PDF, preservado como texto original.</t>
         </is>
       </c>
     </row>
@@ -4802,12 +4802,12 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ld</t>
+          <t>ld_minimo</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J19" t="b">
@@ -4815,12 +4815,12 @@
       </c>
       <c r="K19" t="inlineStr">
         <is>
-          <t>table_extraction_rules.ld_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>LD extraido diretamente do PDF, preservado como texto original.</t>
+          <t>Valor minimo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
         </is>
       </c>
     </row>
@@ -4856,7 +4856,7 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>ld_minimo</t>
+          <t>ld_maximo</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Valor minimo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
+          <t>Valor maximo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
         </is>
       </c>
     </row>
@@ -4910,12 +4910,12 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>ld_maximo</t>
+          <t>ld_unidade</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J21" t="b">
@@ -4928,7 +4928,7 @@
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Valor maximo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
+          <t>Unidade de medida do LD, quando informada no campo ld.</t>
         </is>
       </c>
     </row>
@@ -4964,7 +4964,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>ld_unidade</t>
+          <t>lq</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -4977,12 +4977,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.lq_col</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>Unidade de medida do LD, quando informada no campo ld.</t>
+          <t>LQ extraido diretamente do PDF, preservado como texto original.</t>
         </is>
       </c>
     </row>
@@ -5018,12 +5018,12 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>lq</t>
+          <t>lq_minimo</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J23" t="b">
@@ -5031,12 +5031,12 @@
       </c>
       <c r="K23" t="inlineStr">
         <is>
-          <t>table_extraction_rules.lq_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>LQ extraido diretamente do PDF, preservado como texto original.</t>
+          <t>Valor minimo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
         </is>
       </c>
     </row>
@@ -5072,7 +5072,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>lq_minimo</t>
+          <t>lq_maximo</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Valor minimo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
+          <t>Valor maximo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
         </is>
       </c>
     </row>
@@ -5126,12 +5126,12 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>lq_maximo</t>
+          <t>lq_unidade</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J25" t="b">
@@ -5144,7 +5144,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Valor maximo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
+          <t>Unidade de medida do LQ, quando informada no campo lq.</t>
         </is>
       </c>
     </row>
@@ -5180,7 +5180,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>lq_unidade</t>
+          <t>referencia</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -5198,7 +5198,7 @@
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Unidade de medida do LQ, quando informada no campo lq.</t>
+          <t>Coluna referencia da aba results_extract.</t>
         </is>
       </c>
     </row>
@@ -5234,7 +5234,7 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>referencia</t>
+          <t>incerteza</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
@@ -5247,12 +5247,12 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.incerteza_col</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Coluna referencia da aba results_extract.</t>
+          <t>Incerteza extraida diretamente do PDF, preservada como texto original.</t>
         </is>
       </c>
     </row>
@@ -5288,12 +5288,12 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>incerteza</t>
+          <t>incerteza_valor</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J28" t="b">
@@ -5301,12 +5301,12 @@
       </c>
       <c r="K28" t="inlineStr">
         <is>
-          <t>table_extraction_rules.incerteza_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Incerteza extraida diretamente do PDF, preservada como texto original.</t>
+          <t>Valor da incerteza gravado como numero no Excel, com casas decimais preservadas conforme o campo incerteza.</t>
         </is>
       </c>
     </row>
@@ -5342,12 +5342,12 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>incerteza_valor</t>
+          <t>incerteza_unidade</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J29" t="b">
@@ -5360,7 +5360,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Valor da incerteza gravado como numero no Excel, com casas decimais preservadas conforme o campo incerteza.</t>
+          <t>Unidade de medida da incerteza, quando informada no campo incerteza.</t>
         </is>
       </c>
     </row>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>incerteza_unidade</t>
+          <t>numero_cq</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -5414,7 +5414,7 @@
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Unidade de medida da incerteza, quando informada no campo incerteza.</t>
+          <t>Coluna numero_cq da aba results_extract.</t>
         </is>
       </c>
     </row>
@@ -5450,12 +5450,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>numero_cq</t>
+          <t>duplicata</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>texto_numerico</t>
         </is>
       </c>
       <c r="J31" t="b">
@@ -5463,12 +5463,12 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.duplicata_col</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Coluna numero_cq da aba results_extract.</t>
+          <t>Valor de duplicata extraido diretamente do PDF; validado como texto numerico.</t>
         </is>
       </c>
     </row>
@@ -5504,12 +5504,12 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>duplicata</t>
+          <t>faixa_aceitacao</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>texto_numerico</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J32" t="b">
@@ -5517,12 +5517,12 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>table_extraction_rules.duplicata_col</t>
+          <t>table_extraction_rules.faixa_aceitacao_col</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Valor de duplicata extraido diretamente do PDF; validado como texto numerico.</t>
+          <t>Faixa de aceitacao extraida diretamente do PDF, preservada como texto original.</t>
         </is>
       </c>
     </row>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>faixa_aceitacao</t>
+          <t>faixa_aceitacao_operador</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -5571,12 +5571,12 @@
       </c>
       <c r="K33" t="inlineStr">
         <is>
-          <t>table_extraction_rules.faixa_aceitacao_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Faixa de aceitacao extraida diretamente do PDF, preservada como texto original.</t>
+          <t>Operador extraido da faixa de aceitacao, quando informado no PDF.</t>
         </is>
       </c>
     </row>
@@ -5612,12 +5612,12 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_operador</t>
+          <t>faixa_aceitacao_minimo</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J34" t="b">
@@ -5630,7 +5630,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Operador extraido da faixa de aceitacao, quando informado no PDF.</t>
+          <t>Valor minimo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -5666,7 +5666,7 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_minimo</t>
+          <t>faixa_aceitacao_maximo</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
@@ -5684,7 +5684,7 @@
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Valor minimo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
+          <t>Valor maximo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -5720,12 +5720,12 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_maximo</t>
+          <t>faixa_aceitacao_unidade</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J36" t="b">
@@ -5738,7 +5738,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Valor maximo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
+          <t>Unidade de medida da faixa de aceitacao, quando informada no campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -5774,12 +5774,12 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_unidade</t>
+          <t>variacao_percentual</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J37" t="b">
@@ -5787,12 +5787,12 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.variacao_percentual_col</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Unidade de medida da faixa de aceitacao, quando informada no campo faixa_aceitacao.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
     </row>
@@ -5828,7 +5828,7 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>variacao_percentual</t>
+          <t>quantidade_adicionada</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
@@ -5841,12 +5841,12 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>table_extraction_rules.variacao_percentual_col</t>
+          <t>table_extraction_rules.quantidade_adicionada_col</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
     </row>
@@ -5882,7 +5882,7 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>quantidade_adicionada</t>
+          <t>recuperacao_percentual</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
@@ -5895,12 +5895,12 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>table_extraction_rules.quantidade_adicionada_col</t>
+          <t>table_extraction_rules.recuperacao_percentual_col</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
     </row>
@@ -5917,31 +5917,31 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>results_extract</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E40" t="b">
         <v>1</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Resultados extraidos do PDF para o template.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>39</v>
+        <v>1</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>recuperacao_percentual</t>
+          <t>nome_do_arquivo</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J40" t="b">
@@ -5949,12 +5949,12 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>table_extraction_rules.recuperacao_percentual_col</t>
+          <t>arquivo_pdf</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
+          <t>Nome do arquivo PDF de origem do registro.</t>
         </is>
       </c>
     </row>
@@ -5986,11 +5986,11 @@
         </is>
       </c>
       <c r="G41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>nome_do_arquivo</t>
+          <t>template_id</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -6003,12 +6003,12 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>arquivo_pdf</t>
+          <t>document_scope</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Nome do arquivo PDF de origem do registro.</t>
+          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
         </is>
       </c>
     </row>
@@ -6040,11 +6040,11 @@
         </is>
       </c>
       <c r="G42" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>template_id</t>
+          <t>tipo_laudo</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
@@ -6057,12 +6057,12 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>document_scope</t>
+          <t>templates.theme_id</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
+          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
         </is>
       </c>
     </row>
@@ -6094,16 +6094,16 @@
         </is>
       </c>
       <c r="G43" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>tipo_laudo</t>
+          <t>id_amostra</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>inteiro_ou_texto</t>
         </is>
       </c>
       <c r="J43" t="b">
@@ -6111,12 +6111,12 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>templates.theme_id</t>
+          <t>text_extraction_rules.metadata.id_amostra</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
+          <t>Coluna id_amostra da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6148,16 +6148,16 @@
         </is>
       </c>
       <c r="G44" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>id_amostra</t>
+          <t>tipo_amostra</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
         <is>
-          <t>inteiro_ou_texto</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J44" t="b">
@@ -6165,12 +6165,12 @@
       </c>
       <c r="K44" t="inlineStr">
         <is>
-          <t>text_extraction_rules.metadata.id_amostra</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Coluna id_amostra da aba sample.</t>
+          <t>Coluna tipo_amostra da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6202,11 +6202,11 @@
         </is>
       </c>
       <c r="G45" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>tipo_amostra</t>
+          <t>criterio_conformidade</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
@@ -6224,7 +6224,7 @@
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Coluna tipo_amostra da aba sample.</t>
+          <t>Coluna criterio_conformidade da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6256,16 +6256,16 @@
         </is>
       </c>
       <c r="G46" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>criterio_conformidade</t>
+          <t>data_coleta</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>data</t>
         </is>
       </c>
       <c r="J46" t="b">
@@ -6278,7 +6278,7 @@
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Coluna criterio_conformidade da aba sample.</t>
+          <t>Coluna data_coleta da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6310,16 +6310,16 @@
         </is>
       </c>
       <c r="G47" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>data_coleta</t>
+          <t>dh_coleta</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="J47" t="b">
@@ -6332,7 +6332,7 @@
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Coluna data_coleta da aba sample.</t>
+          <t>Coluna dh_coleta da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6364,16 +6364,16 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>dh_coleta</t>
+          <t>data_publicacao</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>data</t>
         </is>
       </c>
       <c r="J48" t="b">
@@ -6386,7 +6386,7 @@
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Coluna dh_coleta da aba sample.</t>
+          <t>Coluna data_publicacao da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6418,16 +6418,16 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>data_publicacao</t>
+          <t>dh_publicacao</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="J49" t="b">
@@ -6440,7 +6440,7 @@
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Coluna data_publicacao da aba sample.</t>
+          <t>Coluna dh_publicacao da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6472,16 +6472,16 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>dh_publicacao</t>
+          <t>data_recebimento</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>data</t>
         </is>
       </c>
       <c r="J50" t="b">
@@ -6494,7 +6494,7 @@
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Coluna dh_publicacao da aba sample.</t>
+          <t>Coluna data_recebimento da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6526,16 +6526,16 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>data_recebimento</t>
+          <t>dh_recebimento</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="J51" t="b">
@@ -6548,7 +6548,7 @@
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Coluna data_recebimento da aba sample.</t>
+          <t>Coluna dh_recebimento da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6580,16 +6580,16 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>dh_recebimento</t>
+          <t>observacoes</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J52" t="b">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Coluna dh_recebimento da aba sample.</t>
+          <t>Coluna observacoes da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6634,16 +6634,16 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>observacoes</t>
+          <t>dh_inicio_atividade</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>data_ou_data_hora</t>
         </is>
       </c>
       <c r="J53" t="b">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Coluna observacoes da aba sample.</t>
+          <t>Coluna dh_inicio_atividade da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6688,16 +6688,16 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>dh_inicio_atividade</t>
+          <t>localizacao</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>data_ou_data_hora</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J54" t="b">
@@ -6710,7 +6710,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Coluna dh_inicio_atividade da aba sample.</t>
+          <t>Coluna localizacao da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6742,16 +6742,16 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>15</v>
+        <v>16</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>localizacao</t>
+          <t>latitude</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J55" t="b">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Coluna localizacao da aba sample.</t>
+          <t>Coluna latitude da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6796,11 +6796,11 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>latitude</t>
+          <t>longitude</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Coluna latitude da aba sample.</t>
+          <t>Coluna longitude da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6850,16 +6850,16 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>longitude</t>
+          <t>coordenadas</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J57" t="b">
@@ -6872,7 +6872,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Coluna longitude da aba sample.</t>
+          <t>Coluna coordenadas da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6904,11 +6904,11 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>coordenadas</t>
+          <t>clima_ultimas_24h</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
@@ -6926,7 +6926,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Coluna coordenadas da aba sample.</t>
+          <t>Coluna clima_ultimas_24h da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6958,11 +6958,11 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>clima_ultimas_24h</t>
+          <t>clima</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
@@ -6980,7 +6980,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Coluna clima_ultimas_24h da aba sample.</t>
+          <t>Coluna clima da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7012,11 +7012,11 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>clima</t>
+          <t>tipo_coleta</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Coluna clima da aba sample.</t>
+          <t>Coluna tipo_coleta da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7066,11 +7066,11 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>tipo_coleta</t>
+          <t>responsavel_amostra</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
@@ -7088,7 +7088,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Coluna tipo_coleta da aba sample.</t>
+          <t>Coluna responsavel_amostra da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7120,11 +7120,11 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>22</v>
+        <v>23</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>responsavel_amostra</t>
+          <t>planejamento_amostragem</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -7142,7 +7142,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Coluna responsavel_amostra da aba sample.</t>
+          <t>Coluna planejamento_amostragem da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7174,11 +7174,11 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>planejamento_amostragem</t>
+          <t>descricao_nao_conformidade</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
@@ -7196,7 +7196,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Coluna planejamento_amostragem da aba sample.</t>
+          <t>Coluna descricao_nao_conformidade da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7213,26 +7213,26 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>client</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="E64" t="b">
         <v>1</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Dados de identificacao do cliente.</t>
         </is>
       </c>
       <c r="G64" t="n">
-        <v>24</v>
+        <v>1</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>descricao_nao_conformidade</t>
+          <t>nome_do_arquivo</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
@@ -7245,12 +7245,12 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>arquivo_pdf</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Coluna descricao_nao_conformidade da aba sample.</t>
+          <t>Nome do arquivo PDF de origem do registro.</t>
         </is>
       </c>
     </row>
@@ -7282,11 +7282,11 @@
         </is>
       </c>
       <c r="G65" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>nome_do_arquivo</t>
+          <t>template_id</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -7299,12 +7299,12 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>arquivo_pdf</t>
+          <t>document_scope</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Nome do arquivo PDF de origem do registro.</t>
+          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
         </is>
       </c>
     </row>
@@ -7336,11 +7336,11 @@
         </is>
       </c>
       <c r="G66" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>template_id</t>
+          <t>tipo_laudo</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -7353,12 +7353,12 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>document_scope</t>
+          <t>templates.theme_id</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
+          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
         </is>
       </c>
     </row>
@@ -7390,16 +7390,16 @@
         </is>
       </c>
       <c r="G67" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>tipo_laudo</t>
+          <t>id_amostra</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>inteiro_ou_texto</t>
         </is>
       </c>
       <c r="J67" t="b">
@@ -7407,12 +7407,12 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>templates.theme_id</t>
+          <t>text_extraction_rules.metadata.id_amostra</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
+          <t>Coluna id_amostra da aba client.</t>
         </is>
       </c>
     </row>
@@ -7444,16 +7444,16 @@
         </is>
       </c>
       <c r="G68" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>id_amostra</t>
+          <t>proposta_comercial</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
         <is>
-          <t>inteiro_ou_texto</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J68" t="b">
@@ -7461,12 +7461,12 @@
       </c>
       <c r="K68" t="inlineStr">
         <is>
-          <t>text_extraction_rules.metadata.id_amostra</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Coluna id_amostra da aba client.</t>
+          <t>Coluna proposta_comercial da aba client.</t>
         </is>
       </c>
     </row>
@@ -7498,11 +7498,11 @@
         </is>
       </c>
       <c r="G69" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>proposta_comercial</t>
+          <t>cliente</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Coluna proposta_comercial da aba client.</t>
+          <t>Coluna cliente da aba client.</t>
         </is>
       </c>
     </row>
@@ -7552,11 +7552,11 @@
         </is>
       </c>
       <c r="G70" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>cliente</t>
+          <t>cnpj_cpf</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -7574,7 +7574,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>Coluna cliente da aba client.</t>
+          <t>Coluna cnpj_cpf da aba client.</t>
         </is>
       </c>
     </row>
@@ -7606,11 +7606,11 @@
         </is>
       </c>
       <c r="G71" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>cnpj_cpf</t>
+          <t>contato</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -7628,7 +7628,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>Coluna cnpj_cpf da aba client.</t>
+          <t>Coluna contato da aba client.</t>
         </is>
       </c>
     </row>
@@ -7660,11 +7660,11 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>contato</t>
+          <t>telefone</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -7682,7 +7682,7 @@
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Coluna contato da aba client.</t>
+          <t>Coluna telefone da aba client.</t>
         </is>
       </c>
     </row>
@@ -7714,11 +7714,11 @@
         </is>
       </c>
       <c r="G73" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>telefone</t>
+          <t>endereco</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -7736,7 +7736,7 @@
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Coluna telefone da aba client.</t>
+          <t>Coluna endereco da aba client.</t>
         </is>
       </c>
     </row>
@@ -7753,44 +7753,26 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>table_extraction_audit</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>3</v>
+        <v>97</v>
       </c>
       <c r="E74" t="b">
         <v>1</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
-        </is>
-      </c>
-      <c r="G74" t="n">
-        <v>10</v>
-      </c>
-      <c r="H74" t="inlineStr">
-        <is>
-          <t>endereco</t>
-        </is>
-      </c>
-      <c r="I74" t="inlineStr">
-        <is>
-          <t>texto</t>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
         </is>
       </c>
       <c r="J74" t="b">
         <v>0</v>
       </c>
-      <c r="K74" t="inlineStr">
-        <is>
-          <t>parser</t>
-        </is>
-      </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>Coluna endereco da aba client.</t>
+          <t>Aba de auditoria das tabelas processadas, incluindo colunas detectadas, campos esperados e status da leitura.</t>
         </is>
       </c>
     </row>
@@ -7807,18 +7789,18 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>table_extraction_audit</t>
+          <t>classification_audit</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="E75" t="b">
         <v>1</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
+          <t>Auditoria da classificacao do PDF por template.</t>
         </is>
       </c>
       <c r="J75" t="b">
@@ -7826,7 +7808,7 @@
       </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Aba de auditoria das tabelas processadas, incluindo colunas detectadas, campos esperados e status da leitura.</t>
+          <t>Aba de auditoria da classificacao do template, incluindo regras encontradas, score e status por candidato.</t>
         </is>
       </c>
     </row>
@@ -7843,18 +7825,18 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>validation_errors</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="E76" t="b">
         <v>1</v>
       </c>
       <c r="F76" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Erros de validacao da saida.</t>
         </is>
       </c>
       <c r="J76" t="b">
@@ -7862,48 +7844,12 @@
       </c>
       <c r="L76" t="inlineStr">
         <is>
-          <t>Aba de auditoria da classificacao do template, incluindo regras encontradas, score e status por candidato.</t>
-        </is>
-      </c>
-    </row>
-    <row r="77">
-      <c r="A77" t="inlineStr">
-        <is>
-          <t>template_laudo_agua_v1</t>
-        </is>
-      </c>
-      <c r="B77" t="inlineStr">
-        <is>
-          <t>laudo_agua</t>
-        </is>
-      </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>validation_errors</t>
-        </is>
-      </c>
-      <c r="D77" t="n">
-        <v>99</v>
-      </c>
-      <c r="E77" t="b">
-        <v>1</v>
-      </c>
-      <c r="F77" t="inlineStr">
-        <is>
-          <t>Erros de validacao da saida.</t>
-        </is>
-      </c>
-      <c r="J77" t="b">
-        <v>0</v>
-      </c>
-      <c r="L77" t="inlineStr">
-        <is>
           <t>Aba de erros de validacao final, preenchida quando algum campo nao atende ao contrato esperado.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L77"/>
+  <autoFilter ref="A1:L76"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -10915,7 +10861,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I42"/>
+  <dimension ref="A1:I40"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -11214,11 +11160,11 @@
       </c>
       <c r="E7" t="inlineStr">
         <is>
-          <t>criterio_conformidade</t>
+          <t>referencia</t>
         </is>
       </c>
       <c r="F7" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="G7" t="inlineStr">
         <is>
@@ -11257,11 +11203,11 @@
       </c>
       <c r="E8" t="inlineStr">
         <is>
-          <t>referencia</t>
+          <t>data_inicio</t>
         </is>
       </c>
       <c r="F8" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="G8" t="inlineStr">
         <is>
@@ -11295,16 +11241,16 @@
       </c>
       <c r="D9" t="inlineStr">
         <is>
-          <t>AMOSTRA</t>
+          <t>BRANCO</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>data_inicio</t>
+          <t>resultado</t>
         </is>
       </c>
       <c r="F9" t="n">
-        <v>8</v>
+        <v>2</v>
       </c>
       <c r="G9" t="inlineStr">
         <is>
@@ -11343,11 +11289,11 @@
       </c>
       <c r="E10" t="inlineStr">
         <is>
-          <t>resultado</t>
+          <t>unidade</t>
         </is>
       </c>
       <c r="F10" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="G10" t="inlineStr">
         <is>
@@ -11386,11 +11332,11 @@
       </c>
       <c r="E11" t="inlineStr">
         <is>
-          <t>unidade</t>
+          <t>lq</t>
         </is>
       </c>
       <c r="F11" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="G11" t="inlineStr">
         <is>
@@ -11429,11 +11375,11 @@
       </c>
       <c r="E12" t="inlineStr">
         <is>
-          <t>lq</t>
+          <t>numero_cq</t>
         </is>
       </c>
       <c r="F12" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G12" t="inlineStr">
         <is>
@@ -11467,16 +11413,16 @@
       </c>
       <c r="D13" t="inlineStr">
         <is>
-          <t>BRANCO</t>
+          <t>DUPLICATA</t>
         </is>
       </c>
       <c r="E13" t="inlineStr">
         <is>
-          <t>numero_cq</t>
+          <t>resultado</t>
         </is>
       </c>
       <c r="F13" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="G13" t="inlineStr">
         <is>
@@ -11515,11 +11461,11 @@
       </c>
       <c r="E14" t="inlineStr">
         <is>
-          <t>resultado</t>
+          <t>unidade</t>
         </is>
       </c>
       <c r="F14" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="G14" t="inlineStr">
         <is>
@@ -11558,11 +11504,11 @@
       </c>
       <c r="E15" t="inlineStr">
         <is>
-          <t>unidade</t>
+          <t>numero_cq</t>
         </is>
       </c>
       <c r="F15" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="G15" t="inlineStr">
         <is>
@@ -11601,11 +11547,11 @@
       </c>
       <c r="E16" t="inlineStr">
         <is>
-          <t>numero_cq</t>
+          <t>duplicata</t>
         </is>
       </c>
       <c r="F16" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="G16" t="inlineStr">
         <is>
@@ -11644,11 +11590,11 @@
       </c>
       <c r="E17" t="inlineStr">
         <is>
-          <t>duplicata</t>
+          <t>faixa_aceitacao</t>
         </is>
       </c>
       <c r="F17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="G17" t="inlineStr">
         <is>
@@ -11687,11 +11633,11 @@
       </c>
       <c r="E18" t="inlineStr">
         <is>
-          <t>faixa_aceitacao</t>
+          <t>variacao_percentual</t>
         </is>
       </c>
       <c r="F18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="G18" t="inlineStr">
         <is>
@@ -11725,16 +11671,16 @@
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>DUPLICATA</t>
+          <t>RECUPERACAO</t>
         </is>
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>variacao_percentual</t>
+          <t>resultado</t>
         </is>
       </c>
       <c r="F19" t="n">
-        <v>6</v>
+        <v>5</v>
       </c>
       <c r="G19" t="inlineStr">
         <is>
@@ -11773,11 +11719,11 @@
       </c>
       <c r="E20" t="inlineStr">
         <is>
-          <t>resultado</t>
+          <t>unidade</t>
         </is>
       </c>
       <c r="F20" t="n">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="G20" t="inlineStr">
         <is>
@@ -11816,11 +11762,11 @@
       </c>
       <c r="E21" t="inlineStr">
         <is>
-          <t>unidade</t>
+          <t>numero_cq</t>
         </is>
       </c>
       <c r="F21" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="G21" t="inlineStr">
         <is>
@@ -11859,11 +11805,11 @@
       </c>
       <c r="E22" t="inlineStr">
         <is>
-          <t>numero_cq</t>
+          <t>faixa_aceitacao</t>
         </is>
       </c>
       <c r="F22" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="G22" t="inlineStr">
         <is>
@@ -11902,11 +11848,11 @@
       </c>
       <c r="E23" t="inlineStr">
         <is>
-          <t>faixa_aceitacao</t>
+          <t>quantidade_adicionada</t>
         </is>
       </c>
       <c r="F23" t="n">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="G23" t="inlineStr">
         <is>
@@ -11945,11 +11891,11 @@
       </c>
       <c r="E24" t="inlineStr">
         <is>
-          <t>quantidade_adicionada</t>
+          <t>recuperacao_percentual</t>
         </is>
       </c>
       <c r="F24" t="n">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="G24" t="inlineStr">
         <is>
@@ -11968,7 +11914,7 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>layout</t>
+          <t>header_alias</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
@@ -11983,20 +11929,22 @@
       </c>
       <c r="D25" t="inlineStr">
         <is>
-          <t>RECUPERACAO</t>
+          <t>NAO_APLICAVEL</t>
         </is>
       </c>
       <c r="E25" t="inlineStr">
         <is>
-          <t>recuperacao_percentual</t>
-        </is>
-      </c>
-      <c r="F25" t="n">
-        <v>5</v>
+          <t>parameter</t>
+        </is>
+      </c>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>NAO_APLICAVEL</t>
+        </is>
       </c>
       <c r="G25" t="inlineStr">
         <is>
-          <t>NAO_APLICAVEL</t>
+          <t>^(analise|parametros?)$</t>
         </is>
       </c>
       <c r="H25" t="b">
@@ -12004,7 +11952,7 @@
       </c>
       <c r="I25" t="inlineStr">
         <is>
-          <t>Coluna origem da tabela do PDF usada para preencher o campo informado.</t>
+          <t>Reconhece a coluna de parametro/analise.</t>
         </is>
       </c>
     </row>
@@ -12031,7 +11979,7 @@
       </c>
       <c r="E26" t="inlineStr">
         <is>
-          <t>parameter</t>
+          <t>unidade</t>
         </is>
       </c>
       <c r="F26" t="inlineStr">
@@ -12041,7 +11989,7 @@
       </c>
       <c r="G26" t="inlineStr">
         <is>
-          <t>^(analise|parametros?)$</t>
+          <t>^(unidade|unid)$</t>
         </is>
       </c>
       <c r="H26" t="b">
@@ -12049,7 +11997,7 @@
       </c>
       <c r="I26" t="inlineStr">
         <is>
-          <t>Reconhece a coluna de parametro/analise.</t>
+          <t>Reconhece a coluna de unidade de medida.</t>
         </is>
       </c>
     </row>
@@ -12076,7 +12024,7 @@
       </c>
       <c r="E27" t="inlineStr">
         <is>
-          <t>unidade</t>
+          <t>ld</t>
         </is>
       </c>
       <c r="F27" t="inlineStr">
@@ -12086,7 +12034,7 @@
       </c>
       <c r="G27" t="inlineStr">
         <is>
-          <t>^(unidade|unid)$</t>
+          <t>(^ld$|limite\s+de\s+deteccao)</t>
         </is>
       </c>
       <c r="H27" t="b">
@@ -12094,7 +12042,7 @@
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>Reconhece a coluna de unidade de medida.</t>
+          <t>Reconhece a coluna de limite de deteccao.</t>
         </is>
       </c>
     </row>
@@ -12121,7 +12069,7 @@
       </c>
       <c r="E28" t="inlineStr">
         <is>
-          <t>ld</t>
+          <t>lq</t>
         </is>
       </c>
       <c r="F28" t="inlineStr">
@@ -12131,7 +12079,7 @@
       </c>
       <c r="G28" t="inlineStr">
         <is>
-          <t>(^ld$|limite\s+de\s+deteccao)</t>
+          <t>(^lq$|limite\s+de\s+quantificacao)</t>
         </is>
       </c>
       <c r="H28" t="b">
@@ -12139,7 +12087,7 @@
       </c>
       <c r="I28" t="inlineStr">
         <is>
-          <t>Reconhece a coluna de limite de deteccao.</t>
+          <t>Reconhece a coluna de limite de quantificacao.</t>
         </is>
       </c>
     </row>
@@ -12166,7 +12114,7 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>lq</t>
+          <t>resultado</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
@@ -12176,7 +12124,7 @@
       </c>
       <c r="G29" t="inlineStr">
         <is>
-          <t>(^lq$|limite\s+de\s+quantificacao)</t>
+          <t>^resultados?$</t>
         </is>
       </c>
       <c r="H29" t="b">
@@ -12184,7 +12132,7 @@
       </c>
       <c r="I29" t="inlineStr">
         <is>
-          <t>Reconhece a coluna de limite de quantificacao.</t>
+          <t>Reconhece a coluna de resultado.</t>
         </is>
       </c>
     </row>
@@ -12211,7 +12159,7 @@
       </c>
       <c r="E30" t="inlineStr">
         <is>
-          <t>resultado</t>
+          <t>incerteza</t>
         </is>
       </c>
       <c r="F30" t="inlineStr">
@@ -12221,7 +12169,7 @@
       </c>
       <c r="G30" t="inlineStr">
         <is>
-          <t>^resultados?$</t>
+          <t>incerteza</t>
         </is>
       </c>
       <c r="H30" t="b">
@@ -12229,7 +12177,7 @@
       </c>
       <c r="I30" t="inlineStr">
         <is>
-          <t>Reconhece a coluna de resultado.</t>
+          <t>Reconhece a coluna de incerteza.</t>
         </is>
       </c>
     </row>
@@ -12256,7 +12204,7 @@
       </c>
       <c r="E31" t="inlineStr">
         <is>
-          <t>incerteza</t>
+          <t>referencia</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
@@ -12266,7 +12214,7 @@
       </c>
       <c r="G31" t="inlineStr">
         <is>
-          <t>incerteza</t>
+          <t>referencia</t>
         </is>
       </c>
       <c r="H31" t="b">
@@ -12274,7 +12222,7 @@
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>Reconhece a coluna de incerteza.</t>
+          <t>Reconhece a coluna de referencia metodologica.</t>
         </is>
       </c>
     </row>
@@ -12301,7 +12249,7 @@
       </c>
       <c r="E32" t="inlineStr">
         <is>
-          <t>referencia</t>
+          <t>data_inicio</t>
         </is>
       </c>
       <c r="F32" t="inlineStr">
@@ -12311,7 +12259,7 @@
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>referencia</t>
+          <t>data\s+de\s+inicio|data\s+inicio</t>
         </is>
       </c>
       <c r="H32" t="b">
@@ -12319,7 +12267,7 @@
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>Reconhece a coluna de referencia metodologica.</t>
+          <t>Reconhece a coluna de data de inicio da analise.</t>
         </is>
       </c>
     </row>
@@ -12346,7 +12294,7 @@
       </c>
       <c r="E33" t="inlineStr">
         <is>
-          <t>data_inicio</t>
+          <t>numero_cq</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
@@ -12356,7 +12304,7 @@
       </c>
       <c r="G33" t="inlineStr">
         <is>
-          <t>data\s+de\s+inicio|data\s+inicio</t>
+          <t>numero\s+do\s+cq|^cq$</t>
         </is>
       </c>
       <c r="H33" t="b">
@@ -12364,7 +12312,7 @@
       </c>
       <c r="I33" t="inlineStr">
         <is>
-          <t>Reconhece a coluna de data de inicio da analise.</t>
+          <t>Reconhece a coluna de numero do controle de qualidade.</t>
         </is>
       </c>
     </row>
@@ -12391,7 +12339,7 @@
       </c>
       <c r="E34" t="inlineStr">
         <is>
-          <t>numero_cq</t>
+          <t>duplicata</t>
         </is>
       </c>
       <c r="F34" t="inlineStr">
@@ -12401,7 +12349,7 @@
       </c>
       <c r="G34" t="inlineStr">
         <is>
-          <t>numero\s+do\s+cq|^cq$</t>
+          <t>^duplicata$</t>
         </is>
       </c>
       <c r="H34" t="b">
@@ -12409,7 +12357,7 @@
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>Reconhece a coluna de numero do controle de qualidade.</t>
+          <t>Reconhece a coluna de duplicata.</t>
         </is>
       </c>
     </row>
@@ -12436,7 +12384,7 @@
       </c>
       <c r="E35" t="inlineStr">
         <is>
-          <t>duplicata</t>
+          <t>faixa_aceitacao</t>
         </is>
       </c>
       <c r="F35" t="inlineStr">
@@ -12446,7 +12394,7 @@
       </c>
       <c r="G35" t="inlineStr">
         <is>
-          <t>^duplicata$</t>
+          <t>faixa\s+de\s+aceitacao</t>
         </is>
       </c>
       <c r="H35" t="b">
@@ -12454,7 +12402,7 @@
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>Reconhece a coluna de duplicata.</t>
+          <t>Reconhece a coluna de faixa de aceitacao.</t>
         </is>
       </c>
     </row>
@@ -12481,7 +12429,7 @@
       </c>
       <c r="E36" t="inlineStr">
         <is>
-          <t>faixa_aceitacao</t>
+          <t>variacao_percentual</t>
         </is>
       </c>
       <c r="F36" t="inlineStr">
@@ -12491,7 +12439,7 @@
       </c>
       <c r="G36" t="inlineStr">
         <is>
-          <t>faixa\s+de\s+aceitacao</t>
+          <t>variacao</t>
         </is>
       </c>
       <c r="H36" t="b">
@@ -12499,7 +12447,7 @@
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>Reconhece a coluna de faixa de aceitacao.</t>
+          <t>Reconhece a coluna de variacao percentual.</t>
         </is>
       </c>
     </row>
@@ -12526,7 +12474,7 @@
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>variacao_percentual</t>
+          <t>quantidade_adicionada</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -12536,7 +12484,7 @@
       </c>
       <c r="G37" t="inlineStr">
         <is>
-          <t>variacao</t>
+          <t>quantidade\s+adicionada|^qtd\s+adicionada$</t>
         </is>
       </c>
       <c r="H37" t="b">
@@ -12544,7 +12492,7 @@
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>Reconhece a coluna de variacao percentual.</t>
+          <t>Reconhece a coluna de quantidade adicionada.</t>
         </is>
       </c>
     </row>
@@ -12571,7 +12519,7 @@
       </c>
       <c r="E38" t="inlineStr">
         <is>
-          <t>quantidade_adicionada</t>
+          <t>recuperacao_percentual</t>
         </is>
       </c>
       <c r="F38" t="inlineStr">
@@ -12581,7 +12529,7 @@
       </c>
       <c r="G38" t="inlineStr">
         <is>
-          <t>quantidade\s+adicionada|^qtd\s+adicionada$</t>
+          <t>recuperacao</t>
         </is>
       </c>
       <c r="H38" t="b">
@@ -12589,7 +12537,7 @@
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>Reconhece a coluna de quantidade adicionada.</t>
+          <t>Reconhece a coluna de recuperacao percentual.</t>
         </is>
       </c>
     </row>
@@ -12616,7 +12564,7 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>recuperacao_percentual</t>
+          <t>conama</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
@@ -12626,7 +12574,7 @@
       </c>
       <c r="G39" t="inlineStr">
         <is>
-          <t>recuperacao</t>
+          <t>conama</t>
         </is>
       </c>
       <c r="H39" t="b">
@@ -12634,7 +12582,7 @@
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>Reconhece a coluna de recuperacao percentual.</t>
+          <t>Reconhece colunas normativas CONAMA; o valor da linha sai no campo conama.</t>
         </is>
       </c>
     </row>
@@ -12661,7 +12609,7 @@
       </c>
       <c r="E40" t="inlineStr">
         <is>
-          <t>conama</t>
+          <t>copam_cerh</t>
         </is>
       </c>
       <c r="F40" t="inlineStr">
@@ -12671,7 +12619,7 @@
       </c>
       <c r="G40" t="inlineStr">
         <is>
-          <t>conama</t>
+          <t>copam|cerh|deliberacao\s+normativa</t>
         </is>
       </c>
       <c r="H40" t="b">
@@ -12679,102 +12627,12 @@
       </c>
       <c r="I40" t="inlineStr">
         <is>
-          <t>Reconhece colunas normativas CONAMA; o valor da linha sai no campo conama.</t>
-        </is>
-      </c>
-    </row>
-    <row r="41">
-      <c r="A41" t="inlineStr">
-        <is>
-          <t>header_alias</t>
-        </is>
-      </c>
-      <c r="B41" t="inlineStr">
-        <is>
-          <t>template_laudo_agua_v1</t>
-        </is>
-      </c>
-      <c r="C41" t="inlineStr">
-        <is>
-          <t>results_extract</t>
-        </is>
-      </c>
-      <c r="D41" t="inlineStr">
-        <is>
-          <t>NAO_APLICAVEL</t>
-        </is>
-      </c>
-      <c r="E41" t="inlineStr">
-        <is>
-          <t>copam_cerh</t>
-        </is>
-      </c>
-      <c r="F41" t="inlineStr">
-        <is>
-          <t>NAO_APLICAVEL</t>
-        </is>
-      </c>
-      <c r="G41" t="inlineStr">
-        <is>
-          <t>copam|cerh|deliberacao\s+normativa</t>
-        </is>
-      </c>
-      <c r="H41" t="b">
-        <v>1</v>
-      </c>
-      <c r="I41" t="inlineStr">
-        <is>
           <t>Reconhece colunas normativas COPAM/CERH; o valor da linha sai no campo copam_cerh.</t>
         </is>
       </c>
     </row>
-    <row r="42">
-      <c r="A42" t="inlineStr">
-        <is>
-          <t>header_alias</t>
-        </is>
-      </c>
-      <c r="B42" t="inlineStr">
-        <is>
-          <t>template_laudo_agua_v1</t>
-        </is>
-      </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>results_extract</t>
-        </is>
-      </c>
-      <c r="D42" t="inlineStr">
-        <is>
-          <t>NAO_APLICAVEL</t>
-        </is>
-      </c>
-      <c r="E42" t="inlineStr">
-        <is>
-          <t>criterio_conformidade</t>
-        </is>
-      </c>
-      <c r="F42" t="inlineStr">
-        <is>
-          <t>NAO_APLICAVEL</t>
-        </is>
-      </c>
-      <c r="G42" t="inlineStr">
-        <is>
-          <t>criterio</t>
-        </is>
-      </c>
-      <c r="H42" t="b">
-        <v>1</v>
-      </c>
-      <c r="I42" t="inlineStr">
-        <is>
-          <t>Reconhece colunas genericas de criterio de conformidade quando nao forem CONAMA ou COPAM/CERH.</t>
-        </is>
-      </c>
-    </row>
   </sheetData>
-  <autoFilter ref="A1:I42"/>
+  <autoFilter ref="A1:I40"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Structure normative criteria ranges
</commit_message>
<xml_diff>
--- a/config/taxonomy_config_consolidada_v1.xlsx
+++ b/config/taxonomy_config_consolidada_v1.xlsx
@@ -20,7 +20,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'README_FORMATO'!$A$1:$C$8</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'templates'!$A$1:$H$15</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'template_rules'!$A$1:$G$78</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'output_model'!$A$1:$L$76</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'output_model'!$A$1:$L$84</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'text_extraction_rules'!$A$1:$G$85</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'table_extraction_rules'!$A$1:$I$40</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'section_rules'!$A$1:$L$54</definedName>
@@ -3773,7 +3773,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L76"/>
+  <dimension ref="A1:L84"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -4694,7 +4694,7 @@
       </c>
       <c r="H17" t="inlineStr">
         <is>
-          <t>copam_cerh</t>
+          <t>conama_operador</t>
         </is>
       </c>
       <c r="I17" t="inlineStr">
@@ -4707,12 +4707,12 @@
       </c>
       <c r="K17" t="inlineStr">
         <is>
-          <t>table_extraction_rules.copam_cerh_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L17" t="inlineStr">
         <is>
-          <t>Valor extraido da coluna normativa COPAM/CERH, quando esse cabecalho existir na tabela.</t>
+          <t>Operador extraido do valor CONAMA, como &lt;, &gt;, min ou max.</t>
         </is>
       </c>
     </row>
@@ -4748,12 +4748,12 @@
       </c>
       <c r="H18" t="inlineStr">
         <is>
-          <t>ld</t>
+          <t>conama_minimo</t>
         </is>
       </c>
       <c r="I18" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J18" t="b">
@@ -4761,12 +4761,12 @@
       </c>
       <c r="K18" t="inlineStr">
         <is>
-          <t>table_extraction_rules.ld_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L18" t="inlineStr">
         <is>
-          <t>LD extraido diretamente do PDF, preservado como texto original.</t>
+          <t>Valor minimo extraido do campo conama, gravado como numero no Excel.</t>
         </is>
       </c>
     </row>
@@ -4802,7 +4802,7 @@
       </c>
       <c r="H19" t="inlineStr">
         <is>
-          <t>ld_minimo</t>
+          <t>conama_maximo</t>
         </is>
       </c>
       <c r="I19" t="inlineStr">
@@ -4820,7 +4820,7 @@
       </c>
       <c r="L19" t="inlineStr">
         <is>
-          <t>Valor minimo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
+          <t>Valor maximo extraido do campo conama, gravado como numero no Excel.</t>
         </is>
       </c>
     </row>
@@ -4856,12 +4856,12 @@
       </c>
       <c r="H20" t="inlineStr">
         <is>
-          <t>ld_maximo</t>
+          <t>conama_unidade</t>
         </is>
       </c>
       <c r="I20" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J20" t="b">
@@ -4874,7 +4874,7 @@
       </c>
       <c r="L20" t="inlineStr">
         <is>
-          <t>Valor maximo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
+          <t>Unidade de medida extraida do campo conama, quando informada.</t>
         </is>
       </c>
     </row>
@@ -4910,7 +4910,7 @@
       </c>
       <c r="H21" t="inlineStr">
         <is>
-          <t>ld_unidade</t>
+          <t>copam_cerh</t>
         </is>
       </c>
       <c r="I21" t="inlineStr">
@@ -4923,12 +4923,12 @@
       </c>
       <c r="K21" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.copam_cerh_col</t>
         </is>
       </c>
       <c r="L21" t="inlineStr">
         <is>
-          <t>Unidade de medida do LD, quando informada no campo ld.</t>
+          <t>Valor extraido da coluna normativa COPAM/CERH, quando esse cabecalho existir na tabela.</t>
         </is>
       </c>
     </row>
@@ -4964,7 +4964,7 @@
       </c>
       <c r="H22" t="inlineStr">
         <is>
-          <t>lq</t>
+          <t>copam_cerh_operador</t>
         </is>
       </c>
       <c r="I22" t="inlineStr">
@@ -4977,12 +4977,12 @@
       </c>
       <c r="K22" t="inlineStr">
         <is>
-          <t>table_extraction_rules.lq_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L22" t="inlineStr">
         <is>
-          <t>LQ extraido diretamente do PDF, preservado como texto original.</t>
+          <t>Operador extraido do valor COPAM/CERH, como &lt;, &gt;, min ou max.</t>
         </is>
       </c>
     </row>
@@ -5018,7 +5018,7 @@
       </c>
       <c r="H23" t="inlineStr">
         <is>
-          <t>lq_minimo</t>
+          <t>copam_cerh_minimo</t>
         </is>
       </c>
       <c r="I23" t="inlineStr">
@@ -5036,7 +5036,7 @@
       </c>
       <c r="L23" t="inlineStr">
         <is>
-          <t>Valor minimo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
+          <t>Valor minimo extraido do campo copam_cerh, gravado como numero no Excel.</t>
         </is>
       </c>
     </row>
@@ -5072,7 +5072,7 @@
       </c>
       <c r="H24" t="inlineStr">
         <is>
-          <t>lq_maximo</t>
+          <t>copam_cerh_maximo</t>
         </is>
       </c>
       <c r="I24" t="inlineStr">
@@ -5090,7 +5090,7 @@
       </c>
       <c r="L24" t="inlineStr">
         <is>
-          <t>Valor maximo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
+          <t>Valor maximo extraido do campo copam_cerh, gravado como numero no Excel.</t>
         </is>
       </c>
     </row>
@@ -5126,7 +5126,7 @@
       </c>
       <c r="H25" t="inlineStr">
         <is>
-          <t>lq_unidade</t>
+          <t>copam_cerh_unidade</t>
         </is>
       </c>
       <c r="I25" t="inlineStr">
@@ -5144,7 +5144,7 @@
       </c>
       <c r="L25" t="inlineStr">
         <is>
-          <t>Unidade de medida do LQ, quando informada no campo lq.</t>
+          <t>Unidade de medida extraida do campo copam_cerh, quando informada.</t>
         </is>
       </c>
     </row>
@@ -5180,7 +5180,7 @@
       </c>
       <c r="H26" t="inlineStr">
         <is>
-          <t>referencia</t>
+          <t>ld</t>
         </is>
       </c>
       <c r="I26" t="inlineStr">
@@ -5193,12 +5193,12 @@
       </c>
       <c r="K26" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.ld_col</t>
         </is>
       </c>
       <c r="L26" t="inlineStr">
         <is>
-          <t>Coluna referencia da aba results_extract.</t>
+          <t>LD extraido diretamente do PDF, preservado como texto original.</t>
         </is>
       </c>
     </row>
@@ -5234,12 +5234,12 @@
       </c>
       <c r="H27" t="inlineStr">
         <is>
-          <t>incerteza</t>
+          <t>ld_minimo</t>
         </is>
       </c>
       <c r="I27" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J27" t="b">
@@ -5247,12 +5247,12 @@
       </c>
       <c r="K27" t="inlineStr">
         <is>
-          <t>table_extraction_rules.incerteza_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L27" t="inlineStr">
         <is>
-          <t>Incerteza extraida diretamente do PDF, preservada como texto original.</t>
+          <t>Valor minimo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
         </is>
       </c>
     </row>
@@ -5288,7 +5288,7 @@
       </c>
       <c r="H28" t="inlineStr">
         <is>
-          <t>incerteza_valor</t>
+          <t>ld_maximo</t>
         </is>
       </c>
       <c r="I28" t="inlineStr">
@@ -5306,7 +5306,7 @@
       </c>
       <c r="L28" t="inlineStr">
         <is>
-          <t>Valor da incerteza gravado como numero no Excel, com casas decimais preservadas conforme o campo incerteza.</t>
+          <t>Valor maximo do LD gravado como numero no Excel, com casas decimais preservadas conforme o campo ld.</t>
         </is>
       </c>
     </row>
@@ -5342,7 +5342,7 @@
       </c>
       <c r="H29" t="inlineStr">
         <is>
-          <t>incerteza_unidade</t>
+          <t>ld_unidade</t>
         </is>
       </c>
       <c r="I29" t="inlineStr">
@@ -5360,7 +5360,7 @@
       </c>
       <c r="L29" t="inlineStr">
         <is>
-          <t>Unidade de medida da incerteza, quando informada no campo incerteza.</t>
+          <t>Unidade de medida do LD, quando informada no campo ld.</t>
         </is>
       </c>
     </row>
@@ -5396,7 +5396,7 @@
       </c>
       <c r="H30" t="inlineStr">
         <is>
-          <t>numero_cq</t>
+          <t>lq</t>
         </is>
       </c>
       <c r="I30" t="inlineStr">
@@ -5409,12 +5409,12 @@
       </c>
       <c r="K30" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.lq_col</t>
         </is>
       </c>
       <c r="L30" t="inlineStr">
         <is>
-          <t>Coluna numero_cq da aba results_extract.</t>
+          <t>LQ extraido diretamente do PDF, preservado como texto original.</t>
         </is>
       </c>
     </row>
@@ -5450,12 +5450,12 @@
       </c>
       <c r="H31" t="inlineStr">
         <is>
-          <t>duplicata</t>
+          <t>lq_minimo</t>
         </is>
       </c>
       <c r="I31" t="inlineStr">
         <is>
-          <t>texto_numerico</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J31" t="b">
@@ -5463,12 +5463,12 @@
       </c>
       <c r="K31" t="inlineStr">
         <is>
-          <t>table_extraction_rules.duplicata_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L31" t="inlineStr">
         <is>
-          <t>Valor de duplicata extraido diretamente do PDF; validado como texto numerico.</t>
+          <t>Valor minimo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
         </is>
       </c>
     </row>
@@ -5504,12 +5504,12 @@
       </c>
       <c r="H32" t="inlineStr">
         <is>
-          <t>faixa_aceitacao</t>
+          <t>lq_maximo</t>
         </is>
       </c>
       <c r="I32" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J32" t="b">
@@ -5517,12 +5517,12 @@
       </c>
       <c r="K32" t="inlineStr">
         <is>
-          <t>table_extraction_rules.faixa_aceitacao_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L32" t="inlineStr">
         <is>
-          <t>Faixa de aceitacao extraida diretamente do PDF, preservada como texto original.</t>
+          <t>Valor maximo do LQ gravado como numero no Excel, com casas decimais preservadas conforme o campo lq.</t>
         </is>
       </c>
     </row>
@@ -5558,7 +5558,7 @@
       </c>
       <c r="H33" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_operador</t>
+          <t>lq_unidade</t>
         </is>
       </c>
       <c r="I33" t="inlineStr">
@@ -5576,7 +5576,7 @@
       </c>
       <c r="L33" t="inlineStr">
         <is>
-          <t>Operador extraido da faixa de aceitacao, quando informado no PDF.</t>
+          <t>Unidade de medida do LQ, quando informada no campo lq.</t>
         </is>
       </c>
     </row>
@@ -5612,12 +5612,12 @@
       </c>
       <c r="H34" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_minimo</t>
+          <t>referencia</t>
         </is>
       </c>
       <c r="I34" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J34" t="b">
@@ -5630,7 +5630,7 @@
       </c>
       <c r="L34" t="inlineStr">
         <is>
-          <t>Valor minimo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
+          <t>Coluna referencia da aba results_extract.</t>
         </is>
       </c>
     </row>
@@ -5666,12 +5666,12 @@
       </c>
       <c r="H35" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_maximo</t>
+          <t>incerteza</t>
         </is>
       </c>
       <c r="I35" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J35" t="b">
@@ -5679,12 +5679,12 @@
       </c>
       <c r="K35" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.incerteza_col</t>
         </is>
       </c>
       <c r="L35" t="inlineStr">
         <is>
-          <t>Valor maximo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
+          <t>Incerteza extraida diretamente do PDF, preservada como texto original.</t>
         </is>
       </c>
     </row>
@@ -5720,12 +5720,12 @@
       </c>
       <c r="H36" t="inlineStr">
         <is>
-          <t>faixa_aceitacao_unidade</t>
+          <t>incerteza_valor</t>
         </is>
       </c>
       <c r="I36" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J36" t="b">
@@ -5738,7 +5738,7 @@
       </c>
       <c r="L36" t="inlineStr">
         <is>
-          <t>Unidade de medida da faixa de aceitacao, quando informada no campo faixa_aceitacao.</t>
+          <t>Valor da incerteza gravado como numero no Excel, com casas decimais preservadas conforme o campo incerteza.</t>
         </is>
       </c>
     </row>
@@ -5774,12 +5774,12 @@
       </c>
       <c r="H37" t="inlineStr">
         <is>
-          <t>variacao_percentual</t>
+          <t>incerteza_unidade</t>
         </is>
       </c>
       <c r="I37" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J37" t="b">
@@ -5787,12 +5787,12 @@
       </c>
       <c r="K37" t="inlineStr">
         <is>
-          <t>table_extraction_rules.variacao_percentual_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L37" t="inlineStr">
         <is>
-          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
+          <t>Unidade de medida da incerteza, quando informada no campo incerteza.</t>
         </is>
       </c>
     </row>
@@ -5828,12 +5828,12 @@
       </c>
       <c r="H38" t="inlineStr">
         <is>
-          <t>quantidade_adicionada</t>
+          <t>numero_cq</t>
         </is>
       </c>
       <c r="I38" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J38" t="b">
@@ -5841,12 +5841,12 @@
       </c>
       <c r="K38" t="inlineStr">
         <is>
-          <t>table_extraction_rules.quantidade_adicionada_col</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L38" t="inlineStr">
         <is>
-          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
+          <t>Coluna numero_cq da aba results_extract.</t>
         </is>
       </c>
     </row>
@@ -5882,12 +5882,12 @@
       </c>
       <c r="H39" t="inlineStr">
         <is>
-          <t>recuperacao_percentual</t>
+          <t>duplicata</t>
         </is>
       </c>
       <c r="I39" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>texto_numerico</t>
         </is>
       </c>
       <c r="J39" t="b">
@@ -5895,12 +5895,12 @@
       </c>
       <c r="K39" t="inlineStr">
         <is>
-          <t>table_extraction_rules.recuperacao_percentual_col</t>
+          <t>table_extraction_rules.duplicata_col</t>
         </is>
       </c>
       <c r="L39" t="inlineStr">
         <is>
-          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
+          <t>Valor de duplicata extraido diretamente do PDF; validado como texto numerico.</t>
         </is>
       </c>
     </row>
@@ -5917,26 +5917,26 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E40" t="b">
         <v>1</v>
       </c>
       <c r="F40" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
       <c r="G40" t="n">
-        <v>1</v>
+        <v>39</v>
       </c>
       <c r="H40" t="inlineStr">
         <is>
-          <t>nome_do_arquivo</t>
+          <t>faixa_aceitacao</t>
         </is>
       </c>
       <c r="I40" t="inlineStr">
@@ -5949,12 +5949,12 @@
       </c>
       <c r="K40" t="inlineStr">
         <is>
-          <t>arquivo_pdf</t>
+          <t>table_extraction_rules.faixa_aceitacao_col</t>
         </is>
       </c>
       <c r="L40" t="inlineStr">
         <is>
-          <t>Nome do arquivo PDF de origem do registro.</t>
+          <t>Faixa de aceitacao extraida diretamente do PDF, preservada como texto original.</t>
         </is>
       </c>
     </row>
@@ -5971,26 +5971,26 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E41" t="b">
         <v>1</v>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
       <c r="G41" t="n">
-        <v>2</v>
+        <v>40</v>
       </c>
       <c r="H41" t="inlineStr">
         <is>
-          <t>template_id</t>
+          <t>faixa_aceitacao_operador</t>
         </is>
       </c>
       <c r="I41" t="inlineStr">
@@ -6003,12 +6003,12 @@
       </c>
       <c r="K41" t="inlineStr">
         <is>
-          <t>document_scope</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L41" t="inlineStr">
         <is>
-          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
+          <t>Operador extraido da faixa de aceitacao, quando informado no PDF.</t>
         </is>
       </c>
     </row>
@@ -6025,31 +6025,31 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E42" t="b">
         <v>1</v>
       </c>
       <c r="F42" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
       <c r="G42" t="n">
-        <v>3</v>
+        <v>41</v>
       </c>
       <c r="H42" t="inlineStr">
         <is>
-          <t>tipo_laudo</t>
+          <t>faixa_aceitacao_minimo</t>
         </is>
       </c>
       <c r="I42" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J42" t="b">
@@ -6057,12 +6057,12 @@
       </c>
       <c r="K42" t="inlineStr">
         <is>
-          <t>templates.theme_id</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L42" t="inlineStr">
         <is>
-          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
+          <t>Valor minimo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -6079,31 +6079,31 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E43" t="b">
         <v>1</v>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
       <c r="G43" t="n">
-        <v>4</v>
+        <v>42</v>
       </c>
       <c r="H43" t="inlineStr">
         <is>
-          <t>id_amostra</t>
+          <t>faixa_aceitacao_maximo</t>
         </is>
       </c>
       <c r="I43" t="inlineStr">
         <is>
-          <t>inteiro_ou_texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J43" t="b">
@@ -6111,12 +6111,12 @@
       </c>
       <c r="K43" t="inlineStr">
         <is>
-          <t>text_extraction_rules.metadata.id_amostra</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L43" t="inlineStr">
         <is>
-          <t>Coluna id_amostra da aba sample.</t>
+          <t>Valor maximo da aceitacao gravado como numero no Excel, com casas decimais preservadas conforme o campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -6133,26 +6133,26 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E44" t="b">
         <v>1</v>
       </c>
       <c r="F44" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
       <c r="G44" t="n">
-        <v>5</v>
+        <v>43</v>
       </c>
       <c r="H44" t="inlineStr">
         <is>
-          <t>tipo_amostra</t>
+          <t>faixa_aceitacao_unidade</t>
         </is>
       </c>
       <c r="I44" t="inlineStr">
@@ -6170,7 +6170,7 @@
       </c>
       <c r="L44" t="inlineStr">
         <is>
-          <t>Coluna tipo_amostra da aba sample.</t>
+          <t>Unidade de medida da faixa de aceitacao, quando informada no campo faixa_aceitacao.</t>
         </is>
       </c>
     </row>
@@ -6187,31 +6187,31 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E45" t="b">
         <v>1</v>
       </c>
       <c r="F45" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
       <c r="G45" t="n">
-        <v>6</v>
+        <v>44</v>
       </c>
       <c r="H45" t="inlineStr">
         <is>
-          <t>criterio_conformidade</t>
+          <t>variacao_percentual</t>
         </is>
       </c>
       <c r="I45" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J45" t="b">
@@ -6219,12 +6219,12 @@
       </c>
       <c r="K45" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.variacao_percentual_col</t>
         </is>
       </c>
       <c r="L45" t="inlineStr">
         <is>
-          <t>Coluna criterio_conformidade da aba sample.</t>
+          <t>Variacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
     </row>
@@ -6241,31 +6241,31 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E46" t="b">
         <v>1</v>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
       <c r="G46" t="n">
-        <v>7</v>
+        <v>45</v>
       </c>
       <c r="H46" t="inlineStr">
         <is>
-          <t>data_coleta</t>
+          <t>quantidade_adicionada</t>
         </is>
       </c>
       <c r="I46" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J46" t="b">
@@ -6273,12 +6273,12 @@
       </c>
       <c r="K46" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.quantidade_adicionada_col</t>
         </is>
       </c>
       <c r="L46" t="inlineStr">
         <is>
-          <t>Coluna data_coleta da aba sample.</t>
+          <t>Quantidade adicionada esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
     </row>
@@ -6295,31 +6295,31 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>sample</t>
+          <t>results_extract</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E47" t="b">
         <v>1</v>
       </c>
       <c r="F47" t="inlineStr">
         <is>
-          <t>Dados de amostra/cabecalho do PDF.</t>
+          <t>Resultados extraidos do PDF para o template.</t>
         </is>
       </c>
       <c r="G47" t="n">
-        <v>8</v>
+        <v>46</v>
       </c>
       <c r="H47" t="inlineStr">
         <is>
-          <t>dh_coleta</t>
+          <t>recuperacao_percentual</t>
         </is>
       </c>
       <c r="I47" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J47" t="b">
@@ -6327,12 +6327,12 @@
       </c>
       <c r="K47" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>table_extraction_rules.recuperacao_percentual_col</t>
         </is>
       </c>
       <c r="L47" t="inlineStr">
         <is>
-          <t>Coluna dh_coleta da aba sample.</t>
+          <t>Recuperacao percentual esperada como numero. Se o PDF trouxer texto, o valor e preservado na saida e sinalizado em validation_errors.</t>
         </is>
       </c>
     </row>
@@ -6364,16 +6364,16 @@
         </is>
       </c>
       <c r="G48" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H48" t="inlineStr">
         <is>
-          <t>data_publicacao</t>
+          <t>nome_do_arquivo</t>
         </is>
       </c>
       <c r="I48" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J48" t="b">
@@ -6381,12 +6381,12 @@
       </c>
       <c r="K48" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>arquivo_pdf</t>
         </is>
       </c>
       <c r="L48" t="inlineStr">
         <is>
-          <t>Coluna data_publicacao da aba sample.</t>
+          <t>Nome do arquivo PDF de origem do registro.</t>
         </is>
       </c>
     </row>
@@ -6418,16 +6418,16 @@
         </is>
       </c>
       <c r="G49" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H49" t="inlineStr">
         <is>
-          <t>dh_publicacao</t>
+          <t>template_id</t>
         </is>
       </c>
       <c r="I49" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J49" t="b">
@@ -6435,12 +6435,12 @@
       </c>
       <c r="K49" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>document_scope</t>
         </is>
       </c>
       <c r="L49" t="inlineStr">
         <is>
-          <t>Coluna dh_publicacao da aba sample.</t>
+          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
         </is>
       </c>
     </row>
@@ -6472,16 +6472,16 @@
         </is>
       </c>
       <c r="G50" t="n">
-        <v>11</v>
+        <v>3</v>
       </c>
       <c r="H50" t="inlineStr">
         <is>
-          <t>data_recebimento</t>
+          <t>tipo_laudo</t>
         </is>
       </c>
       <c r="I50" t="inlineStr">
         <is>
-          <t>data</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J50" t="b">
@@ -6489,12 +6489,12 @@
       </c>
       <c r="K50" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>templates.theme_id</t>
         </is>
       </c>
       <c r="L50" t="inlineStr">
         <is>
-          <t>Coluna data_recebimento da aba sample.</t>
+          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
         </is>
       </c>
     </row>
@@ -6526,16 +6526,16 @@
         </is>
       </c>
       <c r="G51" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="H51" t="inlineStr">
         <is>
-          <t>dh_recebimento</t>
+          <t>id_amostra</t>
         </is>
       </c>
       <c r="I51" t="inlineStr">
         <is>
-          <t>hora</t>
+          <t>inteiro_ou_texto</t>
         </is>
       </c>
       <c r="J51" t="b">
@@ -6543,12 +6543,12 @@
       </c>
       <c r="K51" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>text_extraction_rules.metadata.id_amostra</t>
         </is>
       </c>
       <c r="L51" t="inlineStr">
         <is>
-          <t>Coluna dh_recebimento da aba sample.</t>
+          <t>Coluna id_amostra da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6580,11 +6580,11 @@
         </is>
       </c>
       <c r="G52" t="n">
-        <v>13</v>
+        <v>5</v>
       </c>
       <c r="H52" t="inlineStr">
         <is>
-          <t>observacoes</t>
+          <t>tipo_amostra</t>
         </is>
       </c>
       <c r="I52" t="inlineStr">
@@ -6602,7 +6602,7 @@
       </c>
       <c r="L52" t="inlineStr">
         <is>
-          <t>Coluna observacoes da aba sample.</t>
+          <t>Coluna tipo_amostra da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6634,16 +6634,16 @@
         </is>
       </c>
       <c r="G53" t="n">
-        <v>14</v>
+        <v>6</v>
       </c>
       <c r="H53" t="inlineStr">
         <is>
-          <t>dh_inicio_atividade</t>
+          <t>criterio_conformidade</t>
         </is>
       </c>
       <c r="I53" t="inlineStr">
         <is>
-          <t>data_ou_data_hora</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J53" t="b">
@@ -6656,7 +6656,7 @@
       </c>
       <c r="L53" t="inlineStr">
         <is>
-          <t>Coluna dh_inicio_atividade da aba sample.</t>
+          <t>Coluna criterio_conformidade da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6688,16 +6688,16 @@
         </is>
       </c>
       <c r="G54" t="n">
-        <v>15</v>
+        <v>7</v>
       </c>
       <c r="H54" t="inlineStr">
         <is>
-          <t>localizacao</t>
+          <t>data_coleta</t>
         </is>
       </c>
       <c r="I54" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>data</t>
         </is>
       </c>
       <c r="J54" t="b">
@@ -6710,7 +6710,7 @@
       </c>
       <c r="L54" t="inlineStr">
         <is>
-          <t>Coluna localizacao da aba sample.</t>
+          <t>Coluna data_coleta da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6742,16 +6742,16 @@
         </is>
       </c>
       <c r="G55" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="H55" t="inlineStr">
         <is>
-          <t>latitude</t>
+          <t>dh_coleta</t>
         </is>
       </c>
       <c r="I55" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="J55" t="b">
@@ -6764,7 +6764,7 @@
       </c>
       <c r="L55" t="inlineStr">
         <is>
-          <t>Coluna latitude da aba sample.</t>
+          <t>Coluna dh_coleta da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6796,16 +6796,16 @@
         </is>
       </c>
       <c r="G56" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="H56" t="inlineStr">
         <is>
-          <t>longitude</t>
+          <t>data_publicacao</t>
         </is>
       </c>
       <c r="I56" t="inlineStr">
         <is>
-          <t>decimal</t>
+          <t>data</t>
         </is>
       </c>
       <c r="J56" t="b">
@@ -6818,7 +6818,7 @@
       </c>
       <c r="L56" t="inlineStr">
         <is>
-          <t>Coluna longitude da aba sample.</t>
+          <t>Coluna data_publicacao da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6850,16 +6850,16 @@
         </is>
       </c>
       <c r="G57" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="H57" t="inlineStr">
         <is>
-          <t>coordenadas</t>
+          <t>dh_publicacao</t>
         </is>
       </c>
       <c r="I57" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="J57" t="b">
@@ -6872,7 +6872,7 @@
       </c>
       <c r="L57" t="inlineStr">
         <is>
-          <t>Coluna coordenadas da aba sample.</t>
+          <t>Coluna dh_publicacao da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6904,16 +6904,16 @@
         </is>
       </c>
       <c r="G58" t="n">
-        <v>19</v>
+        <v>11</v>
       </c>
       <c r="H58" t="inlineStr">
         <is>
-          <t>clima_ultimas_24h</t>
+          <t>data_recebimento</t>
         </is>
       </c>
       <c r="I58" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>data</t>
         </is>
       </c>
       <c r="J58" t="b">
@@ -6926,7 +6926,7 @@
       </c>
       <c r="L58" t="inlineStr">
         <is>
-          <t>Coluna clima_ultimas_24h da aba sample.</t>
+          <t>Coluna data_recebimento da aba sample.</t>
         </is>
       </c>
     </row>
@@ -6958,16 +6958,16 @@
         </is>
       </c>
       <c r="G59" t="n">
-        <v>20</v>
+        <v>12</v>
       </c>
       <c r="H59" t="inlineStr">
         <is>
-          <t>clima</t>
+          <t>dh_recebimento</t>
         </is>
       </c>
       <c r="I59" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>hora</t>
         </is>
       </c>
       <c r="J59" t="b">
@@ -6980,7 +6980,7 @@
       </c>
       <c r="L59" t="inlineStr">
         <is>
-          <t>Coluna clima da aba sample.</t>
+          <t>Coluna dh_recebimento da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7012,11 +7012,11 @@
         </is>
       </c>
       <c r="G60" t="n">
-        <v>21</v>
+        <v>13</v>
       </c>
       <c r="H60" t="inlineStr">
         <is>
-          <t>tipo_coleta</t>
+          <t>observacoes</t>
         </is>
       </c>
       <c r="I60" t="inlineStr">
@@ -7034,7 +7034,7 @@
       </c>
       <c r="L60" t="inlineStr">
         <is>
-          <t>Coluna tipo_coleta da aba sample.</t>
+          <t>Coluna observacoes da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7066,16 +7066,16 @@
         </is>
       </c>
       <c r="G61" t="n">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="H61" t="inlineStr">
         <is>
-          <t>responsavel_amostra</t>
+          <t>dh_inicio_atividade</t>
         </is>
       </c>
       <c r="I61" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>data_ou_data_hora</t>
         </is>
       </c>
       <c r="J61" t="b">
@@ -7088,7 +7088,7 @@
       </c>
       <c r="L61" t="inlineStr">
         <is>
-          <t>Coluna responsavel_amostra da aba sample.</t>
+          <t>Coluna dh_inicio_atividade da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7120,11 +7120,11 @@
         </is>
       </c>
       <c r="G62" t="n">
-        <v>23</v>
+        <v>15</v>
       </c>
       <c r="H62" t="inlineStr">
         <is>
-          <t>planejamento_amostragem</t>
+          <t>localizacao</t>
         </is>
       </c>
       <c r="I62" t="inlineStr">
@@ -7142,7 +7142,7 @@
       </c>
       <c r="L62" t="inlineStr">
         <is>
-          <t>Coluna planejamento_amostragem da aba sample.</t>
+          <t>Coluna localizacao da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7174,16 +7174,16 @@
         </is>
       </c>
       <c r="G63" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="H63" t="inlineStr">
         <is>
-          <t>descricao_nao_conformidade</t>
+          <t>latitude</t>
         </is>
       </c>
       <c r="I63" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J63" t="b">
@@ -7196,7 +7196,7 @@
       </c>
       <c r="L63" t="inlineStr">
         <is>
-          <t>Coluna descricao_nao_conformidade da aba sample.</t>
+          <t>Coluna latitude da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7213,31 +7213,31 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E64" t="b">
         <v>1</v>
       </c>
       <c r="F64" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
       <c r="G64" t="n">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="H64" t="inlineStr">
         <is>
-          <t>nome_do_arquivo</t>
+          <t>longitude</t>
         </is>
       </c>
       <c r="I64" t="inlineStr">
         <is>
-          <t>texto</t>
+          <t>decimal</t>
         </is>
       </c>
       <c r="J64" t="b">
@@ -7245,12 +7245,12 @@
       </c>
       <c r="K64" t="inlineStr">
         <is>
-          <t>arquivo_pdf</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L64" t="inlineStr">
         <is>
-          <t>Nome do arquivo PDF de origem do registro.</t>
+          <t>Coluna longitude da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7267,26 +7267,26 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E65" t="b">
         <v>1</v>
       </c>
       <c r="F65" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
       <c r="G65" t="n">
-        <v>2</v>
+        <v>18</v>
       </c>
       <c r="H65" t="inlineStr">
         <is>
-          <t>template_id</t>
+          <t>coordenadas</t>
         </is>
       </c>
       <c r="I65" t="inlineStr">
@@ -7299,12 +7299,12 @@
       </c>
       <c r="K65" t="inlineStr">
         <is>
-          <t>document_scope</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L65" t="inlineStr">
         <is>
-          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
+          <t>Coluna coordenadas da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7321,26 +7321,26 @@
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E66" t="b">
         <v>1</v>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
       <c r="G66" t="n">
-        <v>3</v>
+        <v>19</v>
       </c>
       <c r="H66" t="inlineStr">
         <is>
-          <t>tipo_laudo</t>
+          <t>clima_ultimas_24h</t>
         </is>
       </c>
       <c r="I66" t="inlineStr">
@@ -7353,12 +7353,12 @@
       </c>
       <c r="K66" t="inlineStr">
         <is>
-          <t>templates.theme_id</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L66" t="inlineStr">
         <is>
-          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
+          <t>Coluna clima_ultimas_24h da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7375,31 +7375,31 @@
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E67" t="b">
         <v>1</v>
       </c>
       <c r="F67" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
       <c r="G67" t="n">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="H67" t="inlineStr">
         <is>
-          <t>id_amostra</t>
+          <t>clima</t>
         </is>
       </c>
       <c r="I67" t="inlineStr">
         <is>
-          <t>inteiro_ou_texto</t>
+          <t>texto</t>
         </is>
       </c>
       <c r="J67" t="b">
@@ -7407,12 +7407,12 @@
       </c>
       <c r="K67" t="inlineStr">
         <is>
-          <t>text_extraction_rules.metadata.id_amostra</t>
+          <t>parser</t>
         </is>
       </c>
       <c r="L67" t="inlineStr">
         <is>
-          <t>Coluna id_amostra da aba client.</t>
+          <t>Coluna clima da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7429,26 +7429,26 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E68" t="b">
         <v>1</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
       <c r="G68" t="n">
-        <v>5</v>
+        <v>21</v>
       </c>
       <c r="H68" t="inlineStr">
         <is>
-          <t>proposta_comercial</t>
+          <t>tipo_coleta</t>
         </is>
       </c>
       <c r="I68" t="inlineStr">
@@ -7466,7 +7466,7 @@
       </c>
       <c r="L68" t="inlineStr">
         <is>
-          <t>Coluna proposta_comercial da aba client.</t>
+          <t>Coluna tipo_coleta da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7483,26 +7483,26 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E69" t="b">
         <v>1</v>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
       <c r="G69" t="n">
-        <v>6</v>
+        <v>22</v>
       </c>
       <c r="H69" t="inlineStr">
         <is>
-          <t>cliente</t>
+          <t>responsavel_amostra</t>
         </is>
       </c>
       <c r="I69" t="inlineStr">
@@ -7520,7 +7520,7 @@
       </c>
       <c r="L69" t="inlineStr">
         <is>
-          <t>Coluna cliente da aba client.</t>
+          <t>Coluna responsavel_amostra da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7537,26 +7537,26 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E70" t="b">
         <v>1</v>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
       <c r="G70" t="n">
-        <v>7</v>
+        <v>23</v>
       </c>
       <c r="H70" t="inlineStr">
         <is>
-          <t>cnpj_cpf</t>
+          <t>planejamento_amostragem</t>
         </is>
       </c>
       <c r="I70" t="inlineStr">
@@ -7574,7 +7574,7 @@
       </c>
       <c r="L70" t="inlineStr">
         <is>
-          <t>Coluna cnpj_cpf da aba client.</t>
+          <t>Coluna planejamento_amostragem da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7591,26 +7591,26 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>client</t>
+          <t>sample</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="E71" t="b">
         <v>1</v>
       </c>
       <c r="F71" t="inlineStr">
         <is>
-          <t>Dados de identificacao do cliente.</t>
+          <t>Dados de amostra/cabecalho do PDF.</t>
         </is>
       </c>
       <c r="G71" t="n">
-        <v>8</v>
+        <v>24</v>
       </c>
       <c r="H71" t="inlineStr">
         <is>
-          <t>contato</t>
+          <t>descricao_nao_conformidade</t>
         </is>
       </c>
       <c r="I71" t="inlineStr">
@@ -7628,7 +7628,7 @@
       </c>
       <c r="L71" t="inlineStr">
         <is>
-          <t>Coluna contato da aba client.</t>
+          <t>Coluna descricao_nao_conformidade da aba sample.</t>
         </is>
       </c>
     </row>
@@ -7660,11 +7660,11 @@
         </is>
       </c>
       <c r="G72" t="n">
-        <v>9</v>
+        <v>1</v>
       </c>
       <c r="H72" t="inlineStr">
         <is>
-          <t>telefone</t>
+          <t>nome_do_arquivo</t>
         </is>
       </c>
       <c r="I72" t="inlineStr">
@@ -7677,12 +7677,12 @@
       </c>
       <c r="K72" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>arquivo_pdf</t>
         </is>
       </c>
       <c r="L72" t="inlineStr">
         <is>
-          <t>Coluna telefone da aba client.</t>
+          <t>Nome do arquivo PDF de origem do registro.</t>
         </is>
       </c>
     </row>
@@ -7714,11 +7714,11 @@
         </is>
       </c>
       <c r="G73" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="H73" t="inlineStr">
         <is>
-          <t>endereco</t>
+          <t>template_id</t>
         </is>
       </c>
       <c r="I73" t="inlineStr">
@@ -7731,12 +7731,12 @@
       </c>
       <c r="K73" t="inlineStr">
         <is>
-          <t>parser</t>
+          <t>document_scope</t>
         </is>
       </c>
       <c r="L73" t="inlineStr">
         <is>
-          <t>Coluna endereco da aba client.</t>
+          <t>Identificador do template/modelo de laudo reconhecido pela taxonomia.</t>
         </is>
       </c>
     </row>
@@ -7753,26 +7753,44 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>table_extraction_audit</t>
+          <t>client</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>97</v>
+        <v>3</v>
       </c>
       <c r="E74" t="b">
         <v>1</v>
       </c>
       <c r="F74" t="inlineStr">
         <is>
-          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+      <c r="G74" t="n">
+        <v>3</v>
+      </c>
+      <c r="H74" t="inlineStr">
+        <is>
+          <t>tipo_laudo</t>
+        </is>
+      </c>
+      <c r="I74" t="inlineStr">
+        <is>
+          <t>texto</t>
         </is>
       </c>
       <c r="J74" t="b">
         <v>0</v>
       </c>
+      <c r="K74" t="inlineStr">
+        <is>
+          <t>templates.theme_id</t>
+        </is>
+      </c>
       <c r="L74" t="inlineStr">
         <is>
-          <t>Aba de auditoria das tabelas processadas, incluindo colunas detectadas, campos esperados e status da leitura.</t>
+          <t>Tipo/familia do laudo identificado pela taxonomia, como agua, sedimento, mps, fito ou bentos.</t>
         </is>
       </c>
     </row>
@@ -7789,26 +7807,44 @@
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>classification_audit</t>
+          <t>client</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>98</v>
+        <v>3</v>
       </c>
       <c r="E75" t="b">
         <v>1</v>
       </c>
       <c r="F75" t="inlineStr">
         <is>
-          <t>Auditoria da classificacao do PDF por template.</t>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+      <c r="G75" t="n">
+        <v>4</v>
+      </c>
+      <c r="H75" t="inlineStr">
+        <is>
+          <t>id_amostra</t>
+        </is>
+      </c>
+      <c r="I75" t="inlineStr">
+        <is>
+          <t>inteiro_ou_texto</t>
         </is>
       </c>
       <c r="J75" t="b">
         <v>0</v>
       </c>
+      <c r="K75" t="inlineStr">
+        <is>
+          <t>text_extraction_rules.metadata.id_amostra</t>
+        </is>
+      </c>
       <c r="L75" t="inlineStr">
         <is>
-          <t>Aba de auditoria da classificacao do template, incluindo regras encontradas, score e status por candidato.</t>
+          <t>Coluna id_amostra da aba client.</t>
         </is>
       </c>
     </row>
@@ -7825,31 +7861,427 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>3</v>
+      </c>
+      <c r="E76" t="b">
+        <v>1</v>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+      <c r="G76" t="n">
+        <v>5</v>
+      </c>
+      <c r="H76" t="inlineStr">
+        <is>
+          <t>proposta_comercial</t>
+        </is>
+      </c>
+      <c r="I76" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="J76" t="b">
+        <v>0</v>
+      </c>
+      <c r="K76" t="inlineStr">
+        <is>
+          <t>parser</t>
+        </is>
+      </c>
+      <c r="L76" t="inlineStr">
+        <is>
+          <t>Coluna proposta_comercial da aba client.</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B77" t="inlineStr">
+        <is>
+          <t>laudo_agua</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D77" t="n">
+        <v>3</v>
+      </c>
+      <c r="E77" t="b">
+        <v>1</v>
+      </c>
+      <c r="F77" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+      <c r="G77" t="n">
+        <v>6</v>
+      </c>
+      <c r="H77" t="inlineStr">
+        <is>
+          <t>cliente</t>
+        </is>
+      </c>
+      <c r="I77" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="J77" t="b">
+        <v>0</v>
+      </c>
+      <c r="K77" t="inlineStr">
+        <is>
+          <t>parser</t>
+        </is>
+      </c>
+      <c r="L77" t="inlineStr">
+        <is>
+          <t>Coluna cliente da aba client.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78">
+      <c r="A78" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B78" t="inlineStr">
+        <is>
+          <t>laudo_agua</t>
+        </is>
+      </c>
+      <c r="C78" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D78" t="n">
+        <v>3</v>
+      </c>
+      <c r="E78" t="b">
+        <v>1</v>
+      </c>
+      <c r="F78" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+      <c r="G78" t="n">
+        <v>7</v>
+      </c>
+      <c r="H78" t="inlineStr">
+        <is>
+          <t>cnpj_cpf</t>
+        </is>
+      </c>
+      <c r="I78" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="J78" t="b">
+        <v>0</v>
+      </c>
+      <c r="K78" t="inlineStr">
+        <is>
+          <t>parser</t>
+        </is>
+      </c>
+      <c r="L78" t="inlineStr">
+        <is>
+          <t>Coluna cnpj_cpf da aba client.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79">
+      <c r="A79" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B79" t="inlineStr">
+        <is>
+          <t>laudo_agua</t>
+        </is>
+      </c>
+      <c r="C79" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D79" t="n">
+        <v>3</v>
+      </c>
+      <c r="E79" t="b">
+        <v>1</v>
+      </c>
+      <c r="F79" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+      <c r="G79" t="n">
+        <v>8</v>
+      </c>
+      <c r="H79" t="inlineStr">
+        <is>
+          <t>contato</t>
+        </is>
+      </c>
+      <c r="I79" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="J79" t="b">
+        <v>0</v>
+      </c>
+      <c r="K79" t="inlineStr">
+        <is>
+          <t>parser</t>
+        </is>
+      </c>
+      <c r="L79" t="inlineStr">
+        <is>
+          <t>Coluna contato da aba client.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80">
+      <c r="A80" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B80" t="inlineStr">
+        <is>
+          <t>laudo_agua</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D80" t="n">
+        <v>3</v>
+      </c>
+      <c r="E80" t="b">
+        <v>1</v>
+      </c>
+      <c r="F80" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+      <c r="G80" t="n">
+        <v>9</v>
+      </c>
+      <c r="H80" t="inlineStr">
+        <is>
+          <t>telefone</t>
+        </is>
+      </c>
+      <c r="I80" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="J80" t="b">
+        <v>0</v>
+      </c>
+      <c r="K80" t="inlineStr">
+        <is>
+          <t>parser</t>
+        </is>
+      </c>
+      <c r="L80" t="inlineStr">
+        <is>
+          <t>Coluna telefone da aba client.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B81" t="inlineStr">
+        <is>
+          <t>laudo_agua</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
+          <t>client</t>
+        </is>
+      </c>
+      <c r="D81" t="n">
+        <v>3</v>
+      </c>
+      <c r="E81" t="b">
+        <v>1</v>
+      </c>
+      <c r="F81" t="inlineStr">
+        <is>
+          <t>Dados de identificacao do cliente.</t>
+        </is>
+      </c>
+      <c r="G81" t="n">
+        <v>10</v>
+      </c>
+      <c r="H81" t="inlineStr">
+        <is>
+          <t>endereco</t>
+        </is>
+      </c>
+      <c r="I81" t="inlineStr">
+        <is>
+          <t>texto</t>
+        </is>
+      </c>
+      <c r="J81" t="b">
+        <v>0</v>
+      </c>
+      <c r="K81" t="inlineStr">
+        <is>
+          <t>parser</t>
+        </is>
+      </c>
+      <c r="L81" t="inlineStr">
+        <is>
+          <t>Coluna endereco da aba client.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B82" t="inlineStr">
+        <is>
+          <t>laudo_agua</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
+          <t>table_extraction_audit</t>
+        </is>
+      </c>
+      <c r="D82" t="n">
+        <v>97</v>
+      </c>
+      <c r="E82" t="b">
+        <v>1</v>
+      </c>
+      <c r="F82" t="inlineStr">
+        <is>
+          <t>Auditoria estrutural dos cabecalhos e colunas de tabelas extraidas.</t>
+        </is>
+      </c>
+      <c r="J82" t="b">
+        <v>0</v>
+      </c>
+      <c r="L82" t="inlineStr">
+        <is>
+          <t>Aba de auditoria das tabelas processadas, incluindo colunas detectadas, campos esperados e status da leitura.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B83" t="inlineStr">
+        <is>
+          <t>laudo_agua</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
+          <t>classification_audit</t>
+        </is>
+      </c>
+      <c r="D83" t="n">
+        <v>98</v>
+      </c>
+      <c r="E83" t="b">
+        <v>1</v>
+      </c>
+      <c r="F83" t="inlineStr">
+        <is>
+          <t>Auditoria da classificacao do PDF por template.</t>
+        </is>
+      </c>
+      <c r="J83" t="b">
+        <v>0</v>
+      </c>
+      <c r="L83" t="inlineStr">
+        <is>
+          <t>Aba de auditoria da classificacao do template, incluindo regras encontradas, score e status por candidato.</t>
+        </is>
+      </c>
+    </row>
+    <row r="84">
+      <c r="A84" t="inlineStr">
+        <is>
+          <t>template_laudo_agua_v1</t>
+        </is>
+      </c>
+      <c r="B84" t="inlineStr">
+        <is>
+          <t>laudo_agua</t>
+        </is>
+      </c>
+      <c r="C84" t="inlineStr">
+        <is>
           <t>validation_errors</t>
         </is>
       </c>
-      <c r="D76" t="n">
+      <c r="D84" t="n">
         <v>99</v>
       </c>
-      <c r="E76" t="b">
-        <v>1</v>
-      </c>
-      <c r="F76" t="inlineStr">
+      <c r="E84" t="b">
+        <v>1</v>
+      </c>
+      <c r="F84" t="inlineStr">
         <is>
           <t>Erros de validacao da saida.</t>
         </is>
       </c>
-      <c r="J76" t="b">
-        <v>0</v>
-      </c>
-      <c r="L76" t="inlineStr">
+      <c r="J84" t="b">
+        <v>0</v>
+      </c>
+      <c r="L84" t="inlineStr">
         <is>
           <t>Aba de erros de validacao final, preenchida quando algum campo nao atende ao contrato esperado.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L76"/>
+  <autoFilter ref="A1:L84"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>